<commit_message>
Daily scrape output - 2026-09-13
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F757"/>
+  <dimension ref="A1:F767"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19192,10 +19192,10 @@
         </is>
       </c>
       <c r="E722" t="n">
-        <v>10.32</v>
+        <v>10.34</v>
       </c>
       <c r="F722" t="n">
-        <v>0.55</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="723">
@@ -19244,10 +19244,10 @@
         </is>
       </c>
       <c r="E724" t="n">
-        <v>10.45</v>
+        <v>10.09</v>
       </c>
       <c r="F724" t="n">
-        <v>1.65</v>
+        <v>1.67</v>
       </c>
     </row>
     <row r="725">
@@ -19270,7 +19270,7 @@
         </is>
       </c>
       <c r="E725" t="n">
-        <v>10.04</v>
+        <v>10.16</v>
       </c>
       <c r="F725" t="n">
         <v>1.85</v>
@@ -19296,10 +19296,10 @@
         </is>
       </c>
       <c r="E726" t="n">
-        <v>10.05</v>
+        <v>9.94</v>
       </c>
       <c r="F726" t="n">
-        <v>0.66</v>
+        <v>0.53</v>
       </c>
     </row>
     <row r="727">
@@ -19313,19 +19313,19 @@
       </c>
       <c r="C727" t="inlineStr">
         <is>
-          <t>Throttur Reykjavik</t>
+          <t>Fylkir</t>
         </is>
       </c>
       <c r="D727" t="inlineStr">
         <is>
-          <t>UMF Njardvik</t>
+          <t>HK Kopavogur</t>
         </is>
       </c>
       <c r="E727" t="n">
-        <v>11.55</v>
+        <v>11.61</v>
       </c>
       <c r="F727" t="n">
-        <v>1.03</v>
+        <v>1.89</v>
       </c>
     </row>
     <row r="728">
@@ -19334,24 +19334,24 @@
       </c>
       <c r="B728" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Iceland - 1. Deild</t>
         </is>
       </c>
       <c r="C728" t="inlineStr">
         <is>
-          <t>Egersunds</t>
+          <t>Throttur Reykjavik</t>
         </is>
       </c>
       <c r="D728" t="inlineStr">
         <is>
-          <t>Kongsvinger</t>
+          <t>UMF Njardvik</t>
         </is>
       </c>
       <c r="E728" t="n">
-        <v>10.66</v>
+        <v>11.55</v>
       </c>
       <c r="F728" t="n">
-        <v>-0.47</v>
+        <v>1.03</v>
       </c>
     </row>
     <row r="729">
@@ -19365,19 +19365,19 @@
       </c>
       <c r="C729" t="inlineStr">
         <is>
-          <t>Hodd</t>
+          <t>Egersunds</t>
         </is>
       </c>
       <c r="D729" t="inlineStr">
         <is>
-          <t>Lyn</t>
+          <t>Kongsvinger</t>
         </is>
       </c>
       <c r="E729" t="n">
-        <v>10.7</v>
+        <v>10.5</v>
       </c>
       <c r="F729" t="n">
-        <v>-1.19</v>
+        <v>-0.8</v>
       </c>
     </row>
     <row r="730">
@@ -19391,19 +19391,19 @@
       </c>
       <c r="C730" t="inlineStr">
         <is>
-          <t>Moss</t>
+          <t>Hodd</t>
         </is>
       </c>
       <c r="D730" t="inlineStr">
         <is>
-          <t>Haugesund</t>
+          <t>Lyn</t>
         </is>
       </c>
       <c r="E730" t="n">
-        <v>11.2</v>
+        <v>10.7</v>
       </c>
       <c r="F730" t="n">
-        <v>-1.33</v>
+        <v>-1.19</v>
       </c>
     </row>
     <row r="731">
@@ -19417,19 +19417,19 @@
       </c>
       <c r="C731" t="inlineStr">
         <is>
-          <t>Raufoss</t>
+          <t>Moss</t>
         </is>
       </c>
       <c r="D731" t="inlineStr">
         <is>
-          <t>Odd BK</t>
+          <t>Haugesund</t>
         </is>
       </c>
       <c r="E731" t="n">
-        <v>11.02</v>
+        <v>11.2</v>
       </c>
       <c r="F731" t="n">
-        <v>-2.09</v>
+        <v>-1.33</v>
       </c>
     </row>
     <row r="732">
@@ -19443,19 +19443,19 @@
       </c>
       <c r="C732" t="inlineStr">
         <is>
-          <t>Sogndal</t>
+          <t>Ranheim</t>
         </is>
       </c>
       <c r="D732" t="inlineStr">
         <is>
-          <t>Strommen</t>
+          <t>Asane</t>
         </is>
       </c>
       <c r="E732" t="n">
-        <v>11.09</v>
+        <v>11.17</v>
       </c>
       <c r="F732" t="n">
-        <v>1.07</v>
+        <v>2.01</v>
       </c>
     </row>
     <row r="733">
@@ -19469,19 +19469,19 @@
       </c>
       <c r="C733" t="inlineStr">
         <is>
-          <t>Stromsgodset</t>
+          <t>Raufoss</t>
         </is>
       </c>
       <c r="D733" t="inlineStr">
         <is>
-          <t>Sandnes Ulf</t>
+          <t>Odd BK</t>
         </is>
       </c>
       <c r="E733" t="n">
-        <v>11.48</v>
+        <v>11.03</v>
       </c>
       <c r="F733" t="n">
-        <v>3.4</v>
+        <v>-2.09</v>
       </c>
     </row>
     <row r="734">
@@ -19490,24 +19490,24 @@
       </c>
       <c r="B734" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C734" t="inlineStr">
         <is>
-          <t>Odra Opole</t>
+          <t>Sogndal</t>
         </is>
       </c>
       <c r="D734" t="inlineStr">
         <is>
-          <t>Stal Rzeszow</t>
+          <t>Strommen</t>
         </is>
       </c>
       <c r="E734" t="n">
-        <v>10.67</v>
+        <v>11.03</v>
       </c>
       <c r="F734" t="n">
-        <v>0.99</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="735">
@@ -19516,24 +19516,24 @@
       </c>
       <c r="B735" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C735" t="inlineStr">
         <is>
-          <t>Legia Warsaw</t>
+          <t>Stromsgodset</t>
         </is>
       </c>
       <c r="D735" t="inlineStr">
         <is>
-          <t>Widzew Lodz</t>
+          <t>Sandnes Ulf</t>
         </is>
       </c>
       <c r="E735" t="n">
-        <v>9.789999999999999</v>
+        <v>11.2</v>
       </c>
       <c r="F735" t="n">
-        <v>1.65</v>
+        <v>3.41</v>
       </c>
     </row>
     <row r="736">
@@ -19542,24 +19542,24 @@
       </c>
       <c r="B736" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C736" t="inlineStr">
         <is>
-          <t>Wisla Plock</t>
+          <t>Lechia Gdansk</t>
         </is>
       </c>
       <c r="D736" t="inlineStr">
         <is>
-          <t>Cracovia Krakow</t>
+          <t>Miedz Legnica</t>
         </is>
       </c>
       <c r="E736" t="n">
-        <v>10.72</v>
+        <v>10.85</v>
       </c>
       <c r="F736" t="n">
-        <v>0.38</v>
+        <v>0.32</v>
       </c>
     </row>
     <row r="737">
@@ -19568,24 +19568,24 @@
       </c>
       <c r="B737" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C737" t="inlineStr">
         <is>
-          <t>Arges Pitesti</t>
+          <t>Odra Opole</t>
         </is>
       </c>
       <c r="D737" t="inlineStr">
         <is>
-          <t>Botosani</t>
+          <t>Stal Rzeszow</t>
         </is>
       </c>
       <c r="E737" t="n">
-        <v>9.6</v>
+        <v>10.98</v>
       </c>
       <c r="F737" t="n">
-        <v>1.06</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="738">
@@ -19594,24 +19594,24 @@
       </c>
       <c r="B738" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C738" t="inlineStr">
         <is>
-          <t>Mallorca</t>
+          <t>Legia Warsaw</t>
         </is>
       </c>
       <c r="D738" t="inlineStr">
         <is>
-          <t>Sabadell</t>
+          <t>Widzew Lodz</t>
         </is>
       </c>
       <c r="E738" t="n">
-        <v>8.609999999999999</v>
+        <v>9.789999999999999</v>
       </c>
       <c r="F738" t="n">
-        <v>1.04</v>
+        <v>1.65</v>
       </c>
     </row>
     <row r="739">
@@ -19620,24 +19620,24 @@
       </c>
       <c r="B739" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C739" t="inlineStr">
         <is>
-          <t>Real Valladolid</t>
+          <t>Pogon Szczecin</t>
         </is>
       </c>
       <c r="D739" t="inlineStr">
         <is>
-          <t>Real Oviedo</t>
+          <t>Wieczysta Krakow</t>
         </is>
       </c>
       <c r="E739" t="n">
-        <v>8.609999999999999</v>
+        <v>9.69</v>
       </c>
       <c r="F739" t="n">
-        <v>0.72</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="740">
@@ -19646,24 +19646,24 @@
       </c>
       <c r="B740" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C740" t="inlineStr">
         <is>
-          <t>Sporting Gijon</t>
+          <t>Wisla Plock</t>
         </is>
       </c>
       <c r="D740" t="inlineStr">
         <is>
-          <t>Eldense</t>
+          <t>Cracovia Krakow</t>
         </is>
       </c>
       <c r="E740" t="n">
-        <v>9.59</v>
+        <v>10.72</v>
       </c>
       <c r="F740" t="n">
-        <v>1.43</v>
+        <v>0.38</v>
       </c>
     </row>
     <row r="741">
@@ -19672,24 +19672,24 @@
       </c>
       <c r="B741" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C741" t="inlineStr">
         <is>
-          <t>Tenerife</t>
+          <t>Arges Pitesti</t>
         </is>
       </c>
       <c r="D741" t="inlineStr">
         <is>
-          <t>Leganes</t>
+          <t>Botosani</t>
         </is>
       </c>
       <c r="E741" t="n">
-        <v>9.6</v>
+        <v>9.720000000000001</v>
       </c>
       <c r="F741" t="n">
-        <v>1.38</v>
+        <v>1.21</v>
       </c>
     </row>
     <row r="742">
@@ -19698,24 +19698,24 @@
       </c>
       <c r="B742" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C742" t="inlineStr">
         <is>
-          <t>Ljungskile</t>
+          <t>Corvinul Hunedoara</t>
         </is>
       </c>
       <c r="D742" t="inlineStr">
         <is>
-          <t>Falkenbergs</t>
+          <t>Universitatea Craiova</t>
         </is>
       </c>
       <c r="E742" t="n">
-        <v>10.29</v>
+        <v>8.83</v>
       </c>
       <c r="F742" t="n">
-        <v>0.9</v>
+        <v>-0.96</v>
       </c>
     </row>
     <row r="743">
@@ -19724,154 +19724,154 @@
       </c>
       <c r="B743" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C743" t="inlineStr">
         <is>
-          <t>Norrkoping</t>
+          <t>Mallorca</t>
         </is>
       </c>
       <c r="D743" t="inlineStr">
         <is>
-          <t>Oddevold</t>
+          <t>Sabadell</t>
         </is>
       </c>
       <c r="E743" t="n">
-        <v>10.16</v>
+        <v>8.710000000000001</v>
       </c>
       <c r="F743" t="n">
-        <v>1.97</v>
+        <v>1.15</v>
       </c>
     </row>
     <row r="744">
       <c r="A744" s="1" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B744" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C744" t="inlineStr">
         <is>
-          <t>America Mineiro</t>
+          <t>Real Valladolid</t>
         </is>
       </c>
       <c r="D744" t="inlineStr">
         <is>
-          <t>Sao Bernardo</t>
+          <t>Real Oviedo</t>
         </is>
       </c>
       <c r="E744" t="n">
-        <v>10.63</v>
+        <v>8.609999999999999</v>
       </c>
       <c r="F744" t="n">
-        <v>1.01</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="745">
       <c r="A745" s="1" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B745" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C745" t="inlineStr">
         <is>
-          <t>Botafogo SP</t>
+          <t>Sporting Gijon</t>
         </is>
       </c>
       <c r="D745" t="inlineStr">
         <is>
-          <t>Goias</t>
+          <t>Eldense</t>
         </is>
       </c>
       <c r="E745" t="n">
-        <v>10.65</v>
+        <v>9.59</v>
       </c>
       <c r="F745" t="n">
-        <v>1.34</v>
+        <v>1.44</v>
       </c>
     </row>
     <row r="746">
       <c r="A746" s="1" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B746" t="inlineStr">
         <is>
-          <t>Finland - Veikkausliiga</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C746" t="inlineStr">
         <is>
-          <t>Inter Turku</t>
+          <t>Tenerife</t>
         </is>
       </c>
       <c r="D746" t="inlineStr">
         <is>
-          <t>VPS</t>
+          <t>Leganes</t>
         </is>
       </c>
       <c r="E746" t="n">
-        <v>9.5</v>
+        <v>9.52</v>
       </c>
       <c r="F746" t="n">
-        <v>1.88</v>
+        <v>1.57</v>
       </c>
     </row>
     <row r="747">
       <c r="A747" s="1" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B747" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="C747" t="inlineStr">
         <is>
-          <t>Radomiak Radom</t>
+          <t>Ljungskile</t>
         </is>
       </c>
       <c r="D747" t="inlineStr">
         <is>
-          <t>Piast Gliwice</t>
+          <t>Falkenbergs</t>
         </is>
       </c>
       <c r="E747" t="n">
-        <v>10.5</v>
+        <v>10.29</v>
       </c>
       <c r="F747" t="n">
-        <v>0.34</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="748">
       <c r="A748" s="1" t="n">
-        <v>46279</v>
+        <v>46278</v>
       </c>
       <c r="B748" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="C748" t="inlineStr">
         <is>
-          <t>FCSB</t>
+          <t>Norrkoping</t>
         </is>
       </c>
       <c r="D748" t="inlineStr">
         <is>
-          <t>Petrolul Ploiesti</t>
+          <t>Oddevold</t>
         </is>
       </c>
       <c r="E748" t="n">
-        <v>10.11</v>
+        <v>10.16</v>
       </c>
       <c r="F748" t="n">
-        <v>3.25</v>
+        <v>1.89</v>
       </c>
     </row>
     <row r="749">
@@ -19880,24 +19880,24 @@
       </c>
       <c r="B749" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C749" t="inlineStr">
         <is>
-          <t>Universitatea Cluj</t>
+          <t>America Mineiro</t>
         </is>
       </c>
       <c r="D749" t="inlineStr">
         <is>
-          <t>Otelul Galati</t>
+          <t>Sao Bernardo</t>
         </is>
       </c>
       <c r="E749" t="n">
-        <v>9.66</v>
+        <v>10.63</v>
       </c>
       <c r="F749" t="n">
-        <v>1.54</v>
+        <v>1.01</v>
       </c>
     </row>
     <row r="750">
@@ -19906,24 +19906,24 @@
       </c>
       <c r="B750" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C750" t="inlineStr">
         <is>
-          <t>Norrby</t>
+          <t>Botafogo SP</t>
         </is>
       </c>
       <c r="D750" t="inlineStr">
         <is>
-          <t>Varbergs BoIS</t>
+          <t>Goias</t>
         </is>
       </c>
       <c r="E750" t="n">
-        <v>10.55</v>
+        <v>10.65</v>
       </c>
       <c r="F750" t="n">
-        <v>-0.5600000000000001</v>
+        <v>1.34</v>
       </c>
     </row>
     <row r="751">
@@ -19932,24 +19932,24 @@
       </c>
       <c r="B751" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Finland - Veikkausliiga</t>
         </is>
       </c>
       <c r="C751" t="inlineStr">
         <is>
-          <t>Orebro SK</t>
+          <t>Inter Turku</t>
         </is>
       </c>
       <c r="D751" t="inlineStr">
         <is>
-          <t>Nordic United</t>
+          <t>VPS</t>
         </is>
       </c>
       <c r="E751" t="n">
-        <v>10.17</v>
+        <v>9.5</v>
       </c>
       <c r="F751" t="n">
-        <v>0.71</v>
+        <v>1.88</v>
       </c>
     </row>
     <row r="752">
@@ -19958,107 +19958,107 @@
       </c>
       <c r="B752" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C752" t="inlineStr">
         <is>
-          <t>Ostersunds FK</t>
+          <t>Radomiak Radom</t>
         </is>
       </c>
       <c r="D752" t="inlineStr">
         <is>
-          <t>Helsingborgs</t>
+          <t>Piast Gliwice</t>
         </is>
       </c>
       <c r="E752" t="n">
-        <v>9.98</v>
+        <v>10.5</v>
       </c>
       <c r="F752" t="n">
-        <v>1.46</v>
+        <v>0.34</v>
       </c>
     </row>
     <row r="753">
       <c r="A753" s="1" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B753" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C753" t="inlineStr">
         <is>
-          <t>Avai</t>
+          <t>FCSB</t>
         </is>
       </c>
       <c r="D753" t="inlineStr">
         <is>
-          <t>Vila Nova</t>
+          <t>Petrolul Ploiesti</t>
         </is>
       </c>
       <c r="E753" t="n">
-        <v>9.82</v>
+        <v>10.11</v>
       </c>
       <c r="F753" t="n">
-        <v>0.17</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="754">
       <c r="A754" s="1" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B754" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C754" t="inlineStr">
         <is>
-          <t>Nautico</t>
+          <t>Universitatea Cluj</t>
         </is>
       </c>
       <c r="D754" t="inlineStr">
         <is>
-          <t>Operario Ferroviario</t>
+          <t>Otelul Galati</t>
         </is>
       </c>
       <c r="E754" t="n">
-        <v>10.69</v>
+        <v>9.66</v>
       </c>
       <c r="F754" t="n">
-        <v>2.09</v>
+        <v>1.54</v>
       </c>
     </row>
     <row r="755">
       <c r="A755" s="1" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B755" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C755" t="inlineStr">
         <is>
-          <t>Brage</t>
+          <t>Celta Vigo II</t>
         </is>
       </c>
       <c r="D755" t="inlineStr">
         <is>
-          <t>Sandvikens IF</t>
+          <t>Eibar</t>
         </is>
       </c>
       <c r="E755" t="n">
-        <v>10.55</v>
+        <v>8.94</v>
       </c>
       <c r="F755" t="n">
-        <v>-0.17</v>
+        <v>-0.16</v>
       </c>
     </row>
     <row r="756">
       <c r="A756" s="1" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B756" t="inlineStr">
         <is>
@@ -20067,45 +20067,305 @@
       </c>
       <c r="C756" t="inlineStr">
         <is>
-          <t>Landskrona</t>
+          <t>Norrby</t>
         </is>
       </c>
       <c r="D756" t="inlineStr">
         <is>
-          <t>Sundsvall</t>
+          <t>Varbergs BoIS</t>
         </is>
       </c>
       <c r="E756" t="n">
-        <v>10.39</v>
+        <v>10.55</v>
       </c>
       <c r="F756" t="n">
-        <v>2.43</v>
+        <v>-0.5600000000000001</v>
       </c>
     </row>
     <row r="757">
       <c r="A757" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B757" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C757" t="inlineStr">
+        <is>
+          <t>Orebro SK</t>
+        </is>
+      </c>
+      <c r="D757" t="inlineStr">
+        <is>
+          <t>Nordic United</t>
+        </is>
+      </c>
+      <c r="E757" t="n">
+        <v>10.17</v>
+      </c>
+      <c r="F757" t="n">
+        <v>0.71</v>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B758" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C758" t="inlineStr">
+        <is>
+          <t>Ostersunds FK</t>
+        </is>
+      </c>
+      <c r="D758" t="inlineStr">
+        <is>
+          <t>Helsingborgs</t>
+        </is>
+      </c>
+      <c r="E758" t="n">
+        <v>9.74</v>
+      </c>
+      <c r="F758" t="n">
+        <v>1.89</v>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" s="1" t="n">
         <v>46280</v>
       </c>
-      <c r="B757" t="inlineStr">
+      <c r="B759" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C759" t="inlineStr">
+        <is>
+          <t>Avai</t>
+        </is>
+      </c>
+      <c r="D759" t="inlineStr">
+        <is>
+          <t>Vila Nova</t>
+        </is>
+      </c>
+      <c r="E759" t="n">
+        <v>9.82</v>
+      </c>
+      <c r="F759" t="n">
+        <v>0.17</v>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" s="1" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B760" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C760" t="inlineStr">
+        <is>
+          <t>Londrina</t>
+        </is>
+      </c>
+      <c r="D760" t="inlineStr">
+        <is>
+          <t>Ponte Preta</t>
+        </is>
+      </c>
+      <c r="E760" t="n">
+        <v>10.81</v>
+      </c>
+      <c r="F760" t="n">
+        <v>3.43</v>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" s="1" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B761" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C761" t="inlineStr">
+        <is>
+          <t>Nautico</t>
+        </is>
+      </c>
+      <c r="D761" t="inlineStr">
+        <is>
+          <t>Operario Ferroviario</t>
+        </is>
+      </c>
+      <c r="E761" t="n">
+        <v>10.69</v>
+      </c>
+      <c r="F761" t="n">
+        <v>2.09</v>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" s="1" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B762" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C762" t="inlineStr">
+        <is>
+          <t>Korona Kielce</t>
+        </is>
+      </c>
+      <c r="D762" t="inlineStr">
+        <is>
+          <t>Gornik Zabrze</t>
+        </is>
+      </c>
+      <c r="E762" t="n">
+        <v>10.22</v>
+      </c>
+      <c r="F762" t="n">
+        <v>-0.38</v>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" s="1" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B763" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C763" t="inlineStr">
+        <is>
+          <t>Rakow Czestochowa</t>
+        </is>
+      </c>
+      <c r="D763" t="inlineStr">
+        <is>
+          <t>Zaglebie Lubin</t>
+        </is>
+      </c>
+      <c r="E763" t="n">
+        <v>9.970000000000001</v>
+      </c>
+      <c r="F763" t="n">
+        <v>2.05</v>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" s="1" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B764" t="inlineStr">
         <is>
           <t>Sweden - Superettan</t>
         </is>
       </c>
-      <c r="C757" t="inlineStr">
+      <c r="C764" t="inlineStr">
+        <is>
+          <t>Brage</t>
+        </is>
+      </c>
+      <c r="D764" t="inlineStr">
+        <is>
+          <t>Sandvikens IF</t>
+        </is>
+      </c>
+      <c r="E764" t="n">
+        <v>10.55</v>
+      </c>
+      <c r="F764" t="n">
+        <v>-0.17</v>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" s="1" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B765" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C765" t="inlineStr">
+        <is>
+          <t>Landskrona</t>
+        </is>
+      </c>
+      <c r="D765" t="inlineStr">
+        <is>
+          <t>Sundsvall</t>
+        </is>
+      </c>
+      <c r="E765" t="n">
+        <v>10.39</v>
+      </c>
+      <c r="F765" t="n">
+        <v>2.43</v>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" s="1" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B766" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C766" t="inlineStr">
         <is>
           <t>Varnamo</t>
         </is>
       </c>
-      <c r="D757" t="inlineStr">
+      <c r="D766" t="inlineStr">
         <is>
           <t>Osters</t>
         </is>
       </c>
-      <c r="E757" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="F757" t="n">
-        <v>1.35</v>
+      <c r="E766" t="n">
+        <v>10.59</v>
+      </c>
+      <c r="F766" t="n">
+        <v>1.36</v>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" s="1" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B767" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C767" t="inlineStr">
+        <is>
+          <t>CRB</t>
+        </is>
+      </c>
+      <c r="D767" t="inlineStr">
+        <is>
+          <t>Sport Recife</t>
+        </is>
+      </c>
+      <c r="E767" t="n">
+        <v>10.84</v>
+      </c>
+      <c r="F767" t="n">
+        <v>2.07</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-09-15
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -20180,10 +20180,10 @@
         </is>
       </c>
       <c r="E760" t="n">
-        <v>10.81</v>
+        <v>10.95</v>
       </c>
       <c r="F760" t="n">
-        <v>3.43</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="761">
@@ -20206,10 +20206,10 @@
         </is>
       </c>
       <c r="E761" t="n">
-        <v>10.69</v>
+        <v>10.6</v>
       </c>
       <c r="F761" t="n">
-        <v>2.09</v>
+        <v>2.44</v>
       </c>
     </row>
     <row r="762">
@@ -20235,7 +20235,7 @@
         <v>10.22</v>
       </c>
       <c r="F762" t="n">
-        <v>-0.38</v>
+        <v>-0.37</v>
       </c>
     </row>
     <row r="763">
@@ -20284,10 +20284,10 @@
         </is>
       </c>
       <c r="E764" t="n">
-        <v>10.55</v>
+        <v>10.99</v>
       </c>
       <c r="F764" t="n">
-        <v>-0.17</v>
+        <v>-0.87</v>
       </c>
     </row>
     <row r="765">
@@ -20310,10 +20310,10 @@
         </is>
       </c>
       <c r="E765" t="n">
-        <v>10.39</v>
+        <v>9.73</v>
       </c>
       <c r="F765" t="n">
-        <v>2.43</v>
+        <v>2.41</v>
       </c>
     </row>
     <row r="766">
@@ -20362,10 +20362,10 @@
         </is>
       </c>
       <c r="E767" t="n">
-        <v>10.84</v>
+        <v>10.81</v>
       </c>
       <c r="F767" t="n">
-        <v>2.07</v>
+        <v>2.14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-09-18
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F767"/>
+  <dimension ref="A1:F827"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20368,6 +20368,1566 @@
         <v>2.14</v>
       </c>
     </row>
+    <row r="768">
+      <c r="A768" s="1" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B768" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C768" t="inlineStr">
+        <is>
+          <t>Ceara</t>
+        </is>
+      </c>
+      <c r="D768" t="inlineStr">
+        <is>
+          <t>Gremio Novorizontino</t>
+        </is>
+      </c>
+      <c r="E768" t="n">
+        <v>10.62</v>
+      </c>
+      <c r="F768" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" s="1" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B769" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C769" t="inlineStr">
+        <is>
+          <t>Vila Nova</t>
+        </is>
+      </c>
+      <c r="D769" t="inlineStr">
+        <is>
+          <t>America Mineiro</t>
+        </is>
+      </c>
+      <c r="E769" t="n">
+        <v>10.59</v>
+      </c>
+      <c r="F769" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" s="1" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B770" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C770" t="inlineStr">
+        <is>
+          <t>FC Lahti</t>
+        </is>
+      </c>
+      <c r="D770" t="inlineStr">
+        <is>
+          <t>Jaro</t>
+        </is>
+      </c>
+      <c r="E770" t="n">
+        <v>9.289999999999999</v>
+      </c>
+      <c r="F770" t="n">
+        <v>2.09</v>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" s="1" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B771" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C771" t="inlineStr">
+        <is>
+          <t>Gnistan</t>
+        </is>
+      </c>
+      <c r="D771" t="inlineStr">
+        <is>
+          <t>HJK Helsinki</t>
+        </is>
+      </c>
+      <c r="E771" t="n">
+        <v>10.37</v>
+      </c>
+      <c r="F771" t="n">
+        <v>-0.87</v>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" s="1" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B772" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C772" t="inlineStr">
+        <is>
+          <t>SJK</t>
+        </is>
+      </c>
+      <c r="D772" t="inlineStr">
+        <is>
+          <t>IFK Mariehamn</t>
+        </is>
+      </c>
+      <c r="E772" t="n">
+        <v>10.69</v>
+      </c>
+      <c r="F772" t="n">
+        <v>1.94</v>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" s="1" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B773" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C773" t="inlineStr">
+        <is>
+          <t>FC Haka</t>
+        </is>
+      </c>
+      <c r="D773" t="inlineStr">
+        <is>
+          <t>HJK Klubi 04</t>
+        </is>
+      </c>
+      <c r="E773" t="n">
+        <v>10.73</v>
+      </c>
+      <c r="F773" t="n">
+        <v>2.97</v>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" s="1" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B774" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C774" t="inlineStr">
+        <is>
+          <t>JaPS</t>
+        </is>
+      </c>
+      <c r="D774" t="inlineStr">
+        <is>
+          <t>EIF</t>
+        </is>
+      </c>
+      <c r="E774" t="n">
+        <v>10.86</v>
+      </c>
+      <c r="F774" t="n">
+        <v>-0.34</v>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" s="1" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B775" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C775" t="inlineStr">
+        <is>
+          <t>Polonia Bytom</t>
+        </is>
+      </c>
+      <c r="D775" t="inlineStr">
+        <is>
+          <t>Ruch Chorzow</t>
+        </is>
+      </c>
+      <c r="E775" t="n">
+        <v>10.49</v>
+      </c>
+      <c r="F775" t="n">
+        <v>0.44</v>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" s="1" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B776" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C776" t="inlineStr">
+        <is>
+          <t>Warta Poznan</t>
+        </is>
+      </c>
+      <c r="D776" t="inlineStr">
+        <is>
+          <t>Puszcza Niepolomice</t>
+        </is>
+      </c>
+      <c r="E776" t="n">
+        <v>10.01</v>
+      </c>
+      <c r="F776" t="n">
+        <v>0.98</v>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" s="1" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B777" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C777" t="inlineStr">
+        <is>
+          <t>Widzew Lodz</t>
+        </is>
+      </c>
+      <c r="D777" t="inlineStr">
+        <is>
+          <t>Wieczysta Krakow</t>
+        </is>
+      </c>
+      <c r="E777" t="n">
+        <v>11.01</v>
+      </c>
+      <c r="F777" t="n">
+        <v>1.17</v>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" s="1" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B778" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C778" t="inlineStr">
+        <is>
+          <t>Wisla Krakow</t>
+        </is>
+      </c>
+      <c r="D778" t="inlineStr">
+        <is>
+          <t>Slask Wroclaw</t>
+        </is>
+      </c>
+      <c r="E778" t="n">
+        <v>10.01</v>
+      </c>
+      <c r="F778" t="n">
+        <v>2.03</v>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" s="1" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B779" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C779" t="inlineStr">
+        <is>
+          <t>Rapid Bucuresti</t>
+        </is>
+      </c>
+      <c r="D779" t="inlineStr">
+        <is>
+          <t>Arges Pitesti</t>
+        </is>
+      </c>
+      <c r="E779" t="n">
+        <v>9.470000000000001</v>
+      </c>
+      <c r="F779" t="n">
+        <v>1.91</v>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" s="1" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B780" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C780" t="inlineStr">
+        <is>
+          <t>UTA Arad</t>
+        </is>
+      </c>
+      <c r="D780" t="inlineStr">
+        <is>
+          <t>Sepsi</t>
+        </is>
+      </c>
+      <c r="E780" t="n">
+        <v>9.73</v>
+      </c>
+      <c r="F780" t="n">
+        <v>1.89</v>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" s="1" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B781" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C781" t="inlineStr">
+        <is>
+          <t>Albacete</t>
+        </is>
+      </c>
+      <c r="D781" t="inlineStr">
+        <is>
+          <t>Cordoba</t>
+        </is>
+      </c>
+      <c r="E781" t="n">
+        <v>10.18</v>
+      </c>
+      <c r="F781" t="n">
+        <v>-0.17</v>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" s="1" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B782" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C782" t="inlineStr">
+        <is>
+          <t>Falkenbergs</t>
+        </is>
+      </c>
+      <c r="D782" t="inlineStr">
+        <is>
+          <t>Ostersunds FK</t>
+        </is>
+      </c>
+      <c r="E782" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="F782" t="n">
+        <v>-0.14</v>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" s="1" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B783" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C783" t="inlineStr">
+        <is>
+          <t>Athletic Club</t>
+        </is>
+      </c>
+      <c r="D783" t="inlineStr">
+        <is>
+          <t>Botafogo SP</t>
+        </is>
+      </c>
+      <c r="E783" t="n">
+        <v>10.32</v>
+      </c>
+      <c r="F783" t="n">
+        <v>0.84</v>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" s="1" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B784" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C784" t="inlineStr">
+        <is>
+          <t>Sao Bernardo</t>
+        </is>
+      </c>
+      <c r="D784" t="inlineStr">
+        <is>
+          <t>Atletico Goianiense</t>
+        </is>
+      </c>
+      <c r="E784" t="n">
+        <v>10.47</v>
+      </c>
+      <c r="F784" t="n">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" s="1" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B785" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C785" t="inlineStr">
+        <is>
+          <t>Sport Recife</t>
+        </is>
+      </c>
+      <c r="D785" t="inlineStr">
+        <is>
+          <t>Juventude</t>
+        </is>
+      </c>
+      <c r="E785" t="n">
+        <v>10.32</v>
+      </c>
+      <c r="F785" t="n">
+        <v>0.47</v>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" s="1" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B786" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C786" t="inlineStr">
+        <is>
+          <t>TPS</t>
+        </is>
+      </c>
+      <c r="D786" t="inlineStr">
+        <is>
+          <t>Ilves</t>
+        </is>
+      </c>
+      <c r="E786" t="n">
+        <v>10.51</v>
+      </c>
+      <c r="F786" t="n">
+        <v>-0.19</v>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" s="1" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B787" t="inlineStr">
+        <is>
+          <t>Finland - Veikkausliiga</t>
+        </is>
+      </c>
+      <c r="C787" t="inlineStr">
+        <is>
+          <t>VPS</t>
+        </is>
+      </c>
+      <c r="D787" t="inlineStr">
+        <is>
+          <t>KuPS</t>
+        </is>
+      </c>
+      <c r="E787" t="n">
+        <v>9.82</v>
+      </c>
+      <c r="F787" t="n">
+        <v>-0.42</v>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" s="1" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B788" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C788" t="inlineStr">
+        <is>
+          <t>Mikkelin Palloilijat</t>
+        </is>
+      </c>
+      <c r="D788" t="inlineStr">
+        <is>
+          <t>JIPPO</t>
+        </is>
+      </c>
+      <c r="E788" t="n">
+        <v>10.03</v>
+      </c>
+      <c r="F788" t="n">
+        <v>-1.99</v>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" s="1" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B789" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C789" t="inlineStr">
+        <is>
+          <t>PK-35</t>
+        </is>
+      </c>
+      <c r="D789" t="inlineStr">
+        <is>
+          <t>KTP</t>
+        </is>
+      </c>
+      <c r="E789" t="n">
+        <v>10.53</v>
+      </c>
+      <c r="F789" t="n">
+        <v>-0.04</v>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" s="1" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B790" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C790" t="inlineStr">
+        <is>
+          <t>SJK Akatemia</t>
+        </is>
+      </c>
+      <c r="D790" t="inlineStr">
+        <is>
+          <t>KaPa</t>
+        </is>
+      </c>
+      <c r="E790" t="n">
+        <v>10.79</v>
+      </c>
+      <c r="F790" t="n">
+        <v>0.44</v>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" s="1" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B791" t="inlineStr">
+        <is>
+          <t>Iceland - 1. Deild</t>
+        </is>
+      </c>
+      <c r="C791" t="inlineStr">
+        <is>
+          <t>Throttur Reykjavik</t>
+        </is>
+      </c>
+      <c r="D791" t="inlineStr">
+        <is>
+          <t>Fylkir</t>
+        </is>
+      </c>
+      <c r="E791" t="n">
+        <v>11.38</v>
+      </c>
+      <c r="F791" t="n">
+        <v>2.13</v>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" s="1" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B792" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C792" t="inlineStr">
+        <is>
+          <t>Miedz Legnica</t>
+        </is>
+      </c>
+      <c r="D792" t="inlineStr">
+        <is>
+          <t>Stal Rzeszow</t>
+        </is>
+      </c>
+      <c r="E792" t="n">
+        <v>10.84</v>
+      </c>
+      <c r="F792" t="n">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" s="1" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B793" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C793" t="inlineStr">
+        <is>
+          <t>Pogon Grodzisk Mazowiecki</t>
+        </is>
+      </c>
+      <c r="D793" t="inlineStr">
+        <is>
+          <t>LKS Lodz</t>
+        </is>
+      </c>
+      <c r="E793" t="n">
+        <v>10.94</v>
+      </c>
+      <c r="F793" t="n">
+        <v>-0.7</v>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" s="1" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B794" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C794" t="inlineStr">
+        <is>
+          <t>Polonia Warsaw</t>
+        </is>
+      </c>
+      <c r="D794" t="inlineStr">
+        <is>
+          <t>Chrobry Glogow</t>
+        </is>
+      </c>
+      <c r="E794" t="n">
+        <v>10.76</v>
+      </c>
+      <c r="F794" t="n">
+        <v>1.49</v>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" s="1" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B795" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C795" t="inlineStr">
+        <is>
+          <t>GKS Katowice</t>
+        </is>
+      </c>
+      <c r="D795" t="inlineStr">
+        <is>
+          <t>Cracovia Krakow</t>
+        </is>
+      </c>
+      <c r="E795" t="n">
+        <v>10.85</v>
+      </c>
+      <c r="F795" t="n">
+        <v>0.34</v>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" s="1" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B796" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C796" t="inlineStr">
+        <is>
+          <t>Korona Kielce</t>
+        </is>
+      </c>
+      <c r="D796" t="inlineStr">
+        <is>
+          <t>Rakow Czestochowa</t>
+        </is>
+      </c>
+      <c r="E796" t="n">
+        <v>9.58</v>
+      </c>
+      <c r="F796" t="n">
+        <v>0.72</v>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" s="1" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B797" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C797" t="inlineStr">
+        <is>
+          <t>Motor Lublin</t>
+        </is>
+      </c>
+      <c r="D797" t="inlineStr">
+        <is>
+          <t>Gornik Zabrze</t>
+        </is>
+      </c>
+      <c r="E797" t="n">
+        <v>8.74</v>
+      </c>
+      <c r="F797" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" s="1" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B798" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C798" t="inlineStr">
+        <is>
+          <t>Universitatea Craiova</t>
+        </is>
+      </c>
+      <c r="D798" t="inlineStr">
+        <is>
+          <t>FCSB</t>
+        </is>
+      </c>
+      <c r="E798" t="n">
+        <v>9.619999999999999</v>
+      </c>
+      <c r="F798" t="n">
+        <v>1.92</v>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" s="1" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B799" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C799" t="inlineStr">
+        <is>
+          <t>FC Andorra</t>
+        </is>
+      </c>
+      <c r="D799" t="inlineStr">
+        <is>
+          <t>Sporting Gijon</t>
+        </is>
+      </c>
+      <c r="E799" t="n">
+        <v>9.06</v>
+      </c>
+      <c r="F799" t="n">
+        <v>1.88</v>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" s="1" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B800" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C800" t="inlineStr">
+        <is>
+          <t>Nordic United</t>
+        </is>
+      </c>
+      <c r="D800" t="inlineStr">
+        <is>
+          <t>Landskrona</t>
+        </is>
+      </c>
+      <c r="E800" t="n">
+        <v>10.11</v>
+      </c>
+      <c r="F800" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" s="1" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B801" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C801" t="inlineStr">
+        <is>
+          <t>Oddevold</t>
+        </is>
+      </c>
+      <c r="D801" t="inlineStr">
+        <is>
+          <t>Varnamo</t>
+        </is>
+      </c>
+      <c r="E801" t="n">
+        <v>9.66</v>
+      </c>
+      <c r="F801" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" s="1" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B802" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C802" t="inlineStr">
+        <is>
+          <t>Osters</t>
+        </is>
+      </c>
+      <c r="D802" t="inlineStr">
+        <is>
+          <t>Norrkoping</t>
+        </is>
+      </c>
+      <c r="E802" t="n">
+        <v>10.59</v>
+      </c>
+      <c r="F802" t="n">
+        <v>-1.51</v>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" s="1" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B803" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C803" t="inlineStr">
+        <is>
+          <t>Sandvikens IF</t>
+        </is>
+      </c>
+      <c r="D803" t="inlineStr">
+        <is>
+          <t>Orebro SK</t>
+        </is>
+      </c>
+      <c r="E803" t="n">
+        <v>10.31</v>
+      </c>
+      <c r="F803" t="n">
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" s="1" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B804" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C804" t="inlineStr">
+        <is>
+          <t>Varbergs BoIS</t>
+        </is>
+      </c>
+      <c r="D804" t="inlineStr">
+        <is>
+          <t>Brage</t>
+        </is>
+      </c>
+      <c r="E804" t="n">
+        <v>10.85</v>
+      </c>
+      <c r="F804" t="n">
+        <v>1.94</v>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" s="1" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B805" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C805" t="inlineStr">
+        <is>
+          <t>Goias</t>
+        </is>
+      </c>
+      <c r="D805" t="inlineStr">
+        <is>
+          <t>Avai</t>
+        </is>
+      </c>
+      <c r="E805" t="n">
+        <v>10.21</v>
+      </c>
+      <c r="F805" t="n">
+        <v>1.86</v>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" s="1" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B806" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C806" t="inlineStr">
+        <is>
+          <t>Londrina</t>
+        </is>
+      </c>
+      <c r="D806" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="E806" t="n">
+        <v>10.53</v>
+      </c>
+      <c r="F806" t="n">
+        <v>-0.16</v>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" s="1" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B807" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C807" t="inlineStr">
+        <is>
+          <t>Ponte Preta</t>
+        </is>
+      </c>
+      <c r="D807" t="inlineStr">
+        <is>
+          <t>CRB</t>
+        </is>
+      </c>
+      <c r="E807" t="n">
+        <v>10.69</v>
+      </c>
+      <c r="F807" t="n">
+        <v>-3.12</v>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" s="1" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B808" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C808" t="inlineStr">
+        <is>
+          <t>Haugesund</t>
+        </is>
+      </c>
+      <c r="D808" t="inlineStr">
+        <is>
+          <t>Strommen</t>
+        </is>
+      </c>
+      <c r="E808" t="n">
+        <v>10.67</v>
+      </c>
+      <c r="F808" t="n">
+        <v>3.49</v>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" s="1" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B809" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C809" t="inlineStr">
+        <is>
+          <t>Kongsvinger</t>
+        </is>
+      </c>
+      <c r="D809" t="inlineStr">
+        <is>
+          <t>Hodd</t>
+        </is>
+      </c>
+      <c r="E809" t="n">
+        <v>11.04</v>
+      </c>
+      <c r="F809" t="n">
+        <v>3.51</v>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" s="1" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B810" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C810" t="inlineStr">
+        <is>
+          <t>Lyn</t>
+        </is>
+      </c>
+      <c r="D810" t="inlineStr">
+        <is>
+          <t>Ranheim</t>
+        </is>
+      </c>
+      <c r="E810" t="n">
+        <v>11.24</v>
+      </c>
+      <c r="F810" t="n">
+        <v>0.71</v>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" s="1" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B811" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C811" t="inlineStr">
+        <is>
+          <t>Odd BK</t>
+        </is>
+      </c>
+      <c r="D811" t="inlineStr">
+        <is>
+          <t>Egersunds</t>
+        </is>
+      </c>
+      <c r="E811" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="F811" t="n">
+        <v>1.46</v>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" s="1" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B812" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C812" t="inlineStr">
+        <is>
+          <t>Raufoss</t>
+        </is>
+      </c>
+      <c r="D812" t="inlineStr">
+        <is>
+          <t>Stromsgodset</t>
+        </is>
+      </c>
+      <c r="E812" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="F812" t="n">
+        <v>-3.67</v>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" s="1" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B813" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C813" t="inlineStr">
+        <is>
+          <t>Sandnes Ulf</t>
+        </is>
+      </c>
+      <c r="D813" t="inlineStr">
+        <is>
+          <t>Moss</t>
+        </is>
+      </c>
+      <c r="E813" t="n">
+        <v>11.23</v>
+      </c>
+      <c r="F813" t="n">
+        <v>0.63</v>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" s="1" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B814" t="inlineStr">
+        <is>
+          <t>Norway - 1st Division</t>
+        </is>
+      </c>
+      <c r="C814" t="inlineStr">
+        <is>
+          <t>Stabaek</t>
+        </is>
+      </c>
+      <c r="D814" t="inlineStr">
+        <is>
+          <t>Sogndal</t>
+        </is>
+      </c>
+      <c r="E814" t="n">
+        <v>11.67</v>
+      </c>
+      <c r="F814" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" s="1" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B815" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C815" t="inlineStr">
+        <is>
+          <t>Jagiellonia Bialystok</t>
+        </is>
+      </c>
+      <c r="D815" t="inlineStr">
+        <is>
+          <t>Legia Warsaw</t>
+        </is>
+      </c>
+      <c r="E815" t="n">
+        <v>9.23</v>
+      </c>
+      <c r="F815" t="n">
+        <v>0.21</v>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" s="1" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B816" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C816" t="inlineStr">
+        <is>
+          <t>Lech Poznan</t>
+        </is>
+      </c>
+      <c r="D816" t="inlineStr">
+        <is>
+          <t>Radomiak Radom</t>
+        </is>
+      </c>
+      <c r="E816" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="F816" t="n">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" s="1" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B817" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C817" t="inlineStr">
+        <is>
+          <t>Piast Gliwice</t>
+        </is>
+      </c>
+      <c r="D817" t="inlineStr">
+        <is>
+          <t>Pogon Szczecin</t>
+        </is>
+      </c>
+      <c r="E817" t="n">
+        <v>9.82</v>
+      </c>
+      <c r="F817" t="n">
+        <v>0.41</v>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" s="1" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B818" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C818" t="inlineStr">
+        <is>
+          <t>Zaglebie Lubin</t>
+        </is>
+      </c>
+      <c r="D818" t="inlineStr">
+        <is>
+          <t>Wisla Plock</t>
+        </is>
+      </c>
+      <c r="E818" t="n">
+        <v>10.09</v>
+      </c>
+      <c r="F818" t="n">
+        <v>-0.03</v>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" s="1" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B819" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C819" t="inlineStr">
+        <is>
+          <t>Voluntari</t>
+        </is>
+      </c>
+      <c r="D819" t="inlineStr">
+        <is>
+          <t>Universitatea Cluj</t>
+        </is>
+      </c>
+      <c r="E819" t="n">
+        <v>8.970000000000001</v>
+      </c>
+      <c r="F819" t="n">
+        <v>-0.59</v>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" s="1" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B820" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C820" t="inlineStr">
+        <is>
+          <t>Ceuta</t>
+        </is>
+      </c>
+      <c r="D820" t="inlineStr">
+        <is>
+          <t>Real Valladolid</t>
+        </is>
+      </c>
+      <c r="E820" t="n">
+        <v>8.98</v>
+      </c>
+      <c r="F820" t="n">
+        <v>0.37</v>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" s="1" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B821" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C821" t="inlineStr">
+        <is>
+          <t>Las Palmas</t>
+        </is>
+      </c>
+      <c r="D821" t="inlineStr">
+        <is>
+          <t>Burgos</t>
+        </is>
+      </c>
+      <c r="E821" t="n">
+        <v>9.039999999999999</v>
+      </c>
+      <c r="F821" t="n">
+        <v>1.47</v>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" s="1" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B822" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C822" t="inlineStr">
+        <is>
+          <t>Leganes</t>
+        </is>
+      </c>
+      <c r="D822" t="inlineStr">
+        <is>
+          <t>Granada</t>
+        </is>
+      </c>
+      <c r="E822" t="n">
+        <v>8.77</v>
+      </c>
+      <c r="F822" t="n">
+        <v>0.83</v>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" s="1" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B823" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C823" t="inlineStr">
+        <is>
+          <t>Helsingborgs</t>
+        </is>
+      </c>
+      <c r="D823" t="inlineStr">
+        <is>
+          <t>Norrby</t>
+        </is>
+      </c>
+      <c r="E823" t="n">
+        <v>10.06</v>
+      </c>
+      <c r="F823" t="n">
+        <v>1.47</v>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" s="1" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B824" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C824" t="inlineStr">
+        <is>
+          <t>Sundsvall</t>
+        </is>
+      </c>
+      <c r="D824" t="inlineStr">
+        <is>
+          <t>Ljungskile</t>
+        </is>
+      </c>
+      <c r="E824" t="n">
+        <v>10.62</v>
+      </c>
+      <c r="F824" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" s="1" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B825" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C825" t="inlineStr">
+        <is>
+          <t>Criciuma</t>
+        </is>
+      </c>
+      <c r="D825" t="inlineStr">
+        <is>
+          <t>Operario Ferroviario</t>
+        </is>
+      </c>
+      <c r="E825" t="n">
+        <v>10.62</v>
+      </c>
+      <c r="F825" t="n">
+        <v>2.51</v>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" s="1" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B826" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C826" t="inlineStr">
+        <is>
+          <t>Petrolul Ploiesti</t>
+        </is>
+      </c>
+      <c r="D826" t="inlineStr">
+        <is>
+          <t>Csikszereda</t>
+        </is>
+      </c>
+      <c r="E826" t="n">
+        <v>9.380000000000001</v>
+      </c>
+      <c r="F826" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" s="1" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B827" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C827" t="inlineStr">
+        <is>
+          <t>Cuiaba</t>
+        </is>
+      </c>
+      <c r="D827" t="inlineStr">
+        <is>
+          <t>Nautico</t>
+        </is>
+      </c>
+      <c r="E827" t="n">
+        <v>10.24</v>
+      </c>
+      <c r="F827" t="n">
+        <v>0.68</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily scrape output - 2026-09-19
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F827"/>
+  <dimension ref="A1:F838"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20830,10 +20830,10 @@
         </is>
       </c>
       <c r="E785" t="n">
-        <v>10.32</v>
+        <v>10.22</v>
       </c>
       <c r="F785" t="n">
-        <v>0.47</v>
+        <v>0.46</v>
       </c>
     </row>
     <row r="786">
@@ -20856,10 +20856,10 @@
         </is>
       </c>
       <c r="E786" t="n">
-        <v>10.51</v>
+        <v>10.36</v>
       </c>
       <c r="F786" t="n">
-        <v>-0.19</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="787">
@@ -20882,10 +20882,10 @@
         </is>
       </c>
       <c r="E787" t="n">
-        <v>9.82</v>
+        <v>9.84</v>
       </c>
       <c r="F787" t="n">
-        <v>-0.42</v>
+        <v>-0.57</v>
       </c>
     </row>
     <row r="788">
@@ -20934,10 +20934,10 @@
         </is>
       </c>
       <c r="E789" t="n">
-        <v>10.53</v>
+        <v>10.7</v>
       </c>
       <c r="F789" t="n">
-        <v>-0.04</v>
+        <v>-0.07000000000000001</v>
       </c>
     </row>
     <row r="790">
@@ -20960,7 +20960,7 @@
         </is>
       </c>
       <c r="E790" t="n">
-        <v>10.79</v>
+        <v>10.78</v>
       </c>
       <c r="F790" t="n">
         <v>0.44</v>
@@ -20998,24 +20998,24 @@
       </c>
       <c r="B792" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C792" t="inlineStr">
         <is>
-          <t>Miedz Legnica</t>
+          <t>Asane</t>
         </is>
       </c>
       <c r="D792" t="inlineStr">
         <is>
-          <t>Stal Rzeszow</t>
+          <t>Bryne</t>
         </is>
       </c>
       <c r="E792" t="n">
-        <v>10.84</v>
+        <v>10.74</v>
       </c>
       <c r="F792" t="n">
-        <v>1.6</v>
+        <v>-2.12</v>
       </c>
     </row>
     <row r="793">
@@ -21029,19 +21029,19 @@
       </c>
       <c r="C793" t="inlineStr">
         <is>
-          <t>Pogon Grodzisk Mazowiecki</t>
+          <t>Lechia Gdansk</t>
         </is>
       </c>
       <c r="D793" t="inlineStr">
         <is>
-          <t>LKS Lodz</t>
+          <t>Stal Mielec</t>
         </is>
       </c>
       <c r="E793" t="n">
-        <v>10.94</v>
+        <v>10.56</v>
       </c>
       <c r="F793" t="n">
-        <v>-0.7</v>
+        <v>1.16</v>
       </c>
     </row>
     <row r="794">
@@ -21055,19 +21055,19 @@
       </c>
       <c r="C794" t="inlineStr">
         <is>
-          <t>Polonia Warsaw</t>
+          <t>Miedz Legnica</t>
         </is>
       </c>
       <c r="D794" t="inlineStr">
         <is>
-          <t>Chrobry Glogow</t>
+          <t>Stal Rzeszow</t>
         </is>
       </c>
       <c r="E794" t="n">
-        <v>10.76</v>
+        <v>11.3</v>
       </c>
       <c r="F794" t="n">
-        <v>1.49</v>
+        <v>1.58</v>
       </c>
     </row>
     <row r="795">
@@ -21076,24 +21076,24 @@
       </c>
       <c r="B795" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C795" t="inlineStr">
         <is>
-          <t>GKS Katowice</t>
+          <t>Nieciecza</t>
         </is>
       </c>
       <c r="D795" t="inlineStr">
         <is>
-          <t>Cracovia Krakow</t>
+          <t>Odra Opole</t>
         </is>
       </c>
       <c r="E795" t="n">
-        <v>10.85</v>
+        <v>10.77</v>
       </c>
       <c r="F795" t="n">
-        <v>0.34</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="796">
@@ -21102,24 +21102,24 @@
       </c>
       <c r="B796" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C796" t="inlineStr">
         <is>
-          <t>Korona Kielce</t>
+          <t>Pogon Grodzisk Mazowiecki</t>
         </is>
       </c>
       <c r="D796" t="inlineStr">
         <is>
-          <t>Rakow Czestochowa</t>
+          <t>LKS Lodz</t>
         </is>
       </c>
       <c r="E796" t="n">
-        <v>9.58</v>
+        <v>10.84</v>
       </c>
       <c r="F796" t="n">
-        <v>0.72</v>
+        <v>-1.37</v>
       </c>
     </row>
     <row r="797">
@@ -21128,24 +21128,24 @@
       </c>
       <c r="B797" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C797" t="inlineStr">
         <is>
-          <t>Motor Lublin</t>
+          <t>Polonia Warsaw</t>
         </is>
       </c>
       <c r="D797" t="inlineStr">
         <is>
-          <t>Gornik Zabrze</t>
+          <t>Chrobry Glogow</t>
         </is>
       </c>
       <c r="E797" t="n">
-        <v>8.74</v>
+        <v>10.84</v>
       </c>
       <c r="F797" t="n">
-        <v>-1</v>
+        <v>1.48</v>
       </c>
     </row>
     <row r="798">
@@ -21154,24 +21154,24 @@
       </c>
       <c r="B798" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C798" t="inlineStr">
         <is>
-          <t>Universitatea Craiova</t>
+          <t>GKS Katowice</t>
         </is>
       </c>
       <c r="D798" t="inlineStr">
         <is>
-          <t>FCSB</t>
+          <t>Cracovia Krakow</t>
         </is>
       </c>
       <c r="E798" t="n">
-        <v>9.619999999999999</v>
+        <v>10.78</v>
       </c>
       <c r="F798" t="n">
-        <v>1.92</v>
+        <v>0.36</v>
       </c>
     </row>
     <row r="799">
@@ -21180,24 +21180,24 @@
       </c>
       <c r="B799" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C799" t="inlineStr">
         <is>
-          <t>FC Andorra</t>
+          <t>Korona Kielce</t>
         </is>
       </c>
       <c r="D799" t="inlineStr">
         <is>
-          <t>Sporting Gijon</t>
+          <t>Rakow Czestochowa</t>
         </is>
       </c>
       <c r="E799" t="n">
-        <v>9.06</v>
+        <v>9.58</v>
       </c>
       <c r="F799" t="n">
-        <v>1.88</v>
+        <v>0.72</v>
       </c>
     </row>
     <row r="800">
@@ -21206,24 +21206,24 @@
       </c>
       <c r="B800" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C800" t="inlineStr">
         <is>
-          <t>Nordic United</t>
+          <t>Motor Lublin</t>
         </is>
       </c>
       <c r="D800" t="inlineStr">
         <is>
-          <t>Landskrona</t>
+          <t>Gornik Zabrze</t>
         </is>
       </c>
       <c r="E800" t="n">
-        <v>10.11</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="F800" t="n">
-        <v>0.7</v>
+        <v>-1.02</v>
       </c>
     </row>
     <row r="801">
@@ -21232,24 +21232,24 @@
       </c>
       <c r="B801" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C801" t="inlineStr">
         <is>
-          <t>Oddevold</t>
+          <t>CFR Cluj</t>
         </is>
       </c>
       <c r="D801" t="inlineStr">
         <is>
-          <t>Varnamo</t>
+          <t>Botosani</t>
         </is>
       </c>
       <c r="E801" t="n">
-        <v>9.66</v>
+        <v>9.68</v>
       </c>
       <c r="F801" t="n">
-        <v>1.2</v>
+        <v>1.69</v>
       </c>
     </row>
     <row r="802">
@@ -21258,24 +21258,24 @@
       </c>
       <c r="B802" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C802" t="inlineStr">
         <is>
-          <t>Osters</t>
+          <t>Universitatea Craiova</t>
         </is>
       </c>
       <c r="D802" t="inlineStr">
         <is>
-          <t>Norrkoping</t>
+          <t>FCSB</t>
         </is>
       </c>
       <c r="E802" t="n">
-        <v>10.59</v>
+        <v>9.76</v>
       </c>
       <c r="F802" t="n">
-        <v>-1.51</v>
+        <v>1.92</v>
       </c>
     </row>
     <row r="803">
@@ -21284,24 +21284,24 @@
       </c>
       <c r="B803" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C803" t="inlineStr">
         <is>
-          <t>Sandvikens IF</t>
+          <t>Cadiz</t>
         </is>
       </c>
       <c r="D803" t="inlineStr">
         <is>
-          <t>Orebro SK</t>
+          <t>Girona</t>
         </is>
       </c>
       <c r="E803" t="n">
-        <v>10.31</v>
+        <v>9.09</v>
       </c>
       <c r="F803" t="n">
-        <v>0.51</v>
+        <v>-1.08</v>
       </c>
     </row>
     <row r="804">
@@ -21310,232 +21310,232 @@
       </c>
       <c r="B804" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C804" t="inlineStr">
         <is>
-          <t>Varbergs BoIS</t>
+          <t>Castellon</t>
         </is>
       </c>
       <c r="D804" t="inlineStr">
         <is>
-          <t>Brage</t>
+          <t>Tenerife</t>
         </is>
       </c>
       <c r="E804" t="n">
-        <v>10.85</v>
+        <v>9.77</v>
       </c>
       <c r="F804" t="n">
-        <v>1.94</v>
+        <v>2.59</v>
       </c>
     </row>
     <row r="805">
       <c r="A805" s="1" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B805" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C805" t="inlineStr">
         <is>
-          <t>Goias</t>
+          <t>Eldense</t>
         </is>
       </c>
       <c r="D805" t="inlineStr">
         <is>
-          <t>Avai</t>
+          <t>Eibar</t>
         </is>
       </c>
       <c r="E805" t="n">
-        <v>10.21</v>
+        <v>9.48</v>
       </c>
       <c r="F805" t="n">
-        <v>1.86</v>
+        <v>0.73</v>
       </c>
     </row>
     <row r="806">
       <c r="A806" s="1" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B806" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C806" t="inlineStr">
         <is>
-          <t>Londrina</t>
+          <t>FC Andorra</t>
         </is>
       </c>
       <c r="D806" t="inlineStr">
         <is>
-          <t>Fortaleza</t>
+          <t>Sporting Gijon</t>
         </is>
       </c>
       <c r="E806" t="n">
-        <v>10.53</v>
+        <v>9.06</v>
       </c>
       <c r="F806" t="n">
-        <v>-0.16</v>
+        <v>1.88</v>
       </c>
     </row>
     <row r="807">
       <c r="A807" s="1" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B807" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C807" t="inlineStr">
         <is>
-          <t>Ponte Preta</t>
+          <t>Real Sociedad II</t>
         </is>
       </c>
       <c r="D807" t="inlineStr">
         <is>
-          <t>CRB</t>
+          <t>Mallorca</t>
         </is>
       </c>
       <c r="E807" t="n">
-        <v>10.69</v>
+        <v>9.48</v>
       </c>
       <c r="F807" t="n">
-        <v>-3.12</v>
+        <v>-0.65</v>
       </c>
     </row>
     <row r="808">
       <c r="A808" s="1" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B808" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="C808" t="inlineStr">
         <is>
-          <t>Haugesund</t>
+          <t>Nordic United</t>
         </is>
       </c>
       <c r="D808" t="inlineStr">
         <is>
-          <t>Strommen</t>
+          <t>Landskrona</t>
         </is>
       </c>
       <c r="E808" t="n">
-        <v>10.67</v>
+        <v>10.03</v>
       </c>
       <c r="F808" t="n">
-        <v>3.49</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="809">
       <c r="A809" s="1" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B809" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="C809" t="inlineStr">
         <is>
-          <t>Kongsvinger</t>
+          <t>Oddevold</t>
         </is>
       </c>
       <c r="D809" t="inlineStr">
         <is>
-          <t>Hodd</t>
+          <t>Varnamo</t>
         </is>
       </c>
       <c r="E809" t="n">
-        <v>11.04</v>
+        <v>9.66</v>
       </c>
       <c r="F809" t="n">
-        <v>3.51</v>
+        <v>1.19</v>
       </c>
     </row>
     <row r="810">
       <c r="A810" s="1" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B810" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="C810" t="inlineStr">
         <is>
-          <t>Lyn</t>
+          <t>Osters</t>
         </is>
       </c>
       <c r="D810" t="inlineStr">
         <is>
-          <t>Ranheim</t>
+          <t>Norrkoping</t>
         </is>
       </c>
       <c r="E810" t="n">
-        <v>11.24</v>
+        <v>10.59</v>
       </c>
       <c r="F810" t="n">
-        <v>0.71</v>
+        <v>-1.52</v>
       </c>
     </row>
     <row r="811">
       <c r="A811" s="1" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B811" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="C811" t="inlineStr">
         <is>
-          <t>Odd BK</t>
+          <t>Sandvikens IF</t>
         </is>
       </c>
       <c r="D811" t="inlineStr">
         <is>
-          <t>Egersunds</t>
+          <t>Orebro SK</t>
         </is>
       </c>
       <c r="E811" t="n">
-        <v>10.7</v>
+        <v>10.3</v>
       </c>
       <c r="F811" t="n">
-        <v>1.46</v>
+        <v>0.62</v>
       </c>
     </row>
     <row r="812">
       <c r="A812" s="1" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="B812" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="C812" t="inlineStr">
         <is>
-          <t>Raufoss</t>
+          <t>Varbergs BoIS</t>
         </is>
       </c>
       <c r="D812" t="inlineStr">
         <is>
-          <t>Stromsgodset</t>
+          <t>Brage</t>
         </is>
       </c>
       <c r="E812" t="n">
-        <v>11.5</v>
+        <v>10.85</v>
       </c>
       <c r="F812" t="n">
-        <v>-3.67</v>
+        <v>1.94</v>
       </c>
     </row>
     <row r="813">
@@ -21544,24 +21544,24 @@
       </c>
       <c r="B813" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C813" t="inlineStr">
         <is>
-          <t>Sandnes Ulf</t>
+          <t>Goias</t>
         </is>
       </c>
       <c r="D813" t="inlineStr">
         <is>
-          <t>Moss</t>
+          <t>Avai</t>
         </is>
       </c>
       <c r="E813" t="n">
-        <v>11.23</v>
+        <v>10.12</v>
       </c>
       <c r="F813" t="n">
-        <v>0.63</v>
+        <v>2.39</v>
       </c>
     </row>
     <row r="814">
@@ -21570,24 +21570,24 @@
       </c>
       <c r="B814" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C814" t="inlineStr">
         <is>
-          <t>Stabaek</t>
+          <t>Londrina</t>
         </is>
       </c>
       <c r="D814" t="inlineStr">
         <is>
-          <t>Sogndal</t>
+          <t>Fortaleza</t>
         </is>
       </c>
       <c r="E814" t="n">
-        <v>11.67</v>
+        <v>10.53</v>
       </c>
       <c r="F814" t="n">
-        <v>4</v>
+        <v>-0.16</v>
       </c>
     </row>
     <row r="815">
@@ -21596,24 +21596,24 @@
       </c>
       <c r="B815" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C815" t="inlineStr">
         <is>
-          <t>Jagiellonia Bialystok</t>
+          <t>Ponte Preta</t>
         </is>
       </c>
       <c r="D815" t="inlineStr">
         <is>
-          <t>Legia Warsaw</t>
+          <t>CRB</t>
         </is>
       </c>
       <c r="E815" t="n">
-        <v>9.23</v>
+        <v>10.69</v>
       </c>
       <c r="F815" t="n">
-        <v>0.21</v>
+        <v>-3.12</v>
       </c>
     </row>
     <row r="816">
@@ -21622,24 +21622,24 @@
       </c>
       <c r="B816" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C816" t="inlineStr">
         <is>
-          <t>Lech Poznan</t>
+          <t>Haugesund</t>
         </is>
       </c>
       <c r="D816" t="inlineStr">
         <is>
-          <t>Radomiak Radom</t>
+          <t>Strommen</t>
         </is>
       </c>
       <c r="E816" t="n">
-        <v>10.9</v>
+        <v>10.37</v>
       </c>
       <c r="F816" t="n">
-        <v>3.5</v>
+        <v>3.46</v>
       </c>
     </row>
     <row r="817">
@@ -21648,24 +21648,24 @@
       </c>
       <c r="B817" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C817" t="inlineStr">
         <is>
-          <t>Piast Gliwice</t>
+          <t>Kongsvinger</t>
         </is>
       </c>
       <c r="D817" t="inlineStr">
         <is>
-          <t>Pogon Szczecin</t>
+          <t>Hodd</t>
         </is>
       </c>
       <c r="E817" t="n">
-        <v>9.82</v>
+        <v>11.04</v>
       </c>
       <c r="F817" t="n">
-        <v>0.41</v>
+        <v>3.51</v>
       </c>
     </row>
     <row r="818">
@@ -21674,24 +21674,24 @@
       </c>
       <c r="B818" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C818" t="inlineStr">
         <is>
-          <t>Zaglebie Lubin</t>
+          <t>Lyn</t>
         </is>
       </c>
       <c r="D818" t="inlineStr">
         <is>
-          <t>Wisla Plock</t>
+          <t>Ranheim</t>
         </is>
       </c>
       <c r="E818" t="n">
-        <v>10.09</v>
+        <v>11.23</v>
       </c>
       <c r="F818" t="n">
-        <v>-0.03</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="819">
@@ -21700,24 +21700,24 @@
       </c>
       <c r="B819" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C819" t="inlineStr">
         <is>
-          <t>Voluntari</t>
+          <t>Odd BK</t>
         </is>
       </c>
       <c r="D819" t="inlineStr">
         <is>
-          <t>Universitatea Cluj</t>
+          <t>Egersunds</t>
         </is>
       </c>
       <c r="E819" t="n">
-        <v>8.970000000000001</v>
+        <v>10.68</v>
       </c>
       <c r="F819" t="n">
-        <v>-0.59</v>
+        <v>1.44</v>
       </c>
     </row>
     <row r="820">
@@ -21726,24 +21726,24 @@
       </c>
       <c r="B820" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C820" t="inlineStr">
         <is>
-          <t>Ceuta</t>
+          <t>Raufoss</t>
         </is>
       </c>
       <c r="D820" t="inlineStr">
         <is>
-          <t>Real Valladolid</t>
+          <t>Stromsgodset</t>
         </is>
       </c>
       <c r="E820" t="n">
-        <v>8.98</v>
+        <v>11.7</v>
       </c>
       <c r="F820" t="n">
-        <v>0.37</v>
+        <v>-3.73</v>
       </c>
     </row>
     <row r="821">
@@ -21752,24 +21752,24 @@
       </c>
       <c r="B821" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C821" t="inlineStr">
         <is>
-          <t>Las Palmas</t>
+          <t>Sandnes Ulf</t>
         </is>
       </c>
       <c r="D821" t="inlineStr">
         <is>
-          <t>Burgos</t>
+          <t>Moss</t>
         </is>
       </c>
       <c r="E821" t="n">
-        <v>9.039999999999999</v>
+        <v>11.13</v>
       </c>
       <c r="F821" t="n">
-        <v>1.47</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="822">
@@ -21778,24 +21778,24 @@
       </c>
       <c r="B822" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="C822" t="inlineStr">
         <is>
-          <t>Leganes</t>
+          <t>Stabaek</t>
         </is>
       </c>
       <c r="D822" t="inlineStr">
         <is>
-          <t>Granada</t>
+          <t>Sogndal</t>
         </is>
       </c>
       <c r="E822" t="n">
-        <v>8.77</v>
+        <v>11.63</v>
       </c>
       <c r="F822" t="n">
-        <v>0.83</v>
+        <v>3.36</v>
       </c>
     </row>
     <row r="823">
@@ -21804,24 +21804,24 @@
       </c>
       <c r="B823" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C823" t="inlineStr">
         <is>
-          <t>Helsingborgs</t>
+          <t>Jagiellonia Bialystok</t>
         </is>
       </c>
       <c r="D823" t="inlineStr">
         <is>
-          <t>Norrby</t>
+          <t>Legia Warsaw</t>
         </is>
       </c>
       <c r="E823" t="n">
-        <v>10.06</v>
+        <v>9.23</v>
       </c>
       <c r="F823" t="n">
-        <v>1.47</v>
+        <v>0.21</v>
       </c>
     </row>
     <row r="824">
@@ -21830,101 +21830,387 @@
       </c>
       <c r="B824" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C824" t="inlineStr">
         <is>
-          <t>Sundsvall</t>
+          <t>Lech Poznan</t>
         </is>
       </c>
       <c r="D824" t="inlineStr">
         <is>
-          <t>Ljungskile</t>
+          <t>Radomiak Radom</t>
         </is>
       </c>
       <c r="E824" t="n">
-        <v>10.62</v>
+        <v>10.9</v>
       </c>
       <c r="F824" t="n">
-        <v>-1</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="825">
       <c r="A825" s="1" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B825" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C825" t="inlineStr">
         <is>
-          <t>Criciuma</t>
+          <t>Piast Gliwice</t>
         </is>
       </c>
       <c r="D825" t="inlineStr">
         <is>
-          <t>Operario Ferroviario</t>
+          <t>Pogon Szczecin</t>
         </is>
       </c>
       <c r="E825" t="n">
-        <v>10.62</v>
+        <v>9.82</v>
       </c>
       <c r="F825" t="n">
-        <v>2.51</v>
+        <v>0.41</v>
       </c>
     </row>
     <row r="826">
       <c r="A826" s="1" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B826" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C826" t="inlineStr">
         <is>
-          <t>Petrolul Ploiesti</t>
+          <t>Zaglebie Lubin</t>
         </is>
       </c>
       <c r="D826" t="inlineStr">
         <is>
-          <t>Csikszereda</t>
+          <t>Wisla Plock</t>
         </is>
       </c>
       <c r="E826" t="n">
-        <v>9.380000000000001</v>
+        <v>10.1</v>
       </c>
       <c r="F826" t="n">
-        <v>2</v>
+        <v>-0.16</v>
       </c>
     </row>
     <row r="827">
       <c r="A827" s="1" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B827" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C827" t="inlineStr">
+        <is>
+          <t>Dinamo Bucuresti</t>
+        </is>
+      </c>
+      <c r="D827" t="inlineStr">
+        <is>
+          <t>Farul Constanta</t>
+        </is>
+      </c>
+      <c r="E827" t="n">
+        <v>9.68</v>
+      </c>
+      <c r="F827" t="n">
+        <v>2.39</v>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" s="1" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B828" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C828" t="inlineStr">
+        <is>
+          <t>Voluntari</t>
+        </is>
+      </c>
+      <c r="D828" t="inlineStr">
+        <is>
+          <t>Universitatea Cluj</t>
+        </is>
+      </c>
+      <c r="E828" t="n">
+        <v>8.970000000000001</v>
+      </c>
+      <c r="F828" t="n">
+        <v>-0.59</v>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" s="1" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B829" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C829" t="inlineStr">
+        <is>
+          <t>Almeria</t>
+        </is>
+      </c>
+      <c r="D829" t="inlineStr">
+        <is>
+          <t>Celta Vigo II</t>
+        </is>
+      </c>
+      <c r="E829" t="n">
+        <v>10.24</v>
+      </c>
+      <c r="F829" t="n">
+        <v>2.63</v>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" s="1" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B830" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C830" t="inlineStr">
+        <is>
+          <t>Ceuta</t>
+        </is>
+      </c>
+      <c r="D830" t="inlineStr">
+        <is>
+          <t>Real Valladolid</t>
+        </is>
+      </c>
+      <c r="E830" t="n">
+        <v>8.94</v>
+      </c>
+      <c r="F830" t="n">
+        <v>0.37</v>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" s="1" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B831" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C831" t="inlineStr">
+        <is>
+          <t>Las Palmas</t>
+        </is>
+      </c>
+      <c r="D831" t="inlineStr">
+        <is>
+          <t>Burgos</t>
+        </is>
+      </c>
+      <c r="E831" t="n">
+        <v>9.039999999999999</v>
+      </c>
+      <c r="F831" t="n">
+        <v>1.47</v>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" s="1" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B832" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C832" t="inlineStr">
+        <is>
+          <t>Leganes</t>
+        </is>
+      </c>
+      <c r="D832" t="inlineStr">
+        <is>
+          <t>Granada</t>
+        </is>
+      </c>
+      <c r="E832" t="n">
+        <v>8.77</v>
+      </c>
+      <c r="F832" t="n">
+        <v>0.83</v>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" s="1" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B833" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C833" t="inlineStr">
+        <is>
+          <t>Sabadell</t>
+        </is>
+      </c>
+      <c r="D833" t="inlineStr">
+        <is>
+          <t>Real Oviedo</t>
+        </is>
+      </c>
+      <c r="E833" t="n">
+        <v>8.69</v>
+      </c>
+      <c r="F833" t="n">
+        <v>0.65</v>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" s="1" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B834" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C834" t="inlineStr">
+        <is>
+          <t>Helsingborgs</t>
+        </is>
+      </c>
+      <c r="D834" t="inlineStr">
+        <is>
+          <t>Norrby</t>
+        </is>
+      </c>
+      <c r="E834" t="n">
+        <v>10.06</v>
+      </c>
+      <c r="F834" t="n">
+        <v>1.47</v>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" s="1" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B835" t="inlineStr">
+        <is>
+          <t>Sweden - Superettan</t>
+        </is>
+      </c>
+      <c r="C835" t="inlineStr">
+        <is>
+          <t>Sundsvall</t>
+        </is>
+      </c>
+      <c r="D835" t="inlineStr">
+        <is>
+          <t>Ljungskile</t>
+        </is>
+      </c>
+      <c r="E835" t="n">
+        <v>10.62</v>
+      </c>
+      <c r="F835" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" s="1" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B836" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C836" t="inlineStr">
+        <is>
+          <t>Criciuma</t>
+        </is>
+      </c>
+      <c r="D836" t="inlineStr">
+        <is>
+          <t>Operario Ferroviario</t>
+        </is>
+      </c>
+      <c r="E836" t="n">
+        <v>10.65</v>
+      </c>
+      <c r="F836" t="n">
+        <v>2.51</v>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" s="1" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B837" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C837" t="inlineStr">
+        <is>
+          <t>Petrolul Ploiesti</t>
+        </is>
+      </c>
+      <c r="D837" t="inlineStr">
+        <is>
+          <t>Csikszereda</t>
+        </is>
+      </c>
+      <c r="E837" t="n">
+        <v>9.23</v>
+      </c>
+      <c r="F837" t="n">
+        <v>2.02</v>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" s="1" t="n">
         <v>46287</v>
       </c>
-      <c r="B827" t="inlineStr">
+      <c r="B838" t="inlineStr">
         <is>
           <t>Brazil - Serie B</t>
         </is>
       </c>
-      <c r="C827" t="inlineStr">
+      <c r="C838" t="inlineStr">
         <is>
           <t>Cuiaba</t>
         </is>
       </c>
-      <c r="D827" t="inlineStr">
+      <c r="D838" t="inlineStr">
         <is>
           <t>Nautico</t>
         </is>
       </c>
-      <c r="E827" t="n">
-        <v>10.24</v>
-      </c>
-      <c r="F827" t="n">
+      <c r="E838" t="n">
+        <v>10.16</v>
+      </c>
+      <c r="F838" t="n">
         <v>0.68</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily scrape output - 2026-09-20
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F838"/>
+  <dimension ref="A1:F840"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21584,10 +21584,10 @@
         </is>
       </c>
       <c r="E814" t="n">
-        <v>10.53</v>
+        <v>10.4</v>
       </c>
       <c r="F814" t="n">
-        <v>-0.16</v>
+        <v>-0.15</v>
       </c>
     </row>
     <row r="815">
@@ -21610,10 +21610,10 @@
         </is>
       </c>
       <c r="E815" t="n">
-        <v>10.69</v>
+        <v>10.57</v>
       </c>
       <c r="F815" t="n">
-        <v>-3.12</v>
+        <v>-3.05</v>
       </c>
     </row>
     <row r="816">
@@ -21662,10 +21662,10 @@
         </is>
       </c>
       <c r="E817" t="n">
-        <v>11.04</v>
+        <v>11.06</v>
       </c>
       <c r="F817" t="n">
-        <v>3.51</v>
+        <v>3.74</v>
       </c>
     </row>
     <row r="818">
@@ -21688,10 +21688,10 @@
         </is>
       </c>
       <c r="E818" t="n">
-        <v>11.23</v>
+        <v>11.22</v>
       </c>
       <c r="F818" t="n">
-        <v>0.88</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="819">
@@ -21714,10 +21714,10 @@
         </is>
       </c>
       <c r="E819" t="n">
-        <v>10.68</v>
+        <v>10.35</v>
       </c>
       <c r="F819" t="n">
-        <v>1.44</v>
+        <v>1.46</v>
       </c>
     </row>
     <row r="820">
@@ -21740,10 +21740,10 @@
         </is>
       </c>
       <c r="E820" t="n">
-        <v>11.7</v>
+        <v>12.15</v>
       </c>
       <c r="F820" t="n">
-        <v>-3.73</v>
+        <v>-3.99</v>
       </c>
     </row>
     <row r="821">
@@ -21792,10 +21792,10 @@
         </is>
       </c>
       <c r="E822" t="n">
-        <v>11.63</v>
+        <v>11.79</v>
       </c>
       <c r="F822" t="n">
-        <v>3.36</v>
+        <v>3.65</v>
       </c>
     </row>
     <row r="823">
@@ -21804,24 +21804,24 @@
       </c>
       <c r="B823" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C823" t="inlineStr">
         <is>
-          <t>Jagiellonia Bialystok</t>
+          <t>Podbeskidzie Bielsko-Biala</t>
         </is>
       </c>
       <c r="D823" t="inlineStr">
         <is>
-          <t>Legia Warsaw</t>
+          <t>Unia Skierniewice</t>
         </is>
       </c>
       <c r="E823" t="n">
-        <v>9.23</v>
+        <v>10.16</v>
       </c>
       <c r="F823" t="n">
-        <v>0.21</v>
+        <v>0.89</v>
       </c>
     </row>
     <row r="824">
@@ -21830,24 +21830,24 @@
       </c>
       <c r="B824" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C824" t="inlineStr">
         <is>
-          <t>Lech Poznan</t>
+          <t>Pogon Siedlce</t>
         </is>
       </c>
       <c r="D824" t="inlineStr">
         <is>
-          <t>Radomiak Radom</t>
+          <t>Arka Gdynia</t>
         </is>
       </c>
       <c r="E824" t="n">
-        <v>10.9</v>
+        <v>10.38</v>
       </c>
       <c r="F824" t="n">
-        <v>3.5</v>
+        <v>-1.12</v>
       </c>
     </row>
     <row r="825">
@@ -21861,19 +21861,19 @@
       </c>
       <c r="C825" t="inlineStr">
         <is>
-          <t>Piast Gliwice</t>
+          <t>Jagiellonia Bialystok</t>
         </is>
       </c>
       <c r="D825" t="inlineStr">
         <is>
-          <t>Pogon Szczecin</t>
+          <t>Legia Warsaw</t>
         </is>
       </c>
       <c r="E825" t="n">
-        <v>9.82</v>
+        <v>9.23</v>
       </c>
       <c r="F825" t="n">
-        <v>0.41</v>
+        <v>0.21</v>
       </c>
     </row>
     <row r="826">
@@ -21887,19 +21887,19 @@
       </c>
       <c r="C826" t="inlineStr">
         <is>
-          <t>Zaglebie Lubin</t>
+          <t>Lech Poznan</t>
         </is>
       </c>
       <c r="D826" t="inlineStr">
         <is>
-          <t>Wisla Plock</t>
+          <t>Radomiak Radom</t>
         </is>
       </c>
       <c r="E826" t="n">
-        <v>10.1</v>
+        <v>10.9</v>
       </c>
       <c r="F826" t="n">
-        <v>-0.16</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="827">
@@ -21908,24 +21908,24 @@
       </c>
       <c r="B827" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C827" t="inlineStr">
         <is>
-          <t>Dinamo Bucuresti</t>
+          <t>Piast Gliwice</t>
         </is>
       </c>
       <c r="D827" t="inlineStr">
         <is>
-          <t>Farul Constanta</t>
+          <t>Pogon Szczecin</t>
         </is>
       </c>
       <c r="E827" t="n">
-        <v>9.68</v>
+        <v>9.82</v>
       </c>
       <c r="F827" t="n">
-        <v>2.39</v>
+        <v>0.41</v>
       </c>
     </row>
     <row r="828">
@@ -21934,24 +21934,24 @@
       </c>
       <c r="B828" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C828" t="inlineStr">
         <is>
-          <t>Voluntari</t>
+          <t>Zaglebie Lubin</t>
         </is>
       </c>
       <c r="D828" t="inlineStr">
         <is>
-          <t>Universitatea Cluj</t>
+          <t>Wisla Plock</t>
         </is>
       </c>
       <c r="E828" t="n">
-        <v>8.970000000000001</v>
+        <v>10.1</v>
       </c>
       <c r="F828" t="n">
-        <v>-0.59</v>
+        <v>-0.16</v>
       </c>
     </row>
     <row r="829">
@@ -21960,24 +21960,24 @@
       </c>
       <c r="B829" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C829" t="inlineStr">
         <is>
-          <t>Almeria</t>
+          <t>Dinamo Bucuresti</t>
         </is>
       </c>
       <c r="D829" t="inlineStr">
         <is>
-          <t>Celta Vigo II</t>
+          <t>Farul Constanta</t>
         </is>
       </c>
       <c r="E829" t="n">
-        <v>10.24</v>
+        <v>9.68</v>
       </c>
       <c r="F829" t="n">
-        <v>2.63</v>
+        <v>2.23</v>
       </c>
     </row>
     <row r="830">
@@ -21986,24 +21986,24 @@
       </c>
       <c r="B830" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="C830" t="inlineStr">
         <is>
-          <t>Ceuta</t>
+          <t>Voluntari</t>
         </is>
       </c>
       <c r="D830" t="inlineStr">
         <is>
-          <t>Real Valladolid</t>
+          <t>Universitatea Cluj</t>
         </is>
       </c>
       <c r="E830" t="n">
-        <v>8.94</v>
+        <v>9.23</v>
       </c>
       <c r="F830" t="n">
-        <v>0.37</v>
+        <v>-0.5</v>
       </c>
     </row>
     <row r="831">
@@ -22017,19 +22017,19 @@
       </c>
       <c r="C831" t="inlineStr">
         <is>
-          <t>Las Palmas</t>
+          <t>Almeria</t>
         </is>
       </c>
       <c r="D831" t="inlineStr">
         <is>
-          <t>Burgos</t>
+          <t>Celta Vigo II</t>
         </is>
       </c>
       <c r="E831" t="n">
-        <v>9.039999999999999</v>
+        <v>10.09</v>
       </c>
       <c r="F831" t="n">
-        <v>1.47</v>
+        <v>2.63</v>
       </c>
     </row>
     <row r="832">
@@ -22043,19 +22043,19 @@
       </c>
       <c r="C832" t="inlineStr">
         <is>
-          <t>Leganes</t>
+          <t>Ceuta</t>
         </is>
       </c>
       <c r="D832" t="inlineStr">
         <is>
-          <t>Granada</t>
+          <t>Real Valladolid</t>
         </is>
       </c>
       <c r="E832" t="n">
-        <v>8.77</v>
+        <v>8.720000000000001</v>
       </c>
       <c r="F832" t="n">
-        <v>0.83</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="833">
@@ -22069,19 +22069,19 @@
       </c>
       <c r="C833" t="inlineStr">
         <is>
-          <t>Sabadell</t>
+          <t>Las Palmas</t>
         </is>
       </c>
       <c r="D833" t="inlineStr">
         <is>
-          <t>Real Oviedo</t>
+          <t>Burgos</t>
         </is>
       </c>
       <c r="E833" t="n">
-        <v>8.69</v>
+        <v>8.85</v>
       </c>
       <c r="F833" t="n">
-        <v>0.65</v>
+        <v>1.48</v>
       </c>
     </row>
     <row r="834">
@@ -22090,24 +22090,24 @@
       </c>
       <c r="B834" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C834" t="inlineStr">
         <is>
-          <t>Helsingborgs</t>
+          <t>Leganes</t>
         </is>
       </c>
       <c r="D834" t="inlineStr">
         <is>
-          <t>Norrby</t>
+          <t>Granada</t>
         </is>
       </c>
       <c r="E834" t="n">
-        <v>10.06</v>
+        <v>8.69</v>
       </c>
       <c r="F834" t="n">
-        <v>1.47</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="835">
@@ -22116,101 +22116,153 @@
       </c>
       <c r="B835" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C835" t="inlineStr">
         <is>
-          <t>Sundsvall</t>
+          <t>Sabadell</t>
         </is>
       </c>
       <c r="D835" t="inlineStr">
         <is>
-          <t>Ljungskile</t>
+          <t>Real Oviedo</t>
         </is>
       </c>
       <c r="E835" t="n">
-        <v>10.62</v>
+        <v>8.69</v>
       </c>
       <c r="F835" t="n">
-        <v>-1</v>
+        <v>0.65</v>
       </c>
     </row>
     <row r="836">
       <c r="A836" s="1" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B836" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="C836" t="inlineStr">
         <is>
-          <t>Criciuma</t>
+          <t>Helsingborgs</t>
         </is>
       </c>
       <c r="D836" t="inlineStr">
         <is>
-          <t>Operario Ferroviario</t>
+          <t>Norrby</t>
         </is>
       </c>
       <c r="E836" t="n">
-        <v>10.65</v>
+        <v>10.26</v>
       </c>
       <c r="F836" t="n">
-        <v>2.51</v>
+        <v>1.47</v>
       </c>
     </row>
     <row r="837">
       <c r="A837" s="1" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B837" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="C837" t="inlineStr">
         <is>
-          <t>Petrolul Ploiesti</t>
+          <t>Sundsvall</t>
         </is>
       </c>
       <c r="D837" t="inlineStr">
         <is>
-          <t>Csikszereda</t>
+          <t>Ljungskile</t>
         </is>
       </c>
       <c r="E837" t="n">
-        <v>9.23</v>
+        <v>10.55</v>
       </c>
       <c r="F837" t="n">
-        <v>2.02</v>
+        <v>-0.99</v>
       </c>
     </row>
     <row r="838">
       <c r="A838" s="1" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B838" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C838" t="inlineStr">
+        <is>
+          <t>Criciuma</t>
+        </is>
+      </c>
+      <c r="D838" t="inlineStr">
+        <is>
+          <t>Operario Ferroviario</t>
+        </is>
+      </c>
+      <c r="E838" t="n">
+        <v>10.73</v>
+      </c>
+      <c r="F838" t="n">
+        <v>2.52</v>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" s="1" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B839" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C839" t="inlineStr">
+        <is>
+          <t>Petrolul Ploiesti</t>
+        </is>
+      </c>
+      <c r="D839" t="inlineStr">
+        <is>
+          <t>Csikszereda</t>
+        </is>
+      </c>
+      <c r="E839" t="n">
+        <v>9.23</v>
+      </c>
+      <c r="F839" t="n">
+        <v>2.02</v>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" s="1" t="n">
         <v>46287</v>
       </c>
-      <c r="B838" t="inlineStr">
+      <c r="B840" t="inlineStr">
         <is>
           <t>Brazil - Serie B</t>
         </is>
       </c>
-      <c r="C838" t="inlineStr">
+      <c r="C840" t="inlineStr">
         <is>
           <t>Cuiaba</t>
         </is>
       </c>
-      <c r="D838" t="inlineStr">
+      <c r="D840" t="inlineStr">
         <is>
           <t>Nautico</t>
         </is>
       </c>
-      <c r="E838" t="n">
+      <c r="E840" t="n">
         <v>10.16</v>
       </c>
-      <c r="F838" t="n">
+      <c r="F840" t="n">
         <v>0.68</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily scrape output - 2026-09-21
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F840"/>
+  <dimension ref="A1:F841"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22208,10 +22208,10 @@
         </is>
       </c>
       <c r="E838" t="n">
-        <v>10.73</v>
+        <v>10.24</v>
       </c>
       <c r="F838" t="n">
-        <v>2.52</v>
+        <v>2.74</v>
       </c>
     </row>
     <row r="839">
@@ -22225,44 +22225,70 @@
       </c>
       <c r="C839" t="inlineStr">
         <is>
-          <t>Petrolul Ploiesti</t>
+          <t>Otelul Galati</t>
         </is>
       </c>
       <c r="D839" t="inlineStr">
         <is>
-          <t>Csikszereda</t>
+          <t>Corvinul Hunedoara</t>
         </is>
       </c>
       <c r="E839" t="n">
-        <v>9.23</v>
+        <v>8.619999999999999</v>
       </c>
       <c r="F839" t="n">
-        <v>2.02</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="840">
       <c r="A840" s="1" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B840" t="inlineStr">
+        <is>
+          <t>Romania - Liga 1</t>
+        </is>
+      </c>
+      <c r="C840" t="inlineStr">
+        <is>
+          <t>Petrolul Ploiesti</t>
+        </is>
+      </c>
+      <c r="D840" t="inlineStr">
+        <is>
+          <t>Csikszereda</t>
+        </is>
+      </c>
+      <c r="E840" t="n">
+        <v>9.32</v>
+      </c>
+      <c r="F840" t="n">
+        <v>2.17</v>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" s="1" t="n">
         <v>46287</v>
       </c>
-      <c r="B840" t="inlineStr">
+      <c r="B841" t="inlineStr">
         <is>
           <t>Brazil - Serie B</t>
         </is>
       </c>
-      <c r="C840" t="inlineStr">
+      <c r="C841" t="inlineStr">
         <is>
           <t>Cuiaba</t>
         </is>
       </c>
-      <c r="D840" t="inlineStr">
+      <c r="D841" t="inlineStr">
         <is>
           <t>Nautico</t>
         </is>
       </c>
-      <c r="E840" t="n">
+      <c r="E841" t="n">
         <v>10.16</v>
       </c>
-      <c r="F840" t="n">
+      <c r="F841" t="n">
         <v>0.68</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily scrape output - 2026-09-22
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F841"/>
+  <dimension ref="A1:F842"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22277,18 +22277,44 @@
       </c>
       <c r="C841" t="inlineStr">
         <is>
+          <t>Criciuma</t>
+        </is>
+      </c>
+      <c r="D841" t="inlineStr">
+        <is>
+          <t>Operario Ferroviario</t>
+        </is>
+      </c>
+      <c r="E841" t="n">
+        <v>10.69</v>
+      </c>
+      <c r="F841" t="n">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" s="1" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B842" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C842" t="inlineStr">
+        <is>
           <t>Cuiaba</t>
         </is>
       </c>
-      <c r="D841" t="inlineStr">
+      <c r="D842" t="inlineStr">
         <is>
           <t>Nautico</t>
         </is>
       </c>
-      <c r="E841" t="n">
+      <c r="E842" t="n">
         <v>10.16</v>
       </c>
-      <c r="F841" t="n">
+      <c r="F842" t="n">
         <v>0.68</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily scrape output - 2026-09-24
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F842"/>
+  <dimension ref="A1:F847"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22318,6 +22318,136 @@
         <v>0.68</v>
       </c>
     </row>
+    <row r="843">
+      <c r="A843" s="1" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B843" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C843" t="inlineStr">
+        <is>
+          <t>Girona</t>
+        </is>
+      </c>
+      <c r="D843" t="inlineStr">
+        <is>
+          <t>Albacete</t>
+        </is>
+      </c>
+      <c r="E843" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="F843" t="n">
+        <v>2.09</v>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" s="1" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B844" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C844" t="inlineStr">
+        <is>
+          <t>Celta Vigo II</t>
+        </is>
+      </c>
+      <c r="D844" t="inlineStr">
+        <is>
+          <t>Sabadell</t>
+        </is>
+      </c>
+      <c r="E844" t="n">
+        <v>8.65</v>
+      </c>
+      <c r="F844" t="n">
+        <v>-0.8100000000000001</v>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" s="1" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B845" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C845" t="inlineStr">
+        <is>
+          <t>Ceuta</t>
+        </is>
+      </c>
+      <c r="D845" t="inlineStr">
+        <is>
+          <t>Real Sociedad II</t>
+        </is>
+      </c>
+      <c r="E845" t="n">
+        <v>9.550000000000001</v>
+      </c>
+      <c r="F845" t="n">
+        <v>0.82</v>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" s="1" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B846" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C846" t="inlineStr">
+        <is>
+          <t>Granada</t>
+        </is>
+      </c>
+      <c r="D846" t="inlineStr">
+        <is>
+          <t>FC Andorra</t>
+        </is>
+      </c>
+      <c r="E846" t="n">
+        <v>8.51</v>
+      </c>
+      <c r="F846" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" s="1" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B847" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C847" t="inlineStr">
+        <is>
+          <t>Tenerife</t>
+        </is>
+      </c>
+      <c r="D847" t="inlineStr">
+        <is>
+          <t>Cadiz</t>
+        </is>
+      </c>
+      <c r="E847" t="n">
+        <v>9.550000000000001</v>
+      </c>
+      <c r="F847" t="n">
+        <v>1.87</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily scrape output - 2026-09-25
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F847"/>
+  <dimension ref="A1:F862"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22324,81 +22324,81 @@
       </c>
       <c r="B843" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C843" t="inlineStr">
         <is>
-          <t>Girona</t>
+          <t>Gremio Novorizontino</t>
         </is>
       </c>
       <c r="D843" t="inlineStr">
         <is>
-          <t>Albacete</t>
+          <t>Sao Bernardo</t>
         </is>
       </c>
       <c r="E843" t="n">
-        <v>9.5</v>
+        <v>11.13</v>
       </c>
       <c r="F843" t="n">
-        <v>2.09</v>
+        <v>2.73</v>
       </c>
     </row>
     <row r="844">
       <c r="A844" s="1" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B844" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C844" t="inlineStr">
         <is>
-          <t>Celta Vigo II</t>
+          <t>Vila Nova</t>
         </is>
       </c>
       <c r="D844" t="inlineStr">
         <is>
-          <t>Sabadell</t>
+          <t>Londrina</t>
         </is>
       </c>
       <c r="E844" t="n">
-        <v>8.65</v>
+        <v>10.62</v>
       </c>
       <c r="F844" t="n">
-        <v>-0.8100000000000001</v>
+        <v>2.12</v>
       </c>
     </row>
     <row r="845">
       <c r="A845" s="1" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B845" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Finland - Ykkosliiga</t>
         </is>
       </c>
       <c r="C845" t="inlineStr">
         <is>
-          <t>Ceuta</t>
+          <t>KaPa</t>
         </is>
       </c>
       <c r="D845" t="inlineStr">
         <is>
-          <t>Real Sociedad II</t>
+          <t>FC Haka</t>
         </is>
       </c>
       <c r="E845" t="n">
-        <v>9.550000000000001</v>
+        <v>10.61</v>
       </c>
       <c r="F845" t="n">
-        <v>0.82</v>
+        <v>-2.43</v>
       </c>
     </row>
     <row r="846">
       <c r="A846" s="1" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B846" t="inlineStr">
         <is>
@@ -22407,19 +22407,19 @@
       </c>
       <c r="C846" t="inlineStr">
         <is>
-          <t>Granada</t>
+          <t>Girona</t>
         </is>
       </c>
       <c r="D846" t="inlineStr">
         <is>
-          <t>FC Andorra</t>
+          <t>Albacete</t>
         </is>
       </c>
       <c r="E846" t="n">
-        <v>8.51</v>
+        <v>9.51</v>
       </c>
       <c r="F846" t="n">
-        <v>0.5600000000000001</v>
+        <v>2.38</v>
       </c>
     </row>
     <row r="847">
@@ -22428,24 +22428,414 @@
       </c>
       <c r="B847" t="inlineStr">
         <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C847" t="inlineStr">
+        <is>
+          <t>Goias</t>
+        </is>
+      </c>
+      <c r="D847" t="inlineStr">
+        <is>
+          <t>Atletico Goianiense</t>
+        </is>
+      </c>
+      <c r="E847" t="n">
+        <v>10.34</v>
+      </c>
+      <c r="F847" t="n">
+        <v>0.86</v>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" s="1" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B848" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C848" t="inlineStr">
+        <is>
+          <t>Operario Ferroviario</t>
+        </is>
+      </c>
+      <c r="D848" t="inlineStr">
+        <is>
+          <t>Ceara</t>
+        </is>
+      </c>
+      <c r="E848" t="n">
+        <v>10.33</v>
+      </c>
+      <c r="F848" t="n">
+        <v>0.64</v>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" s="1" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B849" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C849" t="inlineStr">
+        <is>
+          <t>EIF</t>
+        </is>
+      </c>
+      <c r="D849" t="inlineStr">
+        <is>
+          <t>SJK Akatemia</t>
+        </is>
+      </c>
+      <c r="E849" t="n">
+        <v>10.55</v>
+      </c>
+      <c r="F849" t="n">
+        <v>2.47</v>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" s="1" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B850" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C850" t="inlineStr">
+        <is>
+          <t>HJK Klubi 04</t>
+        </is>
+      </c>
+      <c r="D850" t="inlineStr">
+        <is>
+          <t>JaPS</t>
+        </is>
+      </c>
+      <c r="E850" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="F850" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" s="1" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B851" t="inlineStr">
+        <is>
+          <t>Finland - Ykkosliiga</t>
+        </is>
+      </c>
+      <c r="C851" t="inlineStr">
+        <is>
+          <t>JIPPO</t>
+        </is>
+      </c>
+      <c r="D851" t="inlineStr">
+        <is>
+          <t>PK-35</t>
+        </is>
+      </c>
+      <c r="E851" t="n">
+        <v>9.859999999999999</v>
+      </c>
+      <c r="F851" t="n">
+        <v>1.36</v>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" s="1" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B852" t="inlineStr">
+        <is>
           <t>Spain - Segunda</t>
         </is>
       </c>
-      <c r="C847" t="inlineStr">
+      <c r="C852" t="inlineStr">
+        <is>
+          <t>Celta Vigo II</t>
+        </is>
+      </c>
+      <c r="D852" t="inlineStr">
+        <is>
+          <t>Sabadell</t>
+        </is>
+      </c>
+      <c r="E852" t="n">
+        <v>8.49</v>
+      </c>
+      <c r="F852" t="n">
+        <v>-0.71</v>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" s="1" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B853" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C853" t="inlineStr">
+        <is>
+          <t>Ceuta</t>
+        </is>
+      </c>
+      <c r="D853" t="inlineStr">
+        <is>
+          <t>Real Sociedad II</t>
+        </is>
+      </c>
+      <c r="E853" t="n">
+        <v>9.44</v>
+      </c>
+      <c r="F853" t="n">
+        <v>0.83</v>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" s="1" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B854" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C854" t="inlineStr">
+        <is>
+          <t>Granada</t>
+        </is>
+      </c>
+      <c r="D854" t="inlineStr">
+        <is>
+          <t>FC Andorra</t>
+        </is>
+      </c>
+      <c r="E854" t="n">
+        <v>8.49</v>
+      </c>
+      <c r="F854" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" s="1" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B855" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C855" t="inlineStr">
         <is>
           <t>Tenerife</t>
         </is>
       </c>
-      <c r="D847" t="inlineStr">
+      <c r="D855" t="inlineStr">
         <is>
           <t>Cadiz</t>
         </is>
       </c>
-      <c r="E847" t="n">
-        <v>9.550000000000001</v>
-      </c>
-      <c r="F847" t="n">
-        <v>1.87</v>
+      <c r="E855" t="n">
+        <v>9.640000000000001</v>
+      </c>
+      <c r="F855" t="n">
+        <v>1.86</v>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" s="1" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B856" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C856" t="inlineStr">
+        <is>
+          <t>CRB</t>
+        </is>
+      </c>
+      <c r="D856" t="inlineStr">
+        <is>
+          <t>Cuiaba</t>
+        </is>
+      </c>
+      <c r="E856" t="n">
+        <v>10.05</v>
+      </c>
+      <c r="F856" t="n">
+        <v>1.93</v>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" s="1" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B857" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C857" t="inlineStr">
+        <is>
+          <t>Criciuma</t>
+        </is>
+      </c>
+      <c r="D857" t="inlineStr">
+        <is>
+          <t>Avai</t>
+        </is>
+      </c>
+      <c r="E857" t="n">
+        <v>10.78</v>
+      </c>
+      <c r="F857" t="n">
+        <v>3.56</v>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" s="1" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B858" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C858" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="D858" t="inlineStr">
+        <is>
+          <t>Athletic Club</t>
+        </is>
+      </c>
+      <c r="E858" t="n">
+        <v>10.02</v>
+      </c>
+      <c r="F858" t="n">
+        <v>2.76</v>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" s="1" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B859" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C859" t="inlineStr">
+        <is>
+          <t>Eibar</t>
+        </is>
+      </c>
+      <c r="D859" t="inlineStr">
+        <is>
+          <t>Las Palmas</t>
+        </is>
+      </c>
+      <c r="E859" t="n">
+        <v>9.15</v>
+      </c>
+      <c r="F859" t="n">
+        <v>0.92</v>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" s="1" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B860" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C860" t="inlineStr">
+        <is>
+          <t>Real Valladolid</t>
+        </is>
+      </c>
+      <c r="D860" t="inlineStr">
+        <is>
+          <t>Cordoba</t>
+        </is>
+      </c>
+      <c r="E860" t="n">
+        <v>9.380000000000001</v>
+      </c>
+      <c r="F860" t="n">
+        <v>0.38</v>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" s="1" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B861" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C861" t="inlineStr">
+        <is>
+          <t>America Mineiro</t>
+        </is>
+      </c>
+      <c r="D861" t="inlineStr">
+        <is>
+          <t>Juventude</t>
+        </is>
+      </c>
+      <c r="E861" t="n">
+        <v>10.28</v>
+      </c>
+      <c r="F861" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" s="1" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B862" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C862" t="inlineStr">
+        <is>
+          <t>Leganes</t>
+        </is>
+      </c>
+      <c r="D862" t="inlineStr">
+        <is>
+          <t>Castellon</t>
+        </is>
+      </c>
+      <c r="E862" t="n">
+        <v>9.27</v>
+      </c>
+      <c r="F862" t="n">
+        <v>-0.83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-09-26
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F862"/>
+  <dimension ref="A1:F867"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22442,10 +22442,10 @@
         </is>
       </c>
       <c r="E847" t="n">
-        <v>10.34</v>
+        <v>9.720000000000001</v>
       </c>
       <c r="F847" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="848">
@@ -22459,19 +22459,19 @@
       </c>
       <c r="C848" t="inlineStr">
         <is>
-          <t>Operario Ferroviario</t>
+          <t>Nautico</t>
         </is>
       </c>
       <c r="D848" t="inlineStr">
         <is>
-          <t>Ceara</t>
+          <t>Sport Recife</t>
         </is>
       </c>
       <c r="E848" t="n">
-        <v>10.33</v>
+        <v>10.56</v>
       </c>
       <c r="F848" t="n">
-        <v>0.64</v>
+        <v>1.85</v>
       </c>
     </row>
     <row r="849">
@@ -22480,24 +22480,24 @@
       </c>
       <c r="B849" t="inlineStr">
         <is>
-          <t>Finland - Ykkosliiga</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C849" t="inlineStr">
         <is>
-          <t>EIF</t>
+          <t>Operario Ferroviario</t>
         </is>
       </c>
       <c r="D849" t="inlineStr">
         <is>
-          <t>SJK Akatemia</t>
+          <t>Ceara</t>
         </is>
       </c>
       <c r="E849" t="n">
-        <v>10.55</v>
+        <v>10.21</v>
       </c>
       <c r="F849" t="n">
-        <v>2.47</v>
+        <v>0.65</v>
       </c>
     </row>
     <row r="850">
@@ -22511,19 +22511,19 @@
       </c>
       <c r="C850" t="inlineStr">
         <is>
-          <t>HJK Klubi 04</t>
+          <t>EIF</t>
         </is>
       </c>
       <c r="D850" t="inlineStr">
         <is>
-          <t>JaPS</t>
+          <t>SJK Akatemia</t>
         </is>
       </c>
       <c r="E850" t="n">
-        <v>10.4</v>
+        <v>10.76</v>
       </c>
       <c r="F850" t="n">
-        <v>0.6899999999999999</v>
+        <v>2.47</v>
       </c>
     </row>
     <row r="851">
@@ -22537,19 +22537,19 @@
       </c>
       <c r="C851" t="inlineStr">
         <is>
-          <t>JIPPO</t>
+          <t>HJK Klubi 04</t>
         </is>
       </c>
       <c r="D851" t="inlineStr">
         <is>
-          <t>PK-35</t>
+          <t>JaPS</t>
         </is>
       </c>
       <c r="E851" t="n">
-        <v>9.859999999999999</v>
+        <v>10.4</v>
       </c>
       <c r="F851" t="n">
-        <v>1.36</v>
+        <v>0.6899999999999999</v>
       </c>
     </row>
     <row r="852">
@@ -22558,24 +22558,24 @@
       </c>
       <c r="B852" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Finland - Ykkosliiga</t>
         </is>
       </c>
       <c r="C852" t="inlineStr">
         <is>
-          <t>Celta Vigo II</t>
+          <t>JIPPO</t>
         </is>
       </c>
       <c r="D852" t="inlineStr">
         <is>
-          <t>Sabadell</t>
+          <t>PK-35</t>
         </is>
       </c>
       <c r="E852" t="n">
-        <v>8.49</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="F852" t="n">
-        <v>-0.71</v>
+        <v>1.46</v>
       </c>
     </row>
     <row r="853">
@@ -22589,19 +22589,19 @@
       </c>
       <c r="C853" t="inlineStr">
         <is>
-          <t>Ceuta</t>
+          <t>Celta Vigo II</t>
         </is>
       </c>
       <c r="D853" t="inlineStr">
         <is>
-          <t>Real Sociedad II</t>
+          <t>Sabadell</t>
         </is>
       </c>
       <c r="E853" t="n">
-        <v>9.44</v>
+        <v>8.359999999999999</v>
       </c>
       <c r="F853" t="n">
-        <v>0.83</v>
+        <v>-0.32</v>
       </c>
     </row>
     <row r="854">
@@ -22615,19 +22615,19 @@
       </c>
       <c r="C854" t="inlineStr">
         <is>
-          <t>Granada</t>
+          <t>Ceuta</t>
         </is>
       </c>
       <c r="D854" t="inlineStr">
         <is>
-          <t>FC Andorra</t>
+          <t>Real Sociedad II</t>
         </is>
       </c>
       <c r="E854" t="n">
-        <v>8.49</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="F854" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.58</v>
       </c>
     </row>
     <row r="855">
@@ -22641,45 +22641,45 @@
       </c>
       <c r="C855" t="inlineStr">
         <is>
-          <t>Tenerife</t>
+          <t>Granada</t>
         </is>
       </c>
       <c r="D855" t="inlineStr">
         <is>
-          <t>Cadiz</t>
+          <t>FC Andorra</t>
         </is>
       </c>
       <c r="E855" t="n">
-        <v>9.640000000000001</v>
+        <v>8.529999999999999</v>
       </c>
       <c r="F855" t="n">
-        <v>1.86</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="856">
       <c r="A856" s="1" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B856" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C856" t="inlineStr">
         <is>
-          <t>CRB</t>
+          <t>Tenerife</t>
         </is>
       </c>
       <c r="D856" t="inlineStr">
         <is>
-          <t>Cuiaba</t>
+          <t>Cadiz</t>
         </is>
       </c>
       <c r="E856" t="n">
-        <v>10.05</v>
+        <v>9.5</v>
       </c>
       <c r="F856" t="n">
-        <v>1.93</v>
+        <v>1.95</v>
       </c>
     </row>
     <row r="857">
@@ -22693,19 +22693,19 @@
       </c>
       <c r="C857" t="inlineStr">
         <is>
-          <t>Criciuma</t>
+          <t>CRB</t>
         </is>
       </c>
       <c r="D857" t="inlineStr">
         <is>
-          <t>Avai</t>
+          <t>Cuiaba</t>
         </is>
       </c>
       <c r="E857" t="n">
-        <v>10.78</v>
+        <v>10.05</v>
       </c>
       <c r="F857" t="n">
-        <v>3.56</v>
+        <v>1.93</v>
       </c>
     </row>
     <row r="858">
@@ -22719,19 +22719,19 @@
       </c>
       <c r="C858" t="inlineStr">
         <is>
-          <t>Fortaleza</t>
+          <t>Criciuma</t>
         </is>
       </c>
       <c r="D858" t="inlineStr">
         <is>
-          <t>Athletic Club</t>
+          <t>Avai</t>
         </is>
       </c>
       <c r="E858" t="n">
-        <v>10.02</v>
+        <v>10.78</v>
       </c>
       <c r="F858" t="n">
-        <v>2.76</v>
+        <v>3.56</v>
       </c>
     </row>
     <row r="859">
@@ -22740,24 +22740,24 @@
       </c>
       <c r="B859" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="C859" t="inlineStr">
         <is>
-          <t>Eibar</t>
+          <t>Fortaleza</t>
         </is>
       </c>
       <c r="D859" t="inlineStr">
         <is>
-          <t>Las Palmas</t>
+          <t>Athletic Club</t>
         </is>
       </c>
       <c r="E859" t="n">
-        <v>9.15</v>
+        <v>10.02</v>
       </c>
       <c r="F859" t="n">
-        <v>0.92</v>
+        <v>2.76</v>
       </c>
     </row>
     <row r="860">
@@ -22771,71 +22771,201 @@
       </c>
       <c r="C860" t="inlineStr">
         <is>
-          <t>Real Valladolid</t>
+          <t>Burgos</t>
         </is>
       </c>
       <c r="D860" t="inlineStr">
         <is>
-          <t>Cordoba</t>
+          <t>Eldense</t>
         </is>
       </c>
       <c r="E860" t="n">
-        <v>9.380000000000001</v>
+        <v>9.31</v>
       </c>
       <c r="F860" t="n">
-        <v>0.38</v>
+        <v>0.92</v>
       </c>
     </row>
     <row r="861">
       <c r="A861" s="1" t="n">
-        <v>46293</v>
+        <v>46292</v>
       </c>
       <c r="B861" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="C861" t="inlineStr">
         <is>
-          <t>America Mineiro</t>
+          <t>Eibar</t>
         </is>
       </c>
       <c r="D861" t="inlineStr">
         <is>
-          <t>Juventude</t>
+          <t>Las Palmas</t>
         </is>
       </c>
       <c r="E861" t="n">
-        <v>10.28</v>
+        <v>9.15</v>
       </c>
       <c r="F861" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.92</v>
       </c>
     </row>
     <row r="862">
       <c r="A862" s="1" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B862" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C862" t="inlineStr">
+        <is>
+          <t>Mallorca</t>
+        </is>
+      </c>
+      <c r="D862" t="inlineStr">
+        <is>
+          <t>Almeria</t>
+        </is>
+      </c>
+      <c r="E862" t="n">
+        <v>9.380000000000001</v>
+      </c>
+      <c r="F862" t="n">
+        <v>0.99</v>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" s="1" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B863" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C863" t="inlineStr">
+        <is>
+          <t>Real Oviedo</t>
+        </is>
+      </c>
+      <c r="D863" t="inlineStr">
+        <is>
+          <t>Sporting Gijon</t>
+        </is>
+      </c>
+      <c r="E863" t="n">
+        <v>9</v>
+      </c>
+      <c r="F863" t="n">
+        <v>1.55</v>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" s="1" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B864" t="inlineStr">
+        <is>
+          <t>Spain - Segunda</t>
+        </is>
+      </c>
+      <c r="C864" t="inlineStr">
+        <is>
+          <t>Real Valladolid</t>
+        </is>
+      </c>
+      <c r="D864" t="inlineStr">
+        <is>
+          <t>Cordoba</t>
+        </is>
+      </c>
+      <c r="E864" t="n">
+        <v>9.380000000000001</v>
+      </c>
+      <c r="F864" t="n">
+        <v>0.38</v>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" s="1" t="n">
         <v>46293</v>
       </c>
-      <c r="B862" t="inlineStr">
+      <c r="B865" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C865" t="inlineStr">
+        <is>
+          <t>America Mineiro</t>
+        </is>
+      </c>
+      <c r="D865" t="inlineStr">
+        <is>
+          <t>Juventude</t>
+        </is>
+      </c>
+      <c r="E865" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="F865" t="n">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" s="1" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B866" t="inlineStr">
         <is>
           <t>Spain - Segunda</t>
         </is>
       </c>
-      <c r="C862" t="inlineStr">
+      <c r="C866" t="inlineStr">
         <is>
           <t>Leganes</t>
         </is>
       </c>
-      <c r="D862" t="inlineStr">
+      <c r="D866" t="inlineStr">
         <is>
           <t>Castellon</t>
         </is>
       </c>
-      <c r="E862" t="n">
+      <c r="E866" t="n">
         <v>9.27</v>
       </c>
-      <c r="F862" t="n">
+      <c r="F866" t="n">
         <v>-0.83</v>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" s="1" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B867" t="inlineStr">
+        <is>
+          <t>Brazil - Serie B</t>
+        </is>
+      </c>
+      <c r="C867" t="inlineStr">
+        <is>
+          <t>Botafogo SP</t>
+        </is>
+      </c>
+      <c r="D867" t="inlineStr">
+        <is>
+          <t>Ponte Preta</t>
+        </is>
+      </c>
+      <c r="E867" t="n">
+        <v>11.44</v>
+      </c>
+      <c r="F867" t="n">
+        <v>4.17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-09-27
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -22728,10 +22728,10 @@
         </is>
       </c>
       <c r="E858" t="n">
-        <v>10.78</v>
+        <v>11.05</v>
       </c>
       <c r="F858" t="n">
-        <v>3.56</v>
+        <v>3.33</v>
       </c>
     </row>
     <row r="859">
@@ -22754,10 +22754,10 @@
         </is>
       </c>
       <c r="E859" t="n">
-        <v>10.02</v>
+        <v>9.81</v>
       </c>
       <c r="F859" t="n">
-        <v>2.76</v>
+        <v>2.75</v>
       </c>
     </row>
     <row r="860">
@@ -22780,10 +22780,10 @@
         </is>
       </c>
       <c r="E860" t="n">
-        <v>9.31</v>
+        <v>9.16</v>
       </c>
       <c r="F860" t="n">
-        <v>0.92</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="861">
@@ -22832,7 +22832,7 @@
         </is>
       </c>
       <c r="E862" t="n">
-        <v>9.380000000000001</v>
+        <v>9.48</v>
       </c>
       <c r="F862" t="n">
         <v>0.99</v>
@@ -22861,7 +22861,7 @@
         <v>9</v>
       </c>
       <c r="F863" t="n">
-        <v>1.55</v>
+        <v>1.71</v>
       </c>
     </row>
     <row r="864">
@@ -22884,10 +22884,10 @@
         </is>
       </c>
       <c r="E864" t="n">
-        <v>9.380000000000001</v>
+        <v>9.33</v>
       </c>
       <c r="F864" t="n">
-        <v>0.38</v>
+        <v>0.31</v>
       </c>
     </row>
     <row r="865">
@@ -22913,7 +22913,7 @@
         <v>10.2</v>
       </c>
       <c r="F865" t="n">
-        <v>0.09</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="866">
@@ -22936,10 +22936,10 @@
         </is>
       </c>
       <c r="E866" t="n">
-        <v>9.27</v>
+        <v>9.31</v>
       </c>
       <c r="F866" t="n">
-        <v>-0.83</v>
+        <v>-0.84</v>
       </c>
     </row>
     <row r="867">
@@ -22962,10 +22962,10 @@
         </is>
       </c>
       <c r="E867" t="n">
-        <v>11.44</v>
+        <v>11.31</v>
       </c>
       <c r="F867" t="n">
-        <v>4.17</v>
+        <v>4.21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-10-06
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F867"/>
+  <dimension ref="A1:F873"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22968,6 +22968,162 @@
         <v>4.21</v>
       </c>
     </row>
+    <row r="868">
+      <c r="A868" s="1" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B868" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C868" t="inlineStr">
+        <is>
+          <t>Borussia Dortmund</t>
+        </is>
+      </c>
+      <c r="D868" t="inlineStr">
+        <is>
+          <t>Werder Bremen</t>
+        </is>
+      </c>
+      <c r="E868" t="n">
+        <v>9.69</v>
+      </c>
+      <c r="F868" t="n">
+        <v>2.9</v>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" s="1" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B869" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C869" t="inlineStr">
+        <is>
+          <t>Augsburg</t>
+        </is>
+      </c>
+      <c r="D869" t="inlineStr">
+        <is>
+          <t>Bayern Munich</t>
+        </is>
+      </c>
+      <c r="E869" t="n">
+        <v>10.71</v>
+      </c>
+      <c r="F869" t="n">
+        <v>-3.71</v>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" s="1" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B870" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C870" t="inlineStr">
+        <is>
+          <t>Hoffenheim</t>
+        </is>
+      </c>
+      <c r="D870" t="inlineStr">
+        <is>
+          <t>Hamburger SV</t>
+        </is>
+      </c>
+      <c r="E870" t="n">
+        <v>10.63</v>
+      </c>
+      <c r="F870" t="n">
+        <v>3.44</v>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" s="1" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B871" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C871" t="inlineStr">
+        <is>
+          <t>Mainz 05</t>
+        </is>
+      </c>
+      <c r="D871" t="inlineStr">
+        <is>
+          <t>Bayer Leverkusen</t>
+        </is>
+      </c>
+      <c r="E871" t="n">
+        <v>10.07</v>
+      </c>
+      <c r="F871" t="n">
+        <v>-0.09</v>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" s="1" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B872" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C872" t="inlineStr">
+        <is>
+          <t>RB Leipzig</t>
+        </is>
+      </c>
+      <c r="D872" t="inlineStr">
+        <is>
+          <t>Eintracht Frankfurt</t>
+        </is>
+      </c>
+      <c r="E872" t="n">
+        <v>10.32</v>
+      </c>
+      <c r="F872" t="n">
+        <v>1.86</v>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" s="1" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B873" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C873" t="inlineStr">
+        <is>
+          <t>FC Koln</t>
+        </is>
+      </c>
+      <c r="D873" t="inlineStr">
+        <is>
+          <t>Borussia Monchengladbach</t>
+        </is>
+      </c>
+      <c r="E873" t="n">
+        <v>10.29</v>
+      </c>
+      <c r="F873" t="n">
+        <v>1.05</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily scrape output - 2026-10-07
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -23014,10 +23014,10 @@
         </is>
       </c>
       <c r="E869" t="n">
-        <v>10.71</v>
+        <v>10.7</v>
       </c>
       <c r="F869" t="n">
-        <v>-3.71</v>
+        <v>-3.68</v>
       </c>
     </row>
     <row r="870">
@@ -23118,7 +23118,7 @@
         </is>
       </c>
       <c r="E873" t="n">
-        <v>10.29</v>
+        <v>10.22</v>
       </c>
       <c r="F873" t="n">
         <v>1.05</v>

</xml_diff>

<commit_message>
Daily scrape output - 2026-10-08
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F873"/>
+  <dimension ref="A1:F875"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22988,10 +22988,10 @@
         </is>
       </c>
       <c r="E868" t="n">
-        <v>9.69</v>
+        <v>9.74</v>
       </c>
       <c r="F868" t="n">
-        <v>2.9</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="869">
@@ -23014,10 +23014,10 @@
         </is>
       </c>
       <c r="E869" t="n">
-        <v>10.7</v>
+        <v>10.69</v>
       </c>
       <c r="F869" t="n">
-        <v>-3.68</v>
+        <v>-3.69</v>
       </c>
     </row>
     <row r="870">
@@ -23083,44 +23083,96 @@
       </c>
       <c r="C872" t="inlineStr">
         <is>
-          <t>RB Leipzig</t>
+          <t>Paderborn</t>
         </is>
       </c>
       <c r="D872" t="inlineStr">
         <is>
-          <t>Eintracht Frankfurt</t>
+          <t>Stuttgart</t>
         </is>
       </c>
       <c r="E872" t="n">
-        <v>10.32</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="F872" t="n">
-        <v>1.86</v>
+        <v>-1.21</v>
       </c>
     </row>
     <row r="873">
       <c r="A873" s="1" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B873" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C873" t="inlineStr">
+        <is>
+          <t>RB Leipzig</t>
+        </is>
+      </c>
+      <c r="D873" t="inlineStr">
+        <is>
+          <t>Eintracht Frankfurt</t>
+        </is>
+      </c>
+      <c r="E873" t="n">
+        <v>10.32</v>
+      </c>
+      <c r="F873" t="n">
+        <v>1.86</v>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" s="1" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B874" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C874" t="inlineStr">
+        <is>
+          <t>Union Berlin</t>
+        </is>
+      </c>
+      <c r="D874" t="inlineStr">
+        <is>
+          <t>Elversberg</t>
+        </is>
+      </c>
+      <c r="E874" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="F874" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" s="1" t="n">
         <v>46306</v>
       </c>
-      <c r="B873" t="inlineStr">
+      <c r="B875" t="inlineStr">
         <is>
           <t>Germany - Bundesliga</t>
         </is>
       </c>
-      <c r="C873" t="inlineStr">
+      <c r="C875" t="inlineStr">
         <is>
           <t>FC Koln</t>
         </is>
       </c>
-      <c r="D873" t="inlineStr">
+      <c r="D875" t="inlineStr">
         <is>
           <t>Borussia Monchengladbach</t>
         </is>
       </c>
-      <c r="E873" t="n">
+      <c r="E875" t="n">
         <v>10.22</v>
       </c>
-      <c r="F873" t="n">
+      <c r="F875" t="n">
         <v>1.05</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily scrape output - 2026-10-09
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F875"/>
+  <dimension ref="A1:F900"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22988,192 +22988,842 @@
         </is>
       </c>
       <c r="E868" t="n">
-        <v>9.74</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="F868" t="n">
-        <v>3.4</v>
+        <v>3.19</v>
       </c>
     </row>
     <row r="869">
       <c r="A869" s="1" t="n">
-        <v>46305</v>
+        <v>46304</v>
       </c>
       <c r="B869" t="inlineStr">
         <is>
-          <t>Germany - Bundesliga</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C869" t="inlineStr">
         <is>
-          <t>Augsburg</t>
+          <t>Podbeskidzie Bielsko-Biala</t>
         </is>
       </c>
       <c r="D869" t="inlineStr">
         <is>
-          <t>Bayern Munich</t>
+          <t>Pogon Siedlce</t>
         </is>
       </c>
       <c r="E869" t="n">
-        <v>10.69</v>
+        <v>10.51</v>
       </c>
       <c r="F869" t="n">
-        <v>-3.69</v>
+        <v>1.54</v>
       </c>
     </row>
     <row r="870">
       <c r="A870" s="1" t="n">
-        <v>46305</v>
+        <v>46304</v>
       </c>
       <c r="B870" t="inlineStr">
         <is>
-          <t>Germany - Bundesliga</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C870" t="inlineStr">
         <is>
-          <t>Hoffenheim</t>
+          <t>Rakow Czestochowa</t>
         </is>
       </c>
       <c r="D870" t="inlineStr">
         <is>
-          <t>Hamburger SV</t>
+          <t>GKS Katowice</t>
         </is>
       </c>
       <c r="E870" t="n">
-        <v>10.63</v>
+        <v>9.83</v>
       </c>
       <c r="F870" t="n">
-        <v>3.44</v>
+        <v>0.86</v>
       </c>
     </row>
     <row r="871">
       <c r="A871" s="1" t="n">
-        <v>46305</v>
+        <v>46304</v>
       </c>
       <c r="B871" t="inlineStr">
         <is>
-          <t>Germany - Bundesliga</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C871" t="inlineStr">
         <is>
-          <t>Mainz 05</t>
+          <t>Wieczysta Krakow</t>
         </is>
       </c>
       <c r="D871" t="inlineStr">
         <is>
-          <t>Bayer Leverkusen</t>
+          <t>Wisla Plock</t>
         </is>
       </c>
       <c r="E871" t="n">
-        <v>10.07</v>
+        <v>10.72</v>
       </c>
       <c r="F871" t="n">
-        <v>-0.09</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="872">
       <c r="A872" s="1" t="n">
-        <v>46305</v>
+        <v>46304</v>
       </c>
       <c r="B872" t="inlineStr">
         <is>
-          <t>Germany - Bundesliga</t>
+          <t>Portugal - Primeira Liga</t>
         </is>
       </c>
       <c r="C872" t="inlineStr">
         <is>
-          <t>Paderborn</t>
+          <t>Braga</t>
         </is>
       </c>
       <c r="D872" t="inlineStr">
         <is>
-          <t>Stuttgart</t>
+          <t>Sporting CP</t>
         </is>
       </c>
       <c r="E872" t="n">
-        <v>9.859999999999999</v>
+        <v>8.74</v>
       </c>
       <c r="F872" t="n">
-        <v>-1.21</v>
+        <v>-0.63</v>
       </c>
     </row>
     <row r="873">
       <c r="A873" s="1" t="n">
-        <v>46305</v>
+        <v>46304</v>
       </c>
       <c r="B873" t="inlineStr">
         <is>
-          <t>Germany - Bundesliga</t>
+          <t>Portugal - Primeira Liga</t>
         </is>
       </c>
       <c r="C873" t="inlineStr">
         <is>
-          <t>RB Leipzig</t>
+          <t>Moreirense</t>
         </is>
       </c>
       <c r="D873" t="inlineStr">
         <is>
-          <t>Eintracht Frankfurt</t>
+          <t>Gil Vicente</t>
         </is>
       </c>
       <c r="E873" t="n">
-        <v>10.32</v>
+        <v>8.75</v>
       </c>
       <c r="F873" t="n">
-        <v>1.86</v>
+        <v>-0.9</v>
       </c>
     </row>
     <row r="874">
       <c r="A874" s="1" t="n">
-        <v>46305</v>
+        <v>46304</v>
       </c>
       <c r="B874" t="inlineStr">
         <is>
-          <t>Germany - Bundesliga</t>
+          <t>Turkey - Super Lig</t>
         </is>
       </c>
       <c r="C874" t="inlineStr">
         <is>
-          <t>Union Berlin</t>
+          <t>Galatasaray</t>
         </is>
       </c>
       <c r="D874" t="inlineStr">
         <is>
-          <t>Elversberg</t>
+          <t>Kasimpasa</t>
         </is>
       </c>
       <c r="E874" t="n">
-        <v>9.5</v>
+        <v>10.16</v>
       </c>
       <c r="F874" t="n">
-        <v>0.7</v>
+        <v>3.73</v>
       </c>
     </row>
     <row r="875">
       <c r="A875" s="1" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B875" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C875" t="inlineStr">
+        <is>
+          <t>Augsburg</t>
+        </is>
+      </c>
+      <c r="D875" t="inlineStr">
+        <is>
+          <t>Bayern Munich</t>
+        </is>
+      </c>
+      <c r="E875" t="n">
+        <v>10.65</v>
+      </c>
+      <c r="F875" t="n">
+        <v>-3.68</v>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" s="1" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B876" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C876" t="inlineStr">
+        <is>
+          <t>Hoffenheim</t>
+        </is>
+      </c>
+      <c r="D876" t="inlineStr">
+        <is>
+          <t>Hamburger SV</t>
+        </is>
+      </c>
+      <c r="E876" t="n">
+        <v>10.63</v>
+      </c>
+      <c r="F876" t="n">
+        <v>3.46</v>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" s="1" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B877" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C877" t="inlineStr">
+        <is>
+          <t>Mainz 05</t>
+        </is>
+      </c>
+      <c r="D877" t="inlineStr">
+        <is>
+          <t>Bayer Leverkusen</t>
+        </is>
+      </c>
+      <c r="E877" t="n">
+        <v>10.07</v>
+      </c>
+      <c r="F877" t="n">
+        <v>-0.09</v>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" s="1" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B878" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C878" t="inlineStr">
+        <is>
+          <t>Paderborn</t>
+        </is>
+      </c>
+      <c r="D878" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="E878" t="n">
+        <v>9.859999999999999</v>
+      </c>
+      <c r="F878" t="n">
+        <v>-1.21</v>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" s="1" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B879" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C879" t="inlineStr">
+        <is>
+          <t>RB Leipzig</t>
+        </is>
+      </c>
+      <c r="D879" t="inlineStr">
+        <is>
+          <t>Eintracht Frankfurt</t>
+        </is>
+      </c>
+      <c r="E879" t="n">
+        <v>10.32</v>
+      </c>
+      <c r="F879" t="n">
+        <v>1.86</v>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" s="1" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B880" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C880" t="inlineStr">
+        <is>
+          <t>Union Berlin</t>
+        </is>
+      </c>
+      <c r="D880" t="inlineStr">
+        <is>
+          <t>Elversberg</t>
+        </is>
+      </c>
+      <c r="E880" t="n">
+        <v>9.539999999999999</v>
+      </c>
+      <c r="F880" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" s="1" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B881" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C881" t="inlineStr">
+        <is>
+          <t>Chrobry Glogow</t>
+        </is>
+      </c>
+      <c r="D881" t="inlineStr">
+        <is>
+          <t>Pogon Grodzisk Mazowiecki</t>
+        </is>
+      </c>
+      <c r="E881" t="n">
+        <v>10.66</v>
+      </c>
+      <c r="F881" t="n">
+        <v>0.61</v>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" s="1" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B882" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C882" t="inlineStr">
+        <is>
+          <t>Cracovia Krakow</t>
+        </is>
+      </c>
+      <c r="D882" t="inlineStr">
+        <is>
+          <t>Zaglebie Lubin</t>
+        </is>
+      </c>
+      <c r="E882" t="n">
+        <v>10.63</v>
+      </c>
+      <c r="F882" t="n">
+        <v>1.83</v>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" s="1" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B883" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C883" t="inlineStr">
+        <is>
+          <t>Jagiellonia Bialystok</t>
+        </is>
+      </c>
+      <c r="D883" t="inlineStr">
+        <is>
+          <t>Gornik Zabrze</t>
+        </is>
+      </c>
+      <c r="E883" t="n">
+        <v>9.640000000000001</v>
+      </c>
+      <c r="F883" t="n">
+        <v>-0.34</v>
+      </c>
+    </row>
+    <row r="884">
+      <c r="A884" s="1" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B884" t="inlineStr">
+        <is>
+          <t>Portugal - Primeira Liga</t>
+        </is>
+      </c>
+      <c r="C884" t="inlineStr">
+        <is>
+          <t>Casa Pia</t>
+        </is>
+      </c>
+      <c r="D884" t="inlineStr">
+        <is>
+          <t>Santa Clara</t>
+        </is>
+      </c>
+      <c r="E884" t="n">
+        <v>9.359999999999999</v>
+      </c>
+      <c r="F884" t="n">
+        <v>-0.35</v>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" s="1" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B885" t="inlineStr">
+        <is>
+          <t>Turkey - Super Lig</t>
+        </is>
+      </c>
+      <c r="C885" t="inlineStr">
+        <is>
+          <t>Samsunspor</t>
+        </is>
+      </c>
+      <c r="D885" t="inlineStr">
+        <is>
+          <t>Trabzonspor</t>
+        </is>
+      </c>
+      <c r="E885" t="n">
+        <v>9.460000000000001</v>
+      </c>
+      <c r="F885" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" s="1" t="n">
         <v>46306</v>
       </c>
-      <c r="B875" t="inlineStr">
+      <c r="B886" t="inlineStr">
         <is>
           <t>Germany - Bundesliga</t>
         </is>
       </c>
-      <c r="C875" t="inlineStr">
+      <c r="C886" t="inlineStr">
         <is>
           <t>FC Koln</t>
         </is>
       </c>
-      <c r="D875" t="inlineStr">
+      <c r="D886" t="inlineStr">
         <is>
           <t>Borussia Monchengladbach</t>
         </is>
       </c>
-      <c r="E875" t="n">
+      <c r="E886" t="n">
         <v>10.22</v>
       </c>
-      <c r="F875" t="n">
+      <c r="F886" t="n">
         <v>1.05</v>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" s="1" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B887" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C887" t="inlineStr">
+        <is>
+          <t>Freiburg</t>
+        </is>
+      </c>
+      <c r="D887" t="inlineStr">
+        <is>
+          <t>Schalke 04</t>
+        </is>
+      </c>
+      <c r="E887" t="n">
+        <v>9.109999999999999</v>
+      </c>
+      <c r="F887" t="n">
+        <v>1.95</v>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" s="1" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B888" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C888" t="inlineStr">
+        <is>
+          <t>LKS Lodz</t>
+        </is>
+      </c>
+      <c r="D888" t="inlineStr">
+        <is>
+          <t>Ruch Chorzow</t>
+        </is>
+      </c>
+      <c r="E888" t="n">
+        <v>10.68</v>
+      </c>
+      <c r="F888" t="n">
+        <v>1.11</v>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" s="1" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B889" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C889" t="inlineStr">
+        <is>
+          <t>Odra Opole</t>
+        </is>
+      </c>
+      <c r="D889" t="inlineStr">
+        <is>
+          <t>Miedz Legnica</t>
+        </is>
+      </c>
+      <c r="E889" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="F889" t="n">
+        <v>0.48</v>
+      </c>
+    </row>
+    <row r="890">
+      <c r="A890" s="1" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B890" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C890" t="inlineStr">
+        <is>
+          <t>Puszcza Niepolomice</t>
+        </is>
+      </c>
+      <c r="D890" t="inlineStr">
+        <is>
+          <t>Polonia Bytom</t>
+        </is>
+      </c>
+      <c r="E890" t="n">
+        <v>9.82</v>
+      </c>
+      <c r="F890" t="n">
+        <v>-0.54</v>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" s="1" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B891" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C891" t="inlineStr">
+        <is>
+          <t>Piast Gliwice</t>
+        </is>
+      </c>
+      <c r="D891" t="inlineStr">
+        <is>
+          <t>Widzew Lodz</t>
+        </is>
+      </c>
+      <c r="E891" t="n">
+        <v>10.08</v>
+      </c>
+      <c r="F891" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" s="1" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B892" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C892" t="inlineStr">
+        <is>
+          <t>Pogon Szczecin</t>
+        </is>
+      </c>
+      <c r="D892" t="inlineStr">
+        <is>
+          <t>Korona Kielce</t>
+        </is>
+      </c>
+      <c r="E892" t="n">
+        <v>9.65</v>
+      </c>
+      <c r="F892" t="n">
+        <v>0.96</v>
+      </c>
+    </row>
+    <row r="893">
+      <c r="A893" s="1" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B893" t="inlineStr">
+        <is>
+          <t>Portugal - Primeira Liga</t>
+        </is>
+      </c>
+      <c r="C893" t="inlineStr">
+        <is>
+          <t>Arouca</t>
+        </is>
+      </c>
+      <c r="D893" t="inlineStr">
+        <is>
+          <t>Estrela da Amadora</t>
+        </is>
+      </c>
+      <c r="E893" t="n">
+        <v>9.27</v>
+      </c>
+      <c r="F893" t="n">
+        <v>0.96</v>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" s="1" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B894" t="inlineStr">
+        <is>
+          <t>Portugal - Primeira Liga</t>
+        </is>
+      </c>
+      <c r="C894" t="inlineStr">
+        <is>
+          <t>Benfica</t>
+        </is>
+      </c>
+      <c r="D894" t="inlineStr">
+        <is>
+          <t>Vitoria Guimaraes</t>
+        </is>
+      </c>
+      <c r="E894" t="n">
+        <v>9.84</v>
+      </c>
+      <c r="F894" t="n">
+        <v>3.92</v>
+      </c>
+    </row>
+    <row r="895">
+      <c r="A895" s="1" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B895" t="inlineStr">
+        <is>
+          <t>Portugal - Primeira Liga</t>
+        </is>
+      </c>
+      <c r="C895" t="inlineStr">
+        <is>
+          <t>Rio Ave</t>
+        </is>
+      </c>
+      <c r="D895" t="inlineStr">
+        <is>
+          <t>Nacional da Madeira</t>
+        </is>
+      </c>
+      <c r="E895" t="n">
+        <v>9.710000000000001</v>
+      </c>
+      <c r="F895" t="n">
+        <v>0.49</v>
+      </c>
+    </row>
+    <row r="896">
+      <c r="A896" s="1" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B896" t="inlineStr">
+        <is>
+          <t>Turkey - Super Lig</t>
+        </is>
+      </c>
+      <c r="C896" t="inlineStr">
+        <is>
+          <t>Besiktas</t>
+        </is>
+      </c>
+      <c r="D896" t="inlineStr">
+        <is>
+          <t>Kocaelispor</t>
+        </is>
+      </c>
+      <c r="E896" t="n">
+        <v>9.779999999999999</v>
+      </c>
+      <c r="F896" t="n">
+        <v>3.75</v>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" s="1" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B897" t="inlineStr">
+        <is>
+          <t>Turkey - Super Lig</t>
+        </is>
+      </c>
+      <c r="C897" t="inlineStr">
+        <is>
+          <t>Konyaspor</t>
+        </is>
+      </c>
+      <c r="D897" t="inlineStr">
+        <is>
+          <t>Istanbul Basaksehir</t>
+        </is>
+      </c>
+      <c r="E897" t="n">
+        <v>9.279999999999999</v>
+      </c>
+      <c r="F897" t="n">
+        <v>-0.13</v>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" s="1" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B898" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C898" t="inlineStr">
+        <is>
+          <t>Radomiak Radom</t>
+        </is>
+      </c>
+      <c r="D898" t="inlineStr">
+        <is>
+          <t>Motor Lublin</t>
+        </is>
+      </c>
+      <c r="E898" t="n">
+        <v>9.16</v>
+      </c>
+      <c r="F898" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" s="1" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B899" t="inlineStr">
+        <is>
+          <t>Portugal - Primeira Liga</t>
+        </is>
+      </c>
+      <c r="C899" t="inlineStr">
+        <is>
+          <t>Famalicao</t>
+        </is>
+      </c>
+      <c r="D899" t="inlineStr">
+        <is>
+          <t>Alverca</t>
+        </is>
+      </c>
+      <c r="E899" t="n">
+        <v>9.640000000000001</v>
+      </c>
+      <c r="F899" t="n">
+        <v>1.96</v>
+      </c>
+    </row>
+    <row r="900">
+      <c r="A900" s="1" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B900" t="inlineStr">
+        <is>
+          <t>Turkey - Super Lig</t>
+        </is>
+      </c>
+      <c r="C900" t="inlineStr">
+        <is>
+          <t>Eyupspor</t>
+        </is>
+      </c>
+      <c r="D900" t="inlineStr">
+        <is>
+          <t>Goztepe</t>
+        </is>
+      </c>
+      <c r="E900" t="n">
+        <v>9.539999999999999</v>
+      </c>
+      <c r="F900" t="n">
+        <v>-0.61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-10-10
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F900"/>
+  <dimension ref="A1:F907"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23170,10 +23170,10 @@
         </is>
       </c>
       <c r="E875" t="n">
-        <v>10.65</v>
+        <v>10.59</v>
       </c>
       <c r="F875" t="n">
-        <v>-3.68</v>
+        <v>-3.72</v>
       </c>
     </row>
     <row r="876">
@@ -23196,7 +23196,7 @@
         </is>
       </c>
       <c r="E876" t="n">
-        <v>10.63</v>
+        <v>10.75</v>
       </c>
       <c r="F876" t="n">
         <v>3.46</v>
@@ -23222,10 +23222,10 @@
         </is>
       </c>
       <c r="E877" t="n">
-        <v>10.07</v>
+        <v>10</v>
       </c>
       <c r="F877" t="n">
-        <v>-0.09</v>
+        <v>-0.08</v>
       </c>
     </row>
     <row r="878">
@@ -23248,10 +23248,10 @@
         </is>
       </c>
       <c r="E878" t="n">
-        <v>9.859999999999999</v>
+        <v>9.869999999999999</v>
       </c>
       <c r="F878" t="n">
-        <v>-1.21</v>
+        <v>-1.32</v>
       </c>
     </row>
     <row r="879">
@@ -23274,10 +23274,10 @@
         </is>
       </c>
       <c r="E879" t="n">
-        <v>10.32</v>
+        <v>10.33</v>
       </c>
       <c r="F879" t="n">
-        <v>1.86</v>
+        <v>2.11</v>
       </c>
     </row>
     <row r="880">
@@ -23300,10 +23300,10 @@
         </is>
       </c>
       <c r="E880" t="n">
-        <v>9.539999999999999</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="F880" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.67</v>
       </c>
     </row>
     <row r="881">
@@ -23317,19 +23317,19 @@
       </c>
       <c r="C881" t="inlineStr">
         <is>
-          <t>Chrobry Glogow</t>
+          <t>Arka Gdynia</t>
         </is>
       </c>
       <c r="D881" t="inlineStr">
         <is>
-          <t>Pogon Grodzisk Mazowiecki</t>
+          <t>Polonia Warsaw</t>
         </is>
       </c>
       <c r="E881" t="n">
-        <v>10.66</v>
+        <v>10.6</v>
       </c>
       <c r="F881" t="n">
-        <v>0.61</v>
+        <v>-0.02</v>
       </c>
     </row>
     <row r="882">
@@ -23338,24 +23338,24 @@
       </c>
       <c r="B882" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C882" t="inlineStr">
         <is>
-          <t>Cracovia Krakow</t>
+          <t>Chrobry Glogow</t>
         </is>
       </c>
       <c r="D882" t="inlineStr">
         <is>
-          <t>Zaglebie Lubin</t>
+          <t>Pogon Grodzisk Mazowiecki</t>
         </is>
       </c>
       <c r="E882" t="n">
-        <v>10.63</v>
+        <v>10.59</v>
       </c>
       <c r="F882" t="n">
-        <v>1.83</v>
+        <v>0.62</v>
       </c>
     </row>
     <row r="883">
@@ -23364,24 +23364,24 @@
       </c>
       <c r="B883" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C883" t="inlineStr">
         <is>
-          <t>Jagiellonia Bialystok</t>
+          <t>Unia Skierniewice</t>
         </is>
       </c>
       <c r="D883" t="inlineStr">
         <is>
-          <t>Gornik Zabrze</t>
+          <t>Nieciecza</t>
         </is>
       </c>
       <c r="E883" t="n">
-        <v>9.640000000000001</v>
+        <v>10.45</v>
       </c>
       <c r="F883" t="n">
-        <v>-0.34</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="884">
@@ -23390,24 +23390,24 @@
       </c>
       <c r="B884" t="inlineStr">
         <is>
-          <t>Portugal - Primeira Liga</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C884" t="inlineStr">
         <is>
-          <t>Casa Pia</t>
+          <t>Cracovia Krakow</t>
         </is>
       </c>
       <c r="D884" t="inlineStr">
         <is>
-          <t>Santa Clara</t>
+          <t>Zaglebie Lubin</t>
         </is>
       </c>
       <c r="E884" t="n">
-        <v>9.359999999999999</v>
+        <v>10.43</v>
       </c>
       <c r="F884" t="n">
-        <v>-0.35</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="885">
@@ -23416,206 +23416,206 @@
       </c>
       <c r="B885" t="inlineStr">
         <is>
-          <t>Turkey - Super Lig</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C885" t="inlineStr">
         <is>
-          <t>Samsunspor</t>
+          <t>Jagiellonia Bialystok</t>
         </is>
       </c>
       <c r="D885" t="inlineStr">
         <is>
-          <t>Trabzonspor</t>
+          <t>Gornik Zabrze</t>
         </is>
       </c>
       <c r="E885" t="n">
-        <v>9.460000000000001</v>
+        <v>9.5</v>
       </c>
       <c r="F885" t="n">
-        <v>0.07000000000000001</v>
+        <v>-0.03</v>
       </c>
     </row>
     <row r="886">
       <c r="A886" s="1" t="n">
-        <v>46306</v>
+        <v>46305</v>
       </c>
       <c r="B886" t="inlineStr">
         <is>
-          <t>Germany - Bundesliga</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C886" t="inlineStr">
         <is>
-          <t>FC Koln</t>
+          <t>Slask Wroclaw</t>
         </is>
       </c>
       <c r="D886" t="inlineStr">
         <is>
-          <t>Borussia Monchengladbach</t>
+          <t>Lech Poznan</t>
         </is>
       </c>
       <c r="E886" t="n">
-        <v>10.22</v>
+        <v>9.74</v>
       </c>
       <c r="F886" t="n">
-        <v>1.05</v>
+        <v>-1.91</v>
       </c>
     </row>
     <row r="887">
       <c r="A887" s="1" t="n">
-        <v>46306</v>
+        <v>46305</v>
       </c>
       <c r="B887" t="inlineStr">
         <is>
-          <t>Germany - Bundesliga</t>
+          <t>Portugal - Primeira Liga</t>
         </is>
       </c>
       <c r="C887" t="inlineStr">
         <is>
-          <t>Freiburg</t>
+          <t>Academico de Viseu</t>
         </is>
       </c>
       <c r="D887" t="inlineStr">
         <is>
-          <t>Schalke 04</t>
+          <t>Estoril</t>
         </is>
       </c>
       <c r="E887" t="n">
-        <v>9.109999999999999</v>
+        <v>9.25</v>
       </c>
       <c r="F887" t="n">
-        <v>1.95</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="888">
       <c r="A888" s="1" t="n">
-        <v>46306</v>
+        <v>46305</v>
       </c>
       <c r="B888" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Portugal - Primeira Liga</t>
         </is>
       </c>
       <c r="C888" t="inlineStr">
         <is>
-          <t>LKS Lodz</t>
+          <t>Casa Pia</t>
         </is>
       </c>
       <c r="D888" t="inlineStr">
         <is>
-          <t>Ruch Chorzow</t>
+          <t>Santa Clara</t>
         </is>
       </c>
       <c r="E888" t="n">
-        <v>10.68</v>
+        <v>9.44</v>
       </c>
       <c r="F888" t="n">
-        <v>1.11</v>
+        <v>-0.64</v>
       </c>
     </row>
     <row r="889">
       <c r="A889" s="1" t="n">
-        <v>46306</v>
+        <v>46305</v>
       </c>
       <c r="B889" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Portugal - Primeira Liga</t>
         </is>
       </c>
       <c r="C889" t="inlineStr">
         <is>
-          <t>Odra Opole</t>
+          <t>Maritimo</t>
         </is>
       </c>
       <c r="D889" t="inlineStr">
         <is>
-          <t>Miedz Legnica</t>
+          <t>Porto</t>
         </is>
       </c>
       <c r="E889" t="n">
-        <v>10.3</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="F889" t="n">
-        <v>0.48</v>
+        <v>-2.97</v>
       </c>
     </row>
     <row r="890">
       <c r="A890" s="1" t="n">
-        <v>46306</v>
+        <v>46305</v>
       </c>
       <c r="B890" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Turkey - Super Lig</t>
         </is>
       </c>
       <c r="C890" t="inlineStr">
         <is>
-          <t>Puszcza Niepolomice</t>
+          <t>Alanyaspor</t>
         </is>
       </c>
       <c r="D890" t="inlineStr">
         <is>
-          <t>Polonia Bytom</t>
+          <t>Erzurumspor</t>
         </is>
       </c>
       <c r="E890" t="n">
-        <v>9.82</v>
+        <v>8.960000000000001</v>
       </c>
       <c r="F890" t="n">
-        <v>-0.54</v>
+        <v>1.89</v>
       </c>
     </row>
     <row r="891">
       <c r="A891" s="1" t="n">
-        <v>46306</v>
+        <v>46305</v>
       </c>
       <c r="B891" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Turkey - Super Lig</t>
         </is>
       </c>
       <c r="C891" t="inlineStr">
         <is>
-          <t>Piast Gliwice</t>
+          <t>Caykur Rizespor</t>
         </is>
       </c>
       <c r="D891" t="inlineStr">
         <is>
-          <t>Widzew Lodz</t>
+          <t>Fenerbahce</t>
         </is>
       </c>
       <c r="E891" t="n">
-        <v>10.08</v>
+        <v>10.16</v>
       </c>
       <c r="F891" t="n">
-        <v>0.18</v>
+        <v>-1.43</v>
       </c>
     </row>
     <row r="892">
       <c r="A892" s="1" t="n">
-        <v>46306</v>
+        <v>46305</v>
       </c>
       <c r="B892" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Turkey - Super Lig</t>
         </is>
       </c>
       <c r="C892" t="inlineStr">
         <is>
-          <t>Pogon Szczecin</t>
+          <t>Samsunspor</t>
         </is>
       </c>
       <c r="D892" t="inlineStr">
         <is>
-          <t>Korona Kielce</t>
+          <t>Trabzonspor</t>
         </is>
       </c>
       <c r="E892" t="n">
-        <v>9.65</v>
+        <v>9.48</v>
       </c>
       <c r="F892" t="n">
-        <v>0.96</v>
+        <v>-0.13</v>
       </c>
     </row>
     <row r="893">
@@ -23624,24 +23624,24 @@
       </c>
       <c r="B893" t="inlineStr">
         <is>
-          <t>Portugal - Primeira Liga</t>
+          <t>Germany - Bundesliga</t>
         </is>
       </c>
       <c r="C893" t="inlineStr">
         <is>
-          <t>Arouca</t>
+          <t>FC Koln</t>
         </is>
       </c>
       <c r="D893" t="inlineStr">
         <is>
-          <t>Estrela da Amadora</t>
+          <t>Borussia Monchengladbach</t>
         </is>
       </c>
       <c r="E893" t="n">
-        <v>9.27</v>
+        <v>10.22</v>
       </c>
       <c r="F893" t="n">
-        <v>0.96</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="894">
@@ -23650,24 +23650,24 @@
       </c>
       <c r="B894" t="inlineStr">
         <is>
-          <t>Portugal - Primeira Liga</t>
+          <t>Germany - Bundesliga</t>
         </is>
       </c>
       <c r="C894" t="inlineStr">
         <is>
-          <t>Benfica</t>
+          <t>Freiburg</t>
         </is>
       </c>
       <c r="D894" t="inlineStr">
         <is>
-          <t>Vitoria Guimaraes</t>
+          <t>Schalke 04</t>
         </is>
       </c>
       <c r="E894" t="n">
-        <v>9.84</v>
+        <v>9.109999999999999</v>
       </c>
       <c r="F894" t="n">
-        <v>3.92</v>
+        <v>2.09</v>
       </c>
     </row>
     <row r="895">
@@ -23676,24 +23676,24 @@
       </c>
       <c r="B895" t="inlineStr">
         <is>
-          <t>Portugal - Primeira Liga</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C895" t="inlineStr">
         <is>
-          <t>Rio Ave</t>
+          <t>LKS Lodz</t>
         </is>
       </c>
       <c r="D895" t="inlineStr">
         <is>
-          <t>Nacional da Madeira</t>
+          <t>Ruch Chorzow</t>
         </is>
       </c>
       <c r="E895" t="n">
-        <v>9.710000000000001</v>
+        <v>10.68</v>
       </c>
       <c r="F895" t="n">
-        <v>0.49</v>
+        <v>1.11</v>
       </c>
     </row>
     <row r="896">
@@ -23702,24 +23702,24 @@
       </c>
       <c r="B896" t="inlineStr">
         <is>
-          <t>Turkey - Super Lig</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C896" t="inlineStr">
         <is>
-          <t>Besiktas</t>
+          <t>Odra Opole</t>
         </is>
       </c>
       <c r="D896" t="inlineStr">
         <is>
-          <t>Kocaelispor</t>
+          <t>Miedz Legnica</t>
         </is>
       </c>
       <c r="E896" t="n">
-        <v>9.779999999999999</v>
+        <v>10.3</v>
       </c>
       <c r="F896" t="n">
-        <v>3.75</v>
+        <v>0.48</v>
       </c>
     </row>
     <row r="897">
@@ -23728,29 +23728,29 @@
       </c>
       <c r="B897" t="inlineStr">
         <is>
-          <t>Turkey - Super Lig</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C897" t="inlineStr">
         <is>
-          <t>Konyaspor</t>
+          <t>Puszcza Niepolomice</t>
         </is>
       </c>
       <c r="D897" t="inlineStr">
         <is>
-          <t>Istanbul Basaksehir</t>
+          <t>Polonia Bytom</t>
         </is>
       </c>
       <c r="E897" t="n">
-        <v>9.279999999999999</v>
+        <v>9.82</v>
       </c>
       <c r="F897" t="n">
-        <v>-0.13</v>
+        <v>-0.54</v>
       </c>
     </row>
     <row r="898">
       <c r="A898" s="1" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="B898" t="inlineStr">
         <is>
@@ -23759,71 +23759,253 @@
       </c>
       <c r="C898" t="inlineStr">
         <is>
-          <t>Radomiak Radom</t>
+          <t>Piast Gliwice</t>
         </is>
       </c>
       <c r="D898" t="inlineStr">
         <is>
-          <t>Motor Lublin</t>
+          <t>Widzew Lodz</t>
         </is>
       </c>
       <c r="E898" t="n">
-        <v>9.16</v>
+        <v>10.16</v>
       </c>
       <c r="F898" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="899">
       <c r="A899" s="1" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="B899" t="inlineStr">
         <is>
-          <t>Portugal - Primeira Liga</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C899" t="inlineStr">
         <is>
-          <t>Famalicao</t>
+          <t>Pogon Szczecin</t>
         </is>
       </c>
       <c r="D899" t="inlineStr">
         <is>
-          <t>Alverca</t>
+          <t>Korona Kielce</t>
         </is>
       </c>
       <c r="E899" t="n">
-        <v>9.640000000000001</v>
+        <v>9.6</v>
       </c>
       <c r="F899" t="n">
-        <v>1.96</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="900">
       <c r="A900" s="1" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B900" t="inlineStr">
+        <is>
+          <t>Portugal - Primeira Liga</t>
+        </is>
+      </c>
+      <c r="C900" t="inlineStr">
+        <is>
+          <t>Arouca</t>
+        </is>
+      </c>
+      <c r="D900" t="inlineStr">
+        <is>
+          <t>Estrela da Amadora</t>
+        </is>
+      </c>
+      <c r="E900" t="n">
+        <v>9.27</v>
+      </c>
+      <c r="F900" t="n">
+        <v>0.96</v>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" s="1" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B901" t="inlineStr">
+        <is>
+          <t>Portugal - Primeira Liga</t>
+        </is>
+      </c>
+      <c r="C901" t="inlineStr">
+        <is>
+          <t>Benfica</t>
+        </is>
+      </c>
+      <c r="D901" t="inlineStr">
+        <is>
+          <t>Vitoria Guimaraes</t>
+        </is>
+      </c>
+      <c r="E901" t="n">
+        <v>9.84</v>
+      </c>
+      <c r="F901" t="n">
+        <v>3.92</v>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" s="1" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B902" t="inlineStr">
+        <is>
+          <t>Portugal - Primeira Liga</t>
+        </is>
+      </c>
+      <c r="C902" t="inlineStr">
+        <is>
+          <t>Rio Ave</t>
+        </is>
+      </c>
+      <c r="D902" t="inlineStr">
+        <is>
+          <t>Nacional da Madeira</t>
+        </is>
+      </c>
+      <c r="E902" t="n">
+        <v>9.710000000000001</v>
+      </c>
+      <c r="F902" t="n">
+        <v>0.49</v>
+      </c>
+    </row>
+    <row r="903">
+      <c r="A903" s="1" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B903" t="inlineStr">
+        <is>
+          <t>Turkey - Super Lig</t>
+        </is>
+      </c>
+      <c r="C903" t="inlineStr">
+        <is>
+          <t>Besiktas</t>
+        </is>
+      </c>
+      <c r="D903" t="inlineStr">
+        <is>
+          <t>Kocaelispor</t>
+        </is>
+      </c>
+      <c r="E903" t="n">
+        <v>9.949999999999999</v>
+      </c>
+      <c r="F903" t="n">
+        <v>3.77</v>
+      </c>
+    </row>
+    <row r="904">
+      <c r="A904" s="1" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B904" t="inlineStr">
+        <is>
+          <t>Turkey - Super Lig</t>
+        </is>
+      </c>
+      <c r="C904" t="inlineStr">
+        <is>
+          <t>Konyaspor</t>
+        </is>
+      </c>
+      <c r="D904" t="inlineStr">
+        <is>
+          <t>Istanbul Basaksehir</t>
+        </is>
+      </c>
+      <c r="E904" t="n">
+        <v>9.279999999999999</v>
+      </c>
+      <c r="F904" t="n">
+        <v>-0.13</v>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" s="1" t="n">
         <v>46307</v>
       </c>
-      <c r="B900" t="inlineStr">
+      <c r="B905" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C905" t="inlineStr">
+        <is>
+          <t>Radomiak Radom</t>
+        </is>
+      </c>
+      <c r="D905" t="inlineStr">
+        <is>
+          <t>Motor Lublin</t>
+        </is>
+      </c>
+      <c r="E905" t="n">
+        <v>9.24</v>
+      </c>
+      <c r="F905" t="n">
+        <v>0.93</v>
+      </c>
+    </row>
+    <row r="906">
+      <c r="A906" s="1" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B906" t="inlineStr">
+        <is>
+          <t>Portugal - Primeira Liga</t>
+        </is>
+      </c>
+      <c r="C906" t="inlineStr">
+        <is>
+          <t>Famalicao</t>
+        </is>
+      </c>
+      <c r="D906" t="inlineStr">
+        <is>
+          <t>Alverca</t>
+        </is>
+      </c>
+      <c r="E906" t="n">
+        <v>9.640000000000001</v>
+      </c>
+      <c r="F906" t="n">
+        <v>1.46</v>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" s="1" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B907" t="inlineStr">
         <is>
           <t>Turkey - Super Lig</t>
         </is>
       </c>
-      <c r="C900" t="inlineStr">
+      <c r="C907" t="inlineStr">
         <is>
           <t>Eyupspor</t>
         </is>
       </c>
-      <c r="D900" t="inlineStr">
+      <c r="D907" t="inlineStr">
         <is>
           <t>Goztepe</t>
         </is>
       </c>
-      <c r="E900" t="n">
-        <v>9.539999999999999</v>
-      </c>
-      <c r="F900" t="n">
-        <v>-0.61</v>
+      <c r="E907" t="n">
+        <v>9.289999999999999</v>
+      </c>
+      <c r="F907" t="n">
+        <v>-0.57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-10-11
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F907"/>
+  <dimension ref="A1:F909"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23638,10 +23638,10 @@
         </is>
       </c>
       <c r="E893" t="n">
-        <v>10.22</v>
+        <v>10.24</v>
       </c>
       <c r="F893" t="n">
-        <v>1.05</v>
+        <v>1.41</v>
       </c>
     </row>
     <row r="894">
@@ -23664,7 +23664,7 @@
         </is>
       </c>
       <c r="E894" t="n">
-        <v>9.109999999999999</v>
+        <v>9.18</v>
       </c>
       <c r="F894" t="n">
         <v>2.09</v>
@@ -23690,10 +23690,10 @@
         </is>
       </c>
       <c r="E895" t="n">
-        <v>10.68</v>
+        <v>10.49</v>
       </c>
       <c r="F895" t="n">
-        <v>1.11</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="896">
@@ -23716,10 +23716,10 @@
         </is>
       </c>
       <c r="E896" t="n">
-        <v>10.3</v>
+        <v>10.28</v>
       </c>
       <c r="F896" t="n">
-        <v>0.48</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="897">
@@ -23759,19 +23759,19 @@
       </c>
       <c r="C898" t="inlineStr">
         <is>
-          <t>Piast Gliwice</t>
+          <t>Legia Warsaw</t>
         </is>
       </c>
       <c r="D898" t="inlineStr">
         <is>
-          <t>Widzew Lodz</t>
+          <t>Wisla Krakow</t>
         </is>
       </c>
       <c r="E898" t="n">
-        <v>10.16</v>
+        <v>9.65</v>
       </c>
       <c r="F898" t="n">
-        <v>0.18</v>
+        <v>1.53</v>
       </c>
     </row>
     <row r="899">
@@ -23785,19 +23785,19 @@
       </c>
       <c r="C899" t="inlineStr">
         <is>
-          <t>Pogon Szczecin</t>
+          <t>Piast Gliwice</t>
         </is>
       </c>
       <c r="D899" t="inlineStr">
         <is>
-          <t>Korona Kielce</t>
+          <t>Widzew Lodz</t>
         </is>
       </c>
       <c r="E899" t="n">
-        <v>9.6</v>
+        <v>10.28</v>
       </c>
       <c r="F899" t="n">
-        <v>0.97</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="900">
@@ -23806,24 +23806,24 @@
       </c>
       <c r="B900" t="inlineStr">
         <is>
-          <t>Portugal - Primeira Liga</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C900" t="inlineStr">
         <is>
-          <t>Arouca</t>
+          <t>Pogon Szczecin</t>
         </is>
       </c>
       <c r="D900" t="inlineStr">
         <is>
-          <t>Estrela da Amadora</t>
+          <t>Korona Kielce</t>
         </is>
       </c>
       <c r="E900" t="n">
-        <v>9.27</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="F900" t="n">
-        <v>0.96</v>
+        <v>0.8100000000000001</v>
       </c>
     </row>
     <row r="901">
@@ -23837,19 +23837,19 @@
       </c>
       <c r="C901" t="inlineStr">
         <is>
-          <t>Benfica</t>
+          <t>Arouca</t>
         </is>
       </c>
       <c r="D901" t="inlineStr">
         <is>
-          <t>Vitoria Guimaraes</t>
+          <t>Estrela da Amadora</t>
         </is>
       </c>
       <c r="E901" t="n">
-        <v>9.84</v>
+        <v>9.27</v>
       </c>
       <c r="F901" t="n">
-        <v>3.92</v>
+        <v>0.96</v>
       </c>
     </row>
     <row r="902">
@@ -23863,19 +23863,19 @@
       </c>
       <c r="C902" t="inlineStr">
         <is>
-          <t>Rio Ave</t>
+          <t>Benfica</t>
         </is>
       </c>
       <c r="D902" t="inlineStr">
         <is>
-          <t>Nacional da Madeira</t>
+          <t>Vitoria Guimaraes</t>
         </is>
       </c>
       <c r="E902" t="n">
-        <v>9.710000000000001</v>
+        <v>9.83</v>
       </c>
       <c r="F902" t="n">
-        <v>0.49</v>
+        <v>3.62</v>
       </c>
     </row>
     <row r="903">
@@ -23884,24 +23884,24 @@
       </c>
       <c r="B903" t="inlineStr">
         <is>
-          <t>Turkey - Super Lig</t>
+          <t>Portugal - Primeira Liga</t>
         </is>
       </c>
       <c r="C903" t="inlineStr">
         <is>
-          <t>Besiktas</t>
+          <t>Rio Ave</t>
         </is>
       </c>
       <c r="D903" t="inlineStr">
         <is>
-          <t>Kocaelispor</t>
+          <t>Nacional da Madeira</t>
         </is>
       </c>
       <c r="E903" t="n">
-        <v>9.949999999999999</v>
+        <v>9.869999999999999</v>
       </c>
       <c r="F903" t="n">
-        <v>3.77</v>
+        <v>0.48</v>
       </c>
     </row>
     <row r="904">
@@ -23915,71 +23915,71 @@
       </c>
       <c r="C904" t="inlineStr">
         <is>
-          <t>Konyaspor</t>
+          <t>Besiktas</t>
         </is>
       </c>
       <c r="D904" t="inlineStr">
         <is>
-          <t>Istanbul Basaksehir</t>
+          <t>Kocaelispor</t>
         </is>
       </c>
       <c r="E904" t="n">
-        <v>9.279999999999999</v>
+        <v>9.99</v>
       </c>
       <c r="F904" t="n">
-        <v>-0.13</v>
+        <v>3.99</v>
       </c>
     </row>
     <row r="905">
       <c r="A905" s="1" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="B905" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Turkey - Super Lig</t>
         </is>
       </c>
       <c r="C905" t="inlineStr">
         <is>
-          <t>Radomiak Radom</t>
+          <t>Gaziantep</t>
         </is>
       </c>
       <c r="D905" t="inlineStr">
         <is>
-          <t>Motor Lublin</t>
+          <t>Corum Belediyespor</t>
         </is>
       </c>
       <c r="E905" t="n">
-        <v>9.24</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="F905" t="n">
-        <v>0.93</v>
+        <v>0.49</v>
       </c>
     </row>
     <row r="906">
       <c r="A906" s="1" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="B906" t="inlineStr">
         <is>
-          <t>Portugal - Primeira Liga</t>
+          <t>Turkey - Super Lig</t>
         </is>
       </c>
       <c r="C906" t="inlineStr">
         <is>
-          <t>Famalicao</t>
+          <t>Konyaspor</t>
         </is>
       </c>
       <c r="D906" t="inlineStr">
         <is>
-          <t>Alverca</t>
+          <t>Istanbul Basaksehir</t>
         </is>
       </c>
       <c r="E906" t="n">
-        <v>9.640000000000001</v>
+        <v>9.279999999999999</v>
       </c>
       <c r="F906" t="n">
-        <v>1.46</v>
+        <v>-0.13</v>
       </c>
     </row>
     <row r="907">
@@ -23988,24 +23988,76 @@
       </c>
       <c r="B907" t="inlineStr">
         <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C907" t="inlineStr">
+        <is>
+          <t>Radomiak Radom</t>
+        </is>
+      </c>
+      <c r="D907" t="inlineStr">
+        <is>
+          <t>Motor Lublin</t>
+        </is>
+      </c>
+      <c r="E907" t="n">
+        <v>9.24</v>
+      </c>
+      <c r="F907" t="n">
+        <v>0.93</v>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" s="1" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B908" t="inlineStr">
+        <is>
+          <t>Portugal - Primeira Liga</t>
+        </is>
+      </c>
+      <c r="C908" t="inlineStr">
+        <is>
+          <t>Famalicao</t>
+        </is>
+      </c>
+      <c r="D908" t="inlineStr">
+        <is>
+          <t>Alverca</t>
+        </is>
+      </c>
+      <c r="E908" t="n">
+        <v>9.640000000000001</v>
+      </c>
+      <c r="F908" t="n">
+        <v>1.46</v>
+      </c>
+    </row>
+    <row r="909">
+      <c r="A909" s="1" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B909" t="inlineStr">
+        <is>
           <t>Turkey - Super Lig</t>
         </is>
       </c>
-      <c r="C907" t="inlineStr">
+      <c r="C909" t="inlineStr">
         <is>
           <t>Eyupspor</t>
         </is>
       </c>
-      <c r="D907" t="inlineStr">
+      <c r="D909" t="inlineStr">
         <is>
           <t>Goztepe</t>
         </is>
       </c>
-      <c r="E907" t="n">
-        <v>9.289999999999999</v>
-      </c>
-      <c r="F907" t="n">
-        <v>-0.57</v>
+      <c r="E909" t="n">
+        <v>9.130000000000001</v>
+      </c>
+      <c r="F909" t="n">
+        <v>-0.88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-10-12
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F909"/>
+  <dimension ref="A1:F910"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23993,19 +23993,19 @@
       </c>
       <c r="C907" t="inlineStr">
         <is>
-          <t>Radomiak Radom</t>
+          <t>GKS Katowice</t>
         </is>
       </c>
       <c r="D907" t="inlineStr">
         <is>
-          <t>Motor Lublin</t>
+          <t>Wieczysta Krakow</t>
         </is>
       </c>
       <c r="E907" t="n">
-        <v>9.24</v>
+        <v>10.36</v>
       </c>
       <c r="F907" t="n">
-        <v>0.93</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="908">
@@ -24014,24 +24014,24 @@
       </c>
       <c r="B908" t="inlineStr">
         <is>
-          <t>Portugal - Primeira Liga</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C908" t="inlineStr">
         <is>
-          <t>Famalicao</t>
+          <t>Radomiak Radom</t>
         </is>
       </c>
       <c r="D908" t="inlineStr">
         <is>
-          <t>Alverca</t>
+          <t>Motor Lublin</t>
         </is>
       </c>
       <c r="E908" t="n">
-        <v>9.640000000000001</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="F908" t="n">
-        <v>1.46</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="909">
@@ -24040,24 +24040,50 @@
       </c>
       <c r="B909" t="inlineStr">
         <is>
+          <t>Portugal - Primeira Liga</t>
+        </is>
+      </c>
+      <c r="C909" t="inlineStr">
+        <is>
+          <t>Famalicao</t>
+        </is>
+      </c>
+      <c r="D909" t="inlineStr">
+        <is>
+          <t>Alverca</t>
+        </is>
+      </c>
+      <c r="E909" t="n">
+        <v>9.640000000000001</v>
+      </c>
+      <c r="F909" t="n">
+        <v>1.46</v>
+      </c>
+    </row>
+    <row r="910">
+      <c r="A910" s="1" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B910" t="inlineStr">
+        <is>
           <t>Turkey - Super Lig</t>
         </is>
       </c>
-      <c r="C909" t="inlineStr">
+      <c r="C910" t="inlineStr">
         <is>
           <t>Eyupspor</t>
         </is>
       </c>
-      <c r="D909" t="inlineStr">
+      <c r="D910" t="inlineStr">
         <is>
           <t>Goztepe</t>
         </is>
       </c>
-      <c r="E909" t="n">
-        <v>9.130000000000001</v>
-      </c>
-      <c r="F909" t="n">
-        <v>-0.88</v>
+      <c r="E910" t="n">
+        <v>9.24</v>
+      </c>
+      <c r="F910" t="n">
+        <v>-0.89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-10-13
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F910"/>
+  <dimension ref="A1:F916"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24086,6 +24086,162 @@
         <v>-0.89</v>
       </c>
     </row>
+    <row r="911">
+      <c r="A911" s="1" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B911" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C911" t="inlineStr">
+        <is>
+          <t>Eintracht Frankfurt</t>
+        </is>
+      </c>
+      <c r="D911" t="inlineStr">
+        <is>
+          <t>FC Koln</t>
+        </is>
+      </c>
+      <c r="E911" t="n">
+        <v>10.49</v>
+      </c>
+      <c r="F911" t="n">
+        <v>1.33</v>
+      </c>
+    </row>
+    <row r="912">
+      <c r="A912" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B912" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C912" t="inlineStr">
+        <is>
+          <t>Bayern Munich</t>
+        </is>
+      </c>
+      <c r="D912" t="inlineStr">
+        <is>
+          <t>RB Leipzig</t>
+        </is>
+      </c>
+      <c r="E912" t="n">
+        <v>10.77</v>
+      </c>
+      <c r="F912" t="n">
+        <v>4.63</v>
+      </c>
+    </row>
+    <row r="913">
+      <c r="A913" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B913" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C913" t="inlineStr">
+        <is>
+          <t>Hamburger SV</t>
+        </is>
+      </c>
+      <c r="D913" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="E913" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="F913" t="n">
+        <v>-1.84</v>
+      </c>
+    </row>
+    <row r="914">
+      <c r="A914" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B914" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C914" t="inlineStr">
+        <is>
+          <t>Union Berlin</t>
+        </is>
+      </c>
+      <c r="D914" t="inlineStr">
+        <is>
+          <t>Borussia Dortmund</t>
+        </is>
+      </c>
+      <c r="E914" t="n">
+        <v>9.77</v>
+      </c>
+      <c r="F914" t="n">
+        <v>-1.43</v>
+      </c>
+    </row>
+    <row r="915">
+      <c r="A915" s="1" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B915" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C915" t="inlineStr">
+        <is>
+          <t>Bayer Leverkusen</t>
+        </is>
+      </c>
+      <c r="D915" t="inlineStr">
+        <is>
+          <t>Freiburg</t>
+        </is>
+      </c>
+      <c r="E915" t="n">
+        <v>9.789999999999999</v>
+      </c>
+      <c r="F915" t="n">
+        <v>2.65</v>
+      </c>
+    </row>
+    <row r="916">
+      <c r="A916" s="1" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B916" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C916" t="inlineStr">
+        <is>
+          <t>Borussia Monchengladbach</t>
+        </is>
+      </c>
+      <c r="D916" t="inlineStr">
+        <is>
+          <t>Hoffenheim</t>
+        </is>
+      </c>
+      <c r="E916" t="n">
+        <v>10.47</v>
+      </c>
+      <c r="F916" t="n">
+        <v>-0.57</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily scrape output - 2026-10-14
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -24184,10 +24184,10 @@
         </is>
       </c>
       <c r="E914" t="n">
-        <v>9.77</v>
+        <v>9.779999999999999</v>
       </c>
       <c r="F914" t="n">
-        <v>-1.43</v>
+        <v>-1.49</v>
       </c>
     </row>
     <row r="915">
@@ -24236,10 +24236,10 @@
         </is>
       </c>
       <c r="E916" t="n">
-        <v>10.47</v>
+        <v>10.26</v>
       </c>
       <c r="F916" t="n">
-        <v>-0.57</v>
+        <v>-0.53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-10-15
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F916"/>
+  <dimension ref="A1:F919"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24088,33 +24088,33 @@
     </row>
     <row r="911">
       <c r="A911" s="1" t="n">
-        <v>46311</v>
+        <v>46310</v>
       </c>
       <c r="B911" t="inlineStr">
         <is>
-          <t>Germany - Bundesliga</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C911" t="inlineStr">
         <is>
-          <t>Eintracht Frankfurt</t>
+          <t>Pogon Siedlce</t>
         </is>
       </c>
       <c r="D911" t="inlineStr">
         <is>
-          <t>FC Koln</t>
+          <t>Puszcza Niepolomice</t>
         </is>
       </c>
       <c r="E911" t="n">
-        <v>10.49</v>
+        <v>10.34</v>
       </c>
       <c r="F911" t="n">
-        <v>1.33</v>
+        <v>0.38</v>
       </c>
     </row>
     <row r="912">
       <c r="A912" s="1" t="n">
-        <v>46312</v>
+        <v>46311</v>
       </c>
       <c r="B912" t="inlineStr">
         <is>
@@ -24123,19 +24123,19 @@
       </c>
       <c r="C912" t="inlineStr">
         <is>
-          <t>Bayern Munich</t>
+          <t>Eintracht Frankfurt</t>
         </is>
       </c>
       <c r="D912" t="inlineStr">
         <is>
-          <t>RB Leipzig</t>
+          <t>FC Koln</t>
         </is>
       </c>
       <c r="E912" t="n">
-        <v>10.77</v>
+        <v>10.39</v>
       </c>
       <c r="F912" t="n">
-        <v>4.63</v>
+        <v>1.33</v>
       </c>
     </row>
     <row r="913">
@@ -24149,19 +24149,19 @@
       </c>
       <c r="C913" t="inlineStr">
         <is>
-          <t>Hamburger SV</t>
+          <t>Bayern Munich</t>
         </is>
       </c>
       <c r="D913" t="inlineStr">
         <is>
-          <t>Stuttgart</t>
+          <t>RB Leipzig</t>
         </is>
       </c>
       <c r="E913" t="n">
-        <v>10.5</v>
+        <v>10.77</v>
       </c>
       <c r="F913" t="n">
-        <v>-1.84</v>
+        <v>4.63</v>
       </c>
     </row>
     <row r="914">
@@ -24175,24 +24175,24 @@
       </c>
       <c r="C914" t="inlineStr">
         <is>
-          <t>Union Berlin</t>
+          <t>Elversberg</t>
         </is>
       </c>
       <c r="D914" t="inlineStr">
         <is>
-          <t>Borussia Dortmund</t>
+          <t>Augsburg</t>
         </is>
       </c>
       <c r="E914" t="n">
-        <v>9.779999999999999</v>
+        <v>10.1</v>
       </c>
       <c r="F914" t="n">
-        <v>-1.49</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="915">
       <c r="A915" s="1" t="n">
-        <v>46313</v>
+        <v>46312</v>
       </c>
       <c r="B915" t="inlineStr">
         <is>
@@ -24201,44 +24201,122 @@
       </c>
       <c r="C915" t="inlineStr">
         <is>
-          <t>Bayer Leverkusen</t>
+          <t>Hamburger SV</t>
         </is>
       </c>
       <c r="D915" t="inlineStr">
         <is>
-          <t>Freiburg</t>
+          <t>Stuttgart</t>
         </is>
       </c>
       <c r="E915" t="n">
-        <v>9.789999999999999</v>
+        <v>10.47</v>
       </c>
       <c r="F915" t="n">
-        <v>2.65</v>
+        <v>-1.84</v>
       </c>
     </row>
     <row r="916">
       <c r="A916" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B916" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C916" t="inlineStr">
+        <is>
+          <t>Union Berlin</t>
+        </is>
+      </c>
+      <c r="D916" t="inlineStr">
+        <is>
+          <t>Borussia Dortmund</t>
+        </is>
+      </c>
+      <c r="E916" t="n">
+        <v>9.77</v>
+      </c>
+      <c r="F916" t="n">
+        <v>-1.49</v>
+      </c>
+    </row>
+    <row r="917">
+      <c r="A917" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B917" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C917" t="inlineStr">
+        <is>
+          <t>Werder Bremen</t>
+        </is>
+      </c>
+      <c r="D917" t="inlineStr">
+        <is>
+          <t>Paderborn</t>
+        </is>
+      </c>
+      <c r="E917" t="n">
+        <v>9.56</v>
+      </c>
+      <c r="F917" t="n">
+        <v>1.36</v>
+      </c>
+    </row>
+    <row r="918">
+      <c r="A918" s="1" t="n">
         <v>46313</v>
       </c>
-      <c r="B916" t="inlineStr">
+      <c r="B918" t="inlineStr">
         <is>
           <t>Germany - Bundesliga</t>
         </is>
       </c>
-      <c r="C916" t="inlineStr">
+      <c r="C918" t="inlineStr">
+        <is>
+          <t>Bayer Leverkusen</t>
+        </is>
+      </c>
+      <c r="D918" t="inlineStr">
+        <is>
+          <t>Freiburg</t>
+        </is>
+      </c>
+      <c r="E918" t="n">
+        <v>9.789999999999999</v>
+      </c>
+      <c r="F918" t="n">
+        <v>2.65</v>
+      </c>
+    </row>
+    <row r="919">
+      <c r="A919" s="1" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B919" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C919" t="inlineStr">
         <is>
           <t>Borussia Monchengladbach</t>
         </is>
       </c>
-      <c r="D916" t="inlineStr">
+      <c r="D919" t="inlineStr">
         <is>
           <t>Hoffenheim</t>
         </is>
       </c>
-      <c r="E916" t="n">
+      <c r="E919" t="n">
         <v>10.26</v>
       </c>
-      <c r="F916" t="n">
+      <c r="F919" t="n">
         <v>-0.53</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily scrape output - 2026-10-16
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F919"/>
+  <dimension ref="A1:F944"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24132,7 +24132,7 @@
         </is>
       </c>
       <c r="E912" t="n">
-        <v>10.39</v>
+        <v>10.44</v>
       </c>
       <c r="F912" t="n">
         <v>1.33</v>
@@ -24140,137 +24140,137 @@
     </row>
     <row r="913">
       <c r="A913" s="1" t="n">
-        <v>46312</v>
+        <v>46311</v>
       </c>
       <c r="B913" t="inlineStr">
         <is>
-          <t>Germany - Bundesliga</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C913" t="inlineStr">
         <is>
-          <t>Bayern Munich</t>
+          <t>Ruch Chorzow</t>
         </is>
       </c>
       <c r="D913" t="inlineStr">
         <is>
-          <t>RB Leipzig</t>
+          <t>Odra Opole</t>
         </is>
       </c>
       <c r="E913" t="n">
-        <v>10.77</v>
+        <v>10.58</v>
       </c>
       <c r="F913" t="n">
-        <v>4.63</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="914">
       <c r="A914" s="1" t="n">
-        <v>46312</v>
+        <v>46311</v>
       </c>
       <c r="B914" t="inlineStr">
         <is>
-          <t>Germany - Bundesliga</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C914" t="inlineStr">
         <is>
-          <t>Elversberg</t>
+          <t>Warta Poznan</t>
         </is>
       </c>
       <c r="D914" t="inlineStr">
         <is>
-          <t>Augsburg</t>
+          <t>Unia Skierniewice</t>
         </is>
       </c>
       <c r="E914" t="n">
-        <v>10.1</v>
+        <v>10.49</v>
       </c>
       <c r="F914" t="n">
-        <v>0.84</v>
+        <v>0.48</v>
       </c>
     </row>
     <row r="915">
       <c r="A915" s="1" t="n">
-        <v>46312</v>
+        <v>46311</v>
       </c>
       <c r="B915" t="inlineStr">
         <is>
-          <t>Germany - Bundesliga</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C915" t="inlineStr">
         <is>
-          <t>Hamburger SV</t>
+          <t>Widzew Lodz</t>
         </is>
       </c>
       <c r="D915" t="inlineStr">
         <is>
-          <t>Stuttgart</t>
+          <t>Wisla Krakow</t>
         </is>
       </c>
       <c r="E915" t="n">
-        <v>10.47</v>
+        <v>10.45</v>
       </c>
       <c r="F915" t="n">
-        <v>-1.84</v>
+        <v>0.68</v>
       </c>
     </row>
     <row r="916">
       <c r="A916" s="1" t="n">
-        <v>46312</v>
+        <v>46311</v>
       </c>
       <c r="B916" t="inlineStr">
         <is>
-          <t>Germany - Bundesliga</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C916" t="inlineStr">
         <is>
-          <t>Union Berlin</t>
+          <t>Wieczysta Krakow</t>
         </is>
       </c>
       <c r="D916" t="inlineStr">
         <is>
-          <t>Borussia Dortmund</t>
+          <t>Rakow Czestochowa</t>
         </is>
       </c>
       <c r="E916" t="n">
-        <v>9.77</v>
+        <v>10.28</v>
       </c>
       <c r="F916" t="n">
-        <v>-1.49</v>
+        <v>1.14</v>
       </c>
     </row>
     <row r="917">
       <c r="A917" s="1" t="n">
-        <v>46312</v>
+        <v>46311</v>
       </c>
       <c r="B917" t="inlineStr">
         <is>
-          <t>Germany - Bundesliga</t>
+          <t>Turkey - Super Lig</t>
         </is>
       </c>
       <c r="C917" t="inlineStr">
         <is>
-          <t>Werder Bremen</t>
+          <t>Corum Belediyespor</t>
         </is>
       </c>
       <c r="D917" t="inlineStr">
         <is>
-          <t>Paderborn</t>
+          <t>Caykur Rizespor</t>
         </is>
       </c>
       <c r="E917" t="n">
-        <v>9.56</v>
+        <v>9.460000000000001</v>
       </c>
       <c r="F917" t="n">
-        <v>1.36</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="918">
       <c r="A918" s="1" t="n">
-        <v>46313</v>
+        <v>46312</v>
       </c>
       <c r="B918" t="inlineStr">
         <is>
@@ -24279,45 +24279,695 @@
       </c>
       <c r="C918" t="inlineStr">
         <is>
-          <t>Bayer Leverkusen</t>
+          <t>Bayern Munich</t>
         </is>
       </c>
       <c r="D918" t="inlineStr">
         <is>
-          <t>Freiburg</t>
+          <t>RB Leipzig</t>
         </is>
       </c>
       <c r="E918" t="n">
-        <v>9.789999999999999</v>
+        <v>10.75</v>
       </c>
       <c r="F918" t="n">
-        <v>2.65</v>
+        <v>4.62</v>
       </c>
     </row>
     <row r="919">
       <c r="A919" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B919" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C919" t="inlineStr">
+        <is>
+          <t>Elversberg</t>
+        </is>
+      </c>
+      <c r="D919" t="inlineStr">
+        <is>
+          <t>Augsburg</t>
+        </is>
+      </c>
+      <c r="E919" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="F919" t="n">
+        <v>0.84</v>
+      </c>
+    </row>
+    <row r="920">
+      <c r="A920" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B920" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C920" t="inlineStr">
+        <is>
+          <t>Hamburger SV</t>
+        </is>
+      </c>
+      <c r="D920" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="E920" t="n">
+        <v>10.44</v>
+      </c>
+      <c r="F920" t="n">
+        <v>-1.83</v>
+      </c>
+    </row>
+    <row r="921">
+      <c r="A921" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B921" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C921" t="inlineStr">
+        <is>
+          <t>Schalke 04</t>
+        </is>
+      </c>
+      <c r="D921" t="inlineStr">
+        <is>
+          <t>Mainz 05</t>
+        </is>
+      </c>
+      <c r="E921" t="n">
+        <v>9.56</v>
+      </c>
+      <c r="F921" t="n">
+        <v>-0.49</v>
+      </c>
+    </row>
+    <row r="922">
+      <c r="A922" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B922" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C922" t="inlineStr">
+        <is>
+          <t>Union Berlin</t>
+        </is>
+      </c>
+      <c r="D922" t="inlineStr">
+        <is>
+          <t>Borussia Dortmund</t>
+        </is>
+      </c>
+      <c r="E922" t="n">
+        <v>9.59</v>
+      </c>
+      <c r="F922" t="n">
+        <v>-1.7</v>
+      </c>
+    </row>
+    <row r="923">
+      <c r="A923" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B923" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C923" t="inlineStr">
+        <is>
+          <t>Werder Bremen</t>
+        </is>
+      </c>
+      <c r="D923" t="inlineStr">
+        <is>
+          <t>Paderborn</t>
+        </is>
+      </c>
+      <c r="E923" t="n">
+        <v>9.65</v>
+      </c>
+      <c r="F923" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="924">
+      <c r="A924" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B924" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C924" t="inlineStr">
+        <is>
+          <t>Miedz Legnica</t>
+        </is>
+      </c>
+      <c r="D924" t="inlineStr">
+        <is>
+          <t>Stal Mielec</t>
+        </is>
+      </c>
+      <c r="E924" t="n">
+        <v>10.95</v>
+      </c>
+      <c r="F924" t="n">
+        <v>1.47</v>
+      </c>
+    </row>
+    <row r="925">
+      <c r="A925" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B925" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C925" t="inlineStr">
+        <is>
+          <t>Pogon Grodzisk Mazowiecki</t>
+        </is>
+      </c>
+      <c r="D925" t="inlineStr">
+        <is>
+          <t>Polonia Warsaw</t>
+        </is>
+      </c>
+      <c r="E925" t="n">
+        <v>11.08</v>
+      </c>
+      <c r="F925" t="n">
+        <v>-1.13</v>
+      </c>
+    </row>
+    <row r="926">
+      <c r="A926" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B926" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C926" t="inlineStr">
+        <is>
+          <t>Polonia Bytom</t>
+        </is>
+      </c>
+      <c r="D926" t="inlineStr">
+        <is>
+          <t>Chrobry Glogow</t>
+        </is>
+      </c>
+      <c r="E926" t="n">
+        <v>10.09</v>
+      </c>
+      <c r="F926" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="927">
+      <c r="A927" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B927" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C927" t="inlineStr">
+        <is>
+          <t>Cracovia Krakow</t>
+        </is>
+      </c>
+      <c r="D927" t="inlineStr">
+        <is>
+          <t>Legia Warsaw</t>
+        </is>
+      </c>
+      <c r="E927" t="n">
+        <v>9.73</v>
+      </c>
+      <c r="F927" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B928" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C928" t="inlineStr">
+        <is>
+          <t>GKS Katowice</t>
+        </is>
+      </c>
+      <c r="D928" t="inlineStr">
+        <is>
+          <t>Pogon Szczecin</t>
+        </is>
+      </c>
+      <c r="E928" t="n">
+        <v>10.05</v>
+      </c>
+      <c r="F928" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B929" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C929" t="inlineStr">
+        <is>
+          <t>Motor Lublin</t>
+        </is>
+      </c>
+      <c r="D929" t="inlineStr">
+        <is>
+          <t>Slask Wroclaw</t>
+        </is>
+      </c>
+      <c r="E929" t="n">
+        <v>9.98</v>
+      </c>
+      <c r="F929" t="n">
+        <v>1.33</v>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B930" t="inlineStr">
+        <is>
+          <t>Turkey - Super Lig</t>
+        </is>
+      </c>
+      <c r="C930" t="inlineStr">
+        <is>
+          <t>Fenerbahce</t>
+        </is>
+      </c>
+      <c r="D930" t="inlineStr">
+        <is>
+          <t>Alanyaspor</t>
+        </is>
+      </c>
+      <c r="E930" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="F930" t="n">
+        <v>3.21</v>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" s="1" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B931" t="inlineStr">
+        <is>
+          <t>Turkey - Super Lig</t>
+        </is>
+      </c>
+      <c r="C931" t="inlineStr">
+        <is>
+          <t>Genclerbirligi</t>
+        </is>
+      </c>
+      <c r="D931" t="inlineStr">
+        <is>
+          <t>Galatasaray</t>
+        </is>
+      </c>
+      <c r="E931" t="n">
+        <v>10.09</v>
+      </c>
+      <c r="F931" t="n">
+        <v>-2.89</v>
+      </c>
+    </row>
+    <row r="932">
+      <c r="A932" s="1" t="n">
         <v>46313</v>
       </c>
-      <c r="B919" t="inlineStr">
+      <c r="B932" t="inlineStr">
         <is>
           <t>Germany - Bundesliga</t>
         </is>
       </c>
-      <c r="C919" t="inlineStr">
+      <c r="C932" t="inlineStr">
+        <is>
+          <t>Bayer Leverkusen</t>
+        </is>
+      </c>
+      <c r="D932" t="inlineStr">
+        <is>
+          <t>Freiburg</t>
+        </is>
+      </c>
+      <c r="E932" t="n">
+        <v>9.69</v>
+      </c>
+      <c r="F932" t="n">
+        <v>2.65</v>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933" s="1" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B933" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C933" t="inlineStr">
         <is>
           <t>Borussia Monchengladbach</t>
         </is>
       </c>
-      <c r="D919" t="inlineStr">
+      <c r="D933" t="inlineStr">
         <is>
           <t>Hoffenheim</t>
         </is>
       </c>
-      <c r="E919" t="n">
-        <v>10.26</v>
-      </c>
-      <c r="F919" t="n">
+      <c r="E933" t="n">
+        <v>10.21</v>
+      </c>
+      <c r="F933" t="n">
         <v>-0.53</v>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" s="1" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B934" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C934" t="inlineStr">
+        <is>
+          <t>LKS Lodz</t>
+        </is>
+      </c>
+      <c r="D934" t="inlineStr">
+        <is>
+          <t>Podbeskidzie Bielsko-Biala</t>
+        </is>
+      </c>
+      <c r="E934" t="n">
+        <v>10.63</v>
+      </c>
+      <c r="F934" t="n">
+        <v>1.15</v>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935" s="1" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B935" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C935" t="inlineStr">
+        <is>
+          <t>Pogon Siedlce</t>
+        </is>
+      </c>
+      <c r="D935" t="inlineStr">
+        <is>
+          <t>Stal Rzeszow</t>
+        </is>
+      </c>
+      <c r="E935" t="n">
+        <v>10.56</v>
+      </c>
+      <c r="F935" t="n">
+        <v>-0.1</v>
+      </c>
+    </row>
+    <row r="936">
+      <c r="A936" s="1" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B936" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C936" t="inlineStr">
+        <is>
+          <t>Gornik Zabrze</t>
+        </is>
+      </c>
+      <c r="D936" t="inlineStr">
+        <is>
+          <t>Piast Gliwice</t>
+        </is>
+      </c>
+      <c r="E936" t="n">
+        <v>10.35</v>
+      </c>
+      <c r="F936" t="n">
+        <v>2.61</v>
+      </c>
+    </row>
+    <row r="937">
+      <c r="A937" s="1" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B937" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C937" t="inlineStr">
+        <is>
+          <t>Lech Poznan</t>
+        </is>
+      </c>
+      <c r="D937" t="inlineStr">
+        <is>
+          <t>Korona Kielce</t>
+        </is>
+      </c>
+      <c r="E937" t="n">
+        <v>10.34</v>
+      </c>
+      <c r="F937" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="938">
+      <c r="A938" s="1" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B938" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C938" t="inlineStr">
+        <is>
+          <t>Zaglebie Lubin</t>
+        </is>
+      </c>
+      <c r="D938" t="inlineStr">
+        <is>
+          <t>Jagiellonia Bialystok</t>
+        </is>
+      </c>
+      <c r="E938" t="n">
+        <v>9.82</v>
+      </c>
+      <c r="F938" t="n">
+        <v>-0.46</v>
+      </c>
+    </row>
+    <row r="939">
+      <c r="A939" s="1" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B939" t="inlineStr">
+        <is>
+          <t>Turkey - Super Lig</t>
+        </is>
+      </c>
+      <c r="C939" t="inlineStr">
+        <is>
+          <t>Istanbul Basaksehir</t>
+        </is>
+      </c>
+      <c r="D939" t="inlineStr">
+        <is>
+          <t>Gaziantep</t>
+        </is>
+      </c>
+      <c r="E939" t="n">
+        <v>9.65</v>
+      </c>
+      <c r="F939" t="n">
+        <v>1.95</v>
+      </c>
+    </row>
+    <row r="940">
+      <c r="A940" s="1" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B940" t="inlineStr">
+        <is>
+          <t>Turkey - Super Lig</t>
+        </is>
+      </c>
+      <c r="C940" t="inlineStr">
+        <is>
+          <t>Kasimpasa</t>
+        </is>
+      </c>
+      <c r="D940" t="inlineStr">
+        <is>
+          <t>Samsunspor</t>
+        </is>
+      </c>
+      <c r="E940" t="n">
+        <v>9.67</v>
+      </c>
+      <c r="F940" t="n">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="941">
+      <c r="A941" s="1" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B941" t="inlineStr">
+        <is>
+          <t>Turkey - Super Lig</t>
+        </is>
+      </c>
+      <c r="C941" t="inlineStr">
+        <is>
+          <t>Kocaelispor</t>
+        </is>
+      </c>
+      <c r="D941" t="inlineStr">
+        <is>
+          <t>Goztepe</t>
+        </is>
+      </c>
+      <c r="E941" t="n">
+        <v>9.31</v>
+      </c>
+      <c r="F941" t="n">
+        <v>-0.04</v>
+      </c>
+    </row>
+    <row r="942">
+      <c r="A942" s="1" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B942" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C942" t="inlineStr">
+        <is>
+          <t>Wisla Plock</t>
+        </is>
+      </c>
+      <c r="D942" t="inlineStr">
+        <is>
+          <t>Radomiak Radom</t>
+        </is>
+      </c>
+      <c r="E942" t="n">
+        <v>10.78</v>
+      </c>
+      <c r="F942" t="n">
+        <v>1.11</v>
+      </c>
+    </row>
+    <row r="943">
+      <c r="A943" s="1" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B943" t="inlineStr">
+        <is>
+          <t>Portugal - Primeira Liga</t>
+        </is>
+      </c>
+      <c r="C943" t="inlineStr">
+        <is>
+          <t>Braga</t>
+        </is>
+      </c>
+      <c r="D943" t="inlineStr">
+        <is>
+          <t>Gil Vicente</t>
+        </is>
+      </c>
+      <c r="E943" t="n">
+        <v>9.279999999999999</v>
+      </c>
+      <c r="F943" t="n">
+        <v>2.19</v>
+      </c>
+    </row>
+    <row r="944">
+      <c r="A944" s="1" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B944" t="inlineStr">
+        <is>
+          <t>Turkey - Super Lig</t>
+        </is>
+      </c>
+      <c r="C944" t="inlineStr">
+        <is>
+          <t>Trabzonspor</t>
+        </is>
+      </c>
+      <c r="D944" t="inlineStr">
+        <is>
+          <t>Besiktas</t>
+        </is>
+      </c>
+      <c r="E944" t="n">
+        <v>10.12</v>
+      </c>
+      <c r="F944" t="n">
+        <v>-0.34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-10-17
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F944"/>
+  <dimension ref="A1:F946"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24288,10 +24288,10 @@
         </is>
       </c>
       <c r="E918" t="n">
-        <v>10.75</v>
+        <v>10.97</v>
       </c>
       <c r="F918" t="n">
-        <v>4.62</v>
+        <v>4.54</v>
       </c>
     </row>
     <row r="919">
@@ -24314,10 +24314,10 @@
         </is>
       </c>
       <c r="E919" t="n">
-        <v>10.1</v>
+        <v>10.26</v>
       </c>
       <c r="F919" t="n">
-        <v>0.84</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="920">
@@ -24340,10 +24340,10 @@
         </is>
       </c>
       <c r="E920" t="n">
-        <v>10.44</v>
+        <v>10.23</v>
       </c>
       <c r="F920" t="n">
-        <v>-1.83</v>
+        <v>-1.7</v>
       </c>
     </row>
     <row r="921">
@@ -24392,10 +24392,10 @@
         </is>
       </c>
       <c r="E922" t="n">
-        <v>9.59</v>
+        <v>9.460000000000001</v>
       </c>
       <c r="F922" t="n">
-        <v>-1.7</v>
+        <v>-1.67</v>
       </c>
     </row>
     <row r="923">
@@ -24418,10 +24418,10 @@
         </is>
       </c>
       <c r="E923" t="n">
-        <v>9.65</v>
+        <v>9.69</v>
       </c>
       <c r="F923" t="n">
-        <v>1.2</v>
+        <v>1.18</v>
       </c>
     </row>
     <row r="924">
@@ -24444,10 +24444,10 @@
         </is>
       </c>
       <c r="E924" t="n">
-        <v>10.95</v>
+        <v>10.98</v>
       </c>
       <c r="F924" t="n">
-        <v>1.47</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="925">
@@ -24470,10 +24470,10 @@
         </is>
       </c>
       <c r="E925" t="n">
-        <v>11.08</v>
+        <v>10.8</v>
       </c>
       <c r="F925" t="n">
-        <v>-1.13</v>
+        <v>-1.09</v>
       </c>
     </row>
     <row r="926">
@@ -24499,7 +24499,7 @@
         <v>10.09</v>
       </c>
       <c r="F926" t="n">
-        <v>2</v>
+        <v>1.71</v>
       </c>
     </row>
     <row r="927">
@@ -24522,10 +24522,10 @@
         </is>
       </c>
       <c r="E927" t="n">
-        <v>9.73</v>
+        <v>9.6</v>
       </c>
       <c r="F927" t="n">
-        <v>0.02</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="928">
@@ -24551,7 +24551,7 @@
         <v>10.05</v>
       </c>
       <c r="F928" t="n">
-        <v>1</v>
+        <v>1.16</v>
       </c>
     </row>
     <row r="929">
@@ -24591,19 +24591,19 @@
       </c>
       <c r="C930" t="inlineStr">
         <is>
-          <t>Fenerbahce</t>
+          <t>Amedspor</t>
         </is>
       </c>
       <c r="D930" t="inlineStr">
         <is>
-          <t>Alanyaspor</t>
+          <t>Konyaspor</t>
         </is>
       </c>
       <c r="E930" t="n">
-        <v>9.699999999999999</v>
+        <v>9.220000000000001</v>
       </c>
       <c r="F930" t="n">
-        <v>3.21</v>
+        <v>1.53</v>
       </c>
     </row>
     <row r="931">
@@ -24617,71 +24617,71 @@
       </c>
       <c r="C931" t="inlineStr">
         <is>
-          <t>Genclerbirligi</t>
+          <t>Erzurumspor</t>
         </is>
       </c>
       <c r="D931" t="inlineStr">
         <is>
-          <t>Galatasaray</t>
+          <t>Eyupspor</t>
         </is>
       </c>
       <c r="E931" t="n">
-        <v>10.09</v>
+        <v>8.83</v>
       </c>
       <c r="F931" t="n">
-        <v>-2.89</v>
+        <v>1.98</v>
       </c>
     </row>
     <row r="932">
       <c r="A932" s="1" t="n">
-        <v>46313</v>
+        <v>46312</v>
       </c>
       <c r="B932" t="inlineStr">
         <is>
-          <t>Germany - Bundesliga</t>
+          <t>Turkey - Super Lig</t>
         </is>
       </c>
       <c r="C932" t="inlineStr">
         <is>
-          <t>Bayer Leverkusen</t>
+          <t>Fenerbahce</t>
         </is>
       </c>
       <c r="D932" t="inlineStr">
         <is>
-          <t>Freiburg</t>
+          <t>Alanyaspor</t>
         </is>
       </c>
       <c r="E932" t="n">
-        <v>9.69</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="F932" t="n">
-        <v>2.65</v>
+        <v>3.21</v>
       </c>
     </row>
     <row r="933">
       <c r="A933" s="1" t="n">
-        <v>46313</v>
+        <v>46312</v>
       </c>
       <c r="B933" t="inlineStr">
         <is>
-          <t>Germany - Bundesliga</t>
+          <t>Turkey - Super Lig</t>
         </is>
       </c>
       <c r="C933" t="inlineStr">
         <is>
-          <t>Borussia Monchengladbach</t>
+          <t>Genclerbirligi</t>
         </is>
       </c>
       <c r="D933" t="inlineStr">
         <is>
-          <t>Hoffenheim</t>
+          <t>Galatasaray</t>
         </is>
       </c>
       <c r="E933" t="n">
-        <v>10.21</v>
+        <v>10.09</v>
       </c>
       <c r="F933" t="n">
-        <v>-0.53</v>
+        <v>-2.89</v>
       </c>
     </row>
     <row r="934">
@@ -24690,24 +24690,24 @@
       </c>
       <c r="B934" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Germany - Bundesliga</t>
         </is>
       </c>
       <c r="C934" t="inlineStr">
         <is>
-          <t>LKS Lodz</t>
+          <t>Bayer Leverkusen</t>
         </is>
       </c>
       <c r="D934" t="inlineStr">
         <is>
-          <t>Podbeskidzie Bielsko-Biala</t>
+          <t>Freiburg</t>
         </is>
       </c>
       <c r="E934" t="n">
-        <v>10.63</v>
+        <v>9.69</v>
       </c>
       <c r="F934" t="n">
-        <v>1.15</v>
+        <v>2.65</v>
       </c>
     </row>
     <row r="935">
@@ -24716,24 +24716,24 @@
       </c>
       <c r="B935" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Germany - Bundesliga</t>
         </is>
       </c>
       <c r="C935" t="inlineStr">
         <is>
-          <t>Pogon Siedlce</t>
+          <t>Borussia Monchengladbach</t>
         </is>
       </c>
       <c r="D935" t="inlineStr">
         <is>
-          <t>Stal Rzeszow</t>
+          <t>Hoffenheim</t>
         </is>
       </c>
       <c r="E935" t="n">
-        <v>10.56</v>
+        <v>10.21</v>
       </c>
       <c r="F935" t="n">
-        <v>-0.1</v>
+        <v>-0.53</v>
       </c>
     </row>
     <row r="936">
@@ -24742,24 +24742,24 @@
       </c>
       <c r="B936" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C936" t="inlineStr">
         <is>
-          <t>Gornik Zabrze</t>
+          <t>LKS Lodz</t>
         </is>
       </c>
       <c r="D936" t="inlineStr">
         <is>
-          <t>Piast Gliwice</t>
+          <t>Podbeskidzie Bielsko-Biala</t>
         </is>
       </c>
       <c r="E936" t="n">
-        <v>10.35</v>
+        <v>10.63</v>
       </c>
       <c r="F936" t="n">
-        <v>2.61</v>
+        <v>1.15</v>
       </c>
     </row>
     <row r="937">
@@ -24768,24 +24768,24 @@
       </c>
       <c r="B937" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C937" t="inlineStr">
         <is>
-          <t>Lech Poznan</t>
+          <t>Pogon Siedlce</t>
         </is>
       </c>
       <c r="D937" t="inlineStr">
         <is>
-          <t>Korona Kielce</t>
+          <t>Stal Rzeszow</t>
         </is>
       </c>
       <c r="E937" t="n">
-        <v>10.34</v>
+        <v>10.56</v>
       </c>
       <c r="F937" t="n">
-        <v>2.25</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="938">
@@ -24799,19 +24799,19 @@
       </c>
       <c r="C938" t="inlineStr">
         <is>
-          <t>Zaglebie Lubin</t>
+          <t>Gornik Zabrze</t>
         </is>
       </c>
       <c r="D938" t="inlineStr">
         <is>
-          <t>Jagiellonia Bialystok</t>
+          <t>Piast Gliwice</t>
         </is>
       </c>
       <c r="E938" t="n">
-        <v>9.82</v>
+        <v>10.22</v>
       </c>
       <c r="F938" t="n">
-        <v>-0.46</v>
+        <v>2.61</v>
       </c>
     </row>
     <row r="939">
@@ -24820,24 +24820,24 @@
       </c>
       <c r="B939" t="inlineStr">
         <is>
-          <t>Turkey - Super Lig</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C939" t="inlineStr">
         <is>
-          <t>Istanbul Basaksehir</t>
+          <t>Lech Poznan</t>
         </is>
       </c>
       <c r="D939" t="inlineStr">
         <is>
-          <t>Gaziantep</t>
+          <t>Korona Kielce</t>
         </is>
       </c>
       <c r="E939" t="n">
-        <v>9.65</v>
+        <v>10.4</v>
       </c>
       <c r="F939" t="n">
-        <v>1.95</v>
+        <v>2.32</v>
       </c>
     </row>
     <row r="940">
@@ -24846,24 +24846,24 @@
       </c>
       <c r="B940" t="inlineStr">
         <is>
-          <t>Turkey - Super Lig</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C940" t="inlineStr">
         <is>
-          <t>Kasimpasa</t>
+          <t>Zaglebie Lubin</t>
         </is>
       </c>
       <c r="D940" t="inlineStr">
         <is>
-          <t>Samsunspor</t>
+          <t>Jagiellonia Bialystok</t>
         </is>
       </c>
       <c r="E940" t="n">
-        <v>9.67</v>
+        <v>9.82</v>
       </c>
       <c r="F940" t="n">
-        <v>0.09</v>
+        <v>-0.46</v>
       </c>
     </row>
     <row r="941">
@@ -24877,71 +24877,71 @@
       </c>
       <c r="C941" t="inlineStr">
         <is>
-          <t>Kocaelispor</t>
+          <t>Istanbul Basaksehir</t>
         </is>
       </c>
       <c r="D941" t="inlineStr">
         <is>
-          <t>Goztepe</t>
+          <t>Gaziantep</t>
         </is>
       </c>
       <c r="E941" t="n">
-        <v>9.31</v>
+        <v>9.56</v>
       </c>
       <c r="F941" t="n">
-        <v>-0.04</v>
+        <v>1.95</v>
       </c>
     </row>
     <row r="942">
       <c r="A942" s="1" t="n">
-        <v>46314</v>
+        <v>46313</v>
       </c>
       <c r="B942" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Turkey - Super Lig</t>
         </is>
       </c>
       <c r="C942" t="inlineStr">
         <is>
-          <t>Wisla Plock</t>
+          <t>Kasimpasa</t>
         </is>
       </c>
       <c r="D942" t="inlineStr">
         <is>
-          <t>Radomiak Radom</t>
+          <t>Samsunspor</t>
         </is>
       </c>
       <c r="E942" t="n">
-        <v>10.78</v>
+        <v>9.67</v>
       </c>
       <c r="F942" t="n">
-        <v>1.11</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="943">
       <c r="A943" s="1" t="n">
-        <v>46314</v>
+        <v>46313</v>
       </c>
       <c r="B943" t="inlineStr">
         <is>
-          <t>Portugal - Primeira Liga</t>
+          <t>Turkey - Super Lig</t>
         </is>
       </c>
       <c r="C943" t="inlineStr">
         <is>
-          <t>Braga</t>
+          <t>Kocaelispor</t>
         </is>
       </c>
       <c r="D943" t="inlineStr">
         <is>
-          <t>Gil Vicente</t>
+          <t>Goztepe</t>
         </is>
       </c>
       <c r="E943" t="n">
-        <v>9.279999999999999</v>
+        <v>9.039999999999999</v>
       </c>
       <c r="F943" t="n">
-        <v>2.19</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="944">
@@ -24950,24 +24950,76 @@
       </c>
       <c r="B944" t="inlineStr">
         <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C944" t="inlineStr">
+        <is>
+          <t>Wisla Plock</t>
+        </is>
+      </c>
+      <c r="D944" t="inlineStr">
+        <is>
+          <t>Radomiak Radom</t>
+        </is>
+      </c>
+      <c r="E944" t="n">
+        <v>10.78</v>
+      </c>
+      <c r="F944" t="n">
+        <v>1.11</v>
+      </c>
+    </row>
+    <row r="945">
+      <c r="A945" s="1" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B945" t="inlineStr">
+        <is>
+          <t>Portugal - Primeira Liga</t>
+        </is>
+      </c>
+      <c r="C945" t="inlineStr">
+        <is>
+          <t>Braga</t>
+        </is>
+      </c>
+      <c r="D945" t="inlineStr">
+        <is>
+          <t>Gil Vicente</t>
+        </is>
+      </c>
+      <c r="E945" t="n">
+        <v>9.15</v>
+      </c>
+      <c r="F945" t="n">
+        <v>2.19</v>
+      </c>
+    </row>
+    <row r="946">
+      <c r="A946" s="1" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B946" t="inlineStr">
+        <is>
           <t>Turkey - Super Lig</t>
         </is>
       </c>
-      <c r="C944" t="inlineStr">
+      <c r="C946" t="inlineStr">
         <is>
           <t>Trabzonspor</t>
         </is>
       </c>
-      <c r="D944" t="inlineStr">
+      <c r="D946" t="inlineStr">
         <is>
           <t>Besiktas</t>
         </is>
       </c>
-      <c r="E944" t="n">
-        <v>10.12</v>
-      </c>
-      <c r="F944" t="n">
-        <v>-0.34</v>
+      <c r="E946" t="n">
+        <v>10.14</v>
+      </c>
+      <c r="F946" t="n">
+        <v>-0.47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-10-18
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F946"/>
+  <dimension ref="A1:F947"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24704,10 +24704,10 @@
         </is>
       </c>
       <c r="E934" t="n">
-        <v>9.69</v>
+        <v>9.529999999999999</v>
       </c>
       <c r="F934" t="n">
-        <v>2.65</v>
+        <v>2.66</v>
       </c>
     </row>
     <row r="935">
@@ -24730,10 +24730,10 @@
         </is>
       </c>
       <c r="E935" t="n">
-        <v>10.21</v>
+        <v>10.4</v>
       </c>
       <c r="F935" t="n">
-        <v>-0.53</v>
+        <v>-0.58</v>
       </c>
     </row>
     <row r="936">
@@ -24756,7 +24756,7 @@
         </is>
       </c>
       <c r="E936" t="n">
-        <v>10.63</v>
+        <v>10.49</v>
       </c>
       <c r="F936" t="n">
         <v>1.15</v>
@@ -24773,19 +24773,19 @@
       </c>
       <c r="C937" t="inlineStr">
         <is>
-          <t>Pogon Siedlce</t>
+          <t>Lechia Gdansk</t>
         </is>
       </c>
       <c r="D937" t="inlineStr">
         <is>
-          <t>Stal Rzeszow</t>
+          <t>Arka Gdynia</t>
         </is>
       </c>
       <c r="E937" t="n">
-        <v>10.56</v>
+        <v>10.34</v>
       </c>
       <c r="F937" t="n">
-        <v>-0.1</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="938">
@@ -24794,24 +24794,24 @@
       </c>
       <c r="B938" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C938" t="inlineStr">
         <is>
-          <t>Gornik Zabrze</t>
+          <t>Pogon Siedlce</t>
         </is>
       </c>
       <c r="D938" t="inlineStr">
         <is>
-          <t>Piast Gliwice</t>
+          <t>Stal Rzeszow</t>
         </is>
       </c>
       <c r="E938" t="n">
-        <v>10.22</v>
+        <v>10.82</v>
       </c>
       <c r="F938" t="n">
-        <v>2.61</v>
+        <v>-0.13</v>
       </c>
     </row>
     <row r="939">
@@ -24825,19 +24825,19 @@
       </c>
       <c r="C939" t="inlineStr">
         <is>
-          <t>Lech Poznan</t>
+          <t>Gornik Zabrze</t>
         </is>
       </c>
       <c r="D939" t="inlineStr">
         <is>
-          <t>Korona Kielce</t>
+          <t>Piast Gliwice</t>
         </is>
       </c>
       <c r="E939" t="n">
-        <v>10.4</v>
+        <v>10.22</v>
       </c>
       <c r="F939" t="n">
-        <v>2.32</v>
+        <v>2.62</v>
       </c>
     </row>
     <row r="940">
@@ -24851,19 +24851,19 @@
       </c>
       <c r="C940" t="inlineStr">
         <is>
-          <t>Zaglebie Lubin</t>
+          <t>Lech Poznan</t>
         </is>
       </c>
       <c r="D940" t="inlineStr">
         <is>
-          <t>Jagiellonia Bialystok</t>
+          <t>Korona Kielce</t>
         </is>
       </c>
       <c r="E940" t="n">
-        <v>9.82</v>
+        <v>10.4</v>
       </c>
       <c r="F940" t="n">
-        <v>-0.46</v>
+        <v>2.32</v>
       </c>
     </row>
     <row r="941">
@@ -24872,24 +24872,24 @@
       </c>
       <c r="B941" t="inlineStr">
         <is>
-          <t>Turkey - Super Lig</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C941" t="inlineStr">
         <is>
-          <t>Istanbul Basaksehir</t>
+          <t>Zaglebie Lubin</t>
         </is>
       </c>
       <c r="D941" t="inlineStr">
         <is>
-          <t>Gaziantep</t>
+          <t>Jagiellonia Bialystok</t>
         </is>
       </c>
       <c r="E941" t="n">
-        <v>9.56</v>
+        <v>9.710000000000001</v>
       </c>
       <c r="F941" t="n">
-        <v>1.95</v>
+        <v>-0.45</v>
       </c>
     </row>
     <row r="942">
@@ -24903,19 +24903,19 @@
       </c>
       <c r="C942" t="inlineStr">
         <is>
-          <t>Kasimpasa</t>
+          <t>Istanbul Basaksehir</t>
         </is>
       </c>
       <c r="D942" t="inlineStr">
         <is>
-          <t>Samsunspor</t>
+          <t>Gaziantep</t>
         </is>
       </c>
       <c r="E942" t="n">
-        <v>9.67</v>
+        <v>9.33</v>
       </c>
       <c r="F942" t="n">
-        <v>0.09</v>
+        <v>1.95</v>
       </c>
     </row>
     <row r="943">
@@ -24929,45 +24929,45 @@
       </c>
       <c r="C943" t="inlineStr">
         <is>
-          <t>Kocaelispor</t>
+          <t>Kasimpasa</t>
         </is>
       </c>
       <c r="D943" t="inlineStr">
         <is>
-          <t>Goztepe</t>
+          <t>Samsunspor</t>
         </is>
       </c>
       <c r="E943" t="n">
-        <v>9.039999999999999</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="F943" t="n">
-        <v>-0</v>
+        <v>0.14</v>
       </c>
     </row>
     <row r="944">
       <c r="A944" s="1" t="n">
-        <v>46314</v>
+        <v>46313</v>
       </c>
       <c r="B944" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Turkey - Super Lig</t>
         </is>
       </c>
       <c r="C944" t="inlineStr">
         <is>
-          <t>Wisla Plock</t>
+          <t>Kocaelispor</t>
         </is>
       </c>
       <c r="D944" t="inlineStr">
         <is>
-          <t>Radomiak Radom</t>
+          <t>Goztepe</t>
         </is>
       </c>
       <c r="E944" t="n">
-        <v>10.78</v>
+        <v>9.050000000000001</v>
       </c>
       <c r="F944" t="n">
-        <v>1.11</v>
+        <v>-0.01</v>
       </c>
     </row>
     <row r="945">
@@ -24976,24 +24976,24 @@
       </c>
       <c r="B945" t="inlineStr">
         <is>
-          <t>Portugal - Primeira Liga</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C945" t="inlineStr">
         <is>
-          <t>Braga</t>
+          <t>Wisla Plock</t>
         </is>
       </c>
       <c r="D945" t="inlineStr">
         <is>
-          <t>Gil Vicente</t>
+          <t>Radomiak Radom</t>
         </is>
       </c>
       <c r="E945" t="n">
-        <v>9.15</v>
+        <v>10.78</v>
       </c>
       <c r="F945" t="n">
-        <v>2.19</v>
+        <v>1.11</v>
       </c>
     </row>
     <row r="946">
@@ -25002,24 +25002,50 @@
       </c>
       <c r="B946" t="inlineStr">
         <is>
+          <t>Portugal - Primeira Liga</t>
+        </is>
+      </c>
+      <c r="C946" t="inlineStr">
+        <is>
+          <t>Braga</t>
+        </is>
+      </c>
+      <c r="D946" t="inlineStr">
+        <is>
+          <t>Gil Vicente</t>
+        </is>
+      </c>
+      <c r="E946" t="n">
+        <v>9.15</v>
+      </c>
+      <c r="F946" t="n">
+        <v>2.19</v>
+      </c>
+    </row>
+    <row r="947">
+      <c r="A947" s="1" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B947" t="inlineStr">
+        <is>
           <t>Turkey - Super Lig</t>
         </is>
       </c>
-      <c r="C946" t="inlineStr">
+      <c r="C947" t="inlineStr">
         <is>
           <t>Trabzonspor</t>
         </is>
       </c>
-      <c r="D946" t="inlineStr">
+      <c r="D947" t="inlineStr">
         <is>
           <t>Besiktas</t>
         </is>
       </c>
-      <c r="E946" t="n">
-        <v>10.14</v>
-      </c>
-      <c r="F946" t="n">
-        <v>-0.47</v>
+      <c r="E947" t="n">
+        <v>10.15</v>
+      </c>
+      <c r="F947" t="n">
+        <v>-0.5600000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-10-20
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F947"/>
+  <dimension ref="A1:F953"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25048,6 +25048,162 @@
         <v>-0.5600000000000001</v>
       </c>
     </row>
+    <row r="948">
+      <c r="A948" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B948" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C948" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="D948" t="inlineStr">
+        <is>
+          <t>Borussia Monchengladbach</t>
+        </is>
+      </c>
+      <c r="E948" t="n">
+        <v>10.51</v>
+      </c>
+      <c r="F948" t="n">
+        <v>3.08</v>
+      </c>
+    </row>
+    <row r="949">
+      <c r="A949" s="1" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B949" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C949" t="inlineStr">
+        <is>
+          <t>Augsburg</t>
+        </is>
+      </c>
+      <c r="D949" t="inlineStr">
+        <is>
+          <t>Union Berlin</t>
+        </is>
+      </c>
+      <c r="E949" t="n">
+        <v>10.55</v>
+      </c>
+      <c r="F949" t="n">
+        <v>1.02</v>
+      </c>
+    </row>
+    <row r="950">
+      <c r="A950" s="1" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B950" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C950" t="inlineStr">
+        <is>
+          <t>Borussia Dortmund</t>
+        </is>
+      </c>
+      <c r="D950" t="inlineStr">
+        <is>
+          <t>Eintracht Frankfurt</t>
+        </is>
+      </c>
+      <c r="E950" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="F950" t="n">
+        <v>2.85</v>
+      </c>
+    </row>
+    <row r="951">
+      <c r="A951" s="1" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B951" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C951" t="inlineStr">
+        <is>
+          <t>Mainz 05</t>
+        </is>
+      </c>
+      <c r="D951" t="inlineStr">
+        <is>
+          <t>Werder Bremen</t>
+        </is>
+      </c>
+      <c r="E951" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="F951" t="n">
+        <v>2.08</v>
+      </c>
+    </row>
+    <row r="952">
+      <c r="A952" s="1" t="n">
+        <v>46320</v>
+      </c>
+      <c r="B952" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C952" t="inlineStr">
+        <is>
+          <t>Freiburg</t>
+        </is>
+      </c>
+      <c r="D952" t="inlineStr">
+        <is>
+          <t>Bayern Munich</t>
+        </is>
+      </c>
+      <c r="E952" t="n">
+        <v>9.869999999999999</v>
+      </c>
+      <c r="F952" t="n">
+        <v>-2.5</v>
+      </c>
+    </row>
+    <row r="953">
+      <c r="A953" s="1" t="n">
+        <v>46320</v>
+      </c>
+      <c r="B953" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C953" t="inlineStr">
+        <is>
+          <t>Hoffenheim</t>
+        </is>
+      </c>
+      <c r="D953" t="inlineStr">
+        <is>
+          <t>Bayer Leverkusen</t>
+        </is>
+      </c>
+      <c r="E953" t="n">
+        <v>10.75</v>
+      </c>
+      <c r="F953" t="n">
+        <v>0.06</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily scrape output - 2026-10-21
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -25120,10 +25120,10 @@
         </is>
       </c>
       <c r="E950" t="n">
-        <v>10.2</v>
+        <v>9.99</v>
       </c>
       <c r="F950" t="n">
-        <v>2.85</v>
+        <v>2.75</v>
       </c>
     </row>
     <row r="951">
@@ -25172,10 +25172,10 @@
         </is>
       </c>
       <c r="E952" t="n">
-        <v>9.869999999999999</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="F952" t="n">
-        <v>-2.5</v>
+        <v>-2.51</v>
       </c>
     </row>
     <row r="953">

</xml_diff>

<commit_message>
Daily scrape output - 2026-10-22
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F953"/>
+  <dimension ref="A1:F956"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25068,10 +25068,10 @@
         </is>
       </c>
       <c r="E948" t="n">
-        <v>10.51</v>
+        <v>10.53</v>
       </c>
       <c r="F948" t="n">
-        <v>3.08</v>
+        <v>3.48</v>
       </c>
     </row>
     <row r="949">
@@ -25137,24 +25137,24 @@
       </c>
       <c r="C951" t="inlineStr">
         <is>
-          <t>Mainz 05</t>
+          <t>FC Koln</t>
         </is>
       </c>
       <c r="D951" t="inlineStr">
         <is>
-          <t>Werder Bremen</t>
+          <t>Schalke 04</t>
         </is>
       </c>
       <c r="E951" t="n">
-        <v>9.800000000000001</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="F951" t="n">
-        <v>2.08</v>
+        <v>1.15</v>
       </c>
     </row>
     <row r="952">
       <c r="A952" s="1" t="n">
-        <v>46320</v>
+        <v>46319</v>
       </c>
       <c r="B952" t="inlineStr">
         <is>
@@ -25163,44 +25163,122 @@
       </c>
       <c r="C952" t="inlineStr">
         <is>
-          <t>Freiburg</t>
+          <t>Mainz 05</t>
         </is>
       </c>
       <c r="D952" t="inlineStr">
         <is>
-          <t>Bayern Munich</t>
+          <t>Werder Bremen</t>
         </is>
       </c>
       <c r="E952" t="n">
-        <v>9.859999999999999</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="F952" t="n">
-        <v>-2.51</v>
+        <v>2.08</v>
       </c>
     </row>
     <row r="953">
       <c r="A953" s="1" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B953" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C953" t="inlineStr">
+        <is>
+          <t>Paderborn</t>
+        </is>
+      </c>
+      <c r="D953" t="inlineStr">
+        <is>
+          <t>Hamburger SV</t>
+        </is>
+      </c>
+      <c r="E953" t="n">
+        <v>9.93</v>
+      </c>
+      <c r="F953" t="n">
+        <v>1.11</v>
+      </c>
+    </row>
+    <row r="954">
+      <c r="A954" s="1" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B954" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C954" t="inlineStr">
+        <is>
+          <t>RB Leipzig</t>
+        </is>
+      </c>
+      <c r="D954" t="inlineStr">
+        <is>
+          <t>Elversberg</t>
+        </is>
+      </c>
+      <c r="E954" t="n">
+        <v>10.53</v>
+      </c>
+      <c r="F954" t="n">
+        <v>3.13</v>
+      </c>
+    </row>
+    <row r="955">
+      <c r="A955" s="1" t="n">
         <v>46320</v>
       </c>
-      <c r="B953" t="inlineStr">
+      <c r="B955" t="inlineStr">
         <is>
           <t>Germany - Bundesliga</t>
         </is>
       </c>
-      <c r="C953" t="inlineStr">
+      <c r="C955" t="inlineStr">
+        <is>
+          <t>Freiburg</t>
+        </is>
+      </c>
+      <c r="D955" t="inlineStr">
+        <is>
+          <t>Bayern Munich</t>
+        </is>
+      </c>
+      <c r="E955" t="n">
+        <v>9.83</v>
+      </c>
+      <c r="F955" t="n">
+        <v>-2.5</v>
+      </c>
+    </row>
+    <row r="956">
+      <c r="A956" s="1" t="n">
+        <v>46320</v>
+      </c>
+      <c r="B956" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C956" t="inlineStr">
         <is>
           <t>Hoffenheim</t>
         </is>
       </c>
-      <c r="D953" t="inlineStr">
+      <c r="D956" t="inlineStr">
         <is>
           <t>Bayer Leverkusen</t>
         </is>
       </c>
-      <c r="E953" t="n">
+      <c r="E956" t="n">
         <v>10.75</v>
       </c>
-      <c r="F953" t="n">
+      <c r="F956" t="n">
         <v>0.06</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily scrape output - 2026-10-23
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F956"/>
+  <dimension ref="A1:F986"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25076,132 +25076,132 @@
     </row>
     <row r="949">
       <c r="A949" s="1" t="n">
-        <v>46319</v>
+        <v>46318</v>
       </c>
       <c r="B949" t="inlineStr">
         <is>
-          <t>Germany - Bundesliga</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C949" t="inlineStr">
         <is>
-          <t>Augsburg</t>
+          <t>Polonia Warsaw</t>
         </is>
       </c>
       <c r="D949" t="inlineStr">
         <is>
-          <t>Union Berlin</t>
+          <t>Miedz Legnica</t>
         </is>
       </c>
       <c r="E949" t="n">
-        <v>10.55</v>
+        <v>11.27</v>
       </c>
       <c r="F949" t="n">
-        <v>1.02</v>
+        <v>1.53</v>
       </c>
     </row>
     <row r="950">
       <c r="A950" s="1" t="n">
-        <v>46319</v>
+        <v>46318</v>
       </c>
       <c r="B950" t="inlineStr">
         <is>
-          <t>Germany - Bundesliga</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C950" t="inlineStr">
         <is>
-          <t>Borussia Dortmund</t>
+          <t>Motor Lublin</t>
         </is>
       </c>
       <c r="D950" t="inlineStr">
         <is>
-          <t>Eintracht Frankfurt</t>
+          <t>Zaglebie Lubin</t>
         </is>
       </c>
       <c r="E950" t="n">
-        <v>9.99</v>
+        <v>9.65</v>
       </c>
       <c r="F950" t="n">
-        <v>2.75</v>
+        <v>1.72</v>
       </c>
     </row>
     <row r="951">
       <c r="A951" s="1" t="n">
-        <v>46319</v>
+        <v>46318</v>
       </c>
       <c r="B951" t="inlineStr">
         <is>
-          <t>Germany - Bundesliga</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C951" t="inlineStr">
         <is>
-          <t>FC Koln</t>
+          <t>Widzew Lodz</t>
         </is>
       </c>
       <c r="D951" t="inlineStr">
         <is>
-          <t>Schalke 04</t>
+          <t>Gornik Zabrze</t>
         </is>
       </c>
       <c r="E951" t="n">
-        <v>9.880000000000001</v>
+        <v>9.539999999999999</v>
       </c>
       <c r="F951" t="n">
-        <v>1.15</v>
+        <v>-0.33</v>
       </c>
     </row>
     <row r="952">
       <c r="A952" s="1" t="n">
-        <v>46319</v>
+        <v>46318</v>
       </c>
       <c r="B952" t="inlineStr">
         <is>
-          <t>Germany - Bundesliga</t>
+          <t>Portugal - Primeira Liga</t>
         </is>
       </c>
       <c r="C952" t="inlineStr">
         <is>
-          <t>Mainz 05</t>
+          <t>Vitoria Guimaraes</t>
         </is>
       </c>
       <c r="D952" t="inlineStr">
         <is>
-          <t>Werder Bremen</t>
+          <t>Maritimo</t>
         </is>
       </c>
       <c r="E952" t="n">
-        <v>9.800000000000001</v>
+        <v>9</v>
       </c>
       <c r="F952" t="n">
-        <v>2.08</v>
+        <v>2.44</v>
       </c>
     </row>
     <row r="953">
       <c r="A953" s="1" t="n">
-        <v>46319</v>
+        <v>46318</v>
       </c>
       <c r="B953" t="inlineStr">
         <is>
-          <t>Germany - Bundesliga</t>
+          <t>Turkey - Super Lig</t>
         </is>
       </c>
       <c r="C953" t="inlineStr">
         <is>
-          <t>Paderborn</t>
+          <t>Alanyaspor</t>
         </is>
       </c>
       <c r="D953" t="inlineStr">
         <is>
-          <t>Hamburger SV</t>
+          <t>Kocaelispor</t>
         </is>
       </c>
       <c r="E953" t="n">
-        <v>9.93</v>
+        <v>8.6</v>
       </c>
       <c r="F953" t="n">
-        <v>1.11</v>
+        <v>1.53</v>
       </c>
     </row>
     <row r="954">
@@ -25215,24 +25215,24 @@
       </c>
       <c r="C954" t="inlineStr">
         <is>
-          <t>RB Leipzig</t>
+          <t>Augsburg</t>
         </is>
       </c>
       <c r="D954" t="inlineStr">
         <is>
-          <t>Elversberg</t>
+          <t>Union Berlin</t>
         </is>
       </c>
       <c r="E954" t="n">
-        <v>10.53</v>
+        <v>10.55</v>
       </c>
       <c r="F954" t="n">
-        <v>3.13</v>
+        <v>1.02</v>
       </c>
     </row>
     <row r="955">
       <c r="A955" s="1" t="n">
-        <v>46320</v>
+        <v>46319</v>
       </c>
       <c r="B955" t="inlineStr">
         <is>
@@ -25241,45 +25241,825 @@
       </c>
       <c r="C955" t="inlineStr">
         <is>
-          <t>Freiburg</t>
+          <t>Borussia Dortmund</t>
         </is>
       </c>
       <c r="D955" t="inlineStr">
         <is>
-          <t>Bayern Munich</t>
+          <t>Eintracht Frankfurt</t>
         </is>
       </c>
       <c r="E955" t="n">
-        <v>9.83</v>
+        <v>9.93</v>
       </c>
       <c r="F955" t="n">
-        <v>-2.5</v>
+        <v>2.75</v>
       </c>
     </row>
     <row r="956">
       <c r="A956" s="1" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B956" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C956" t="inlineStr">
+        <is>
+          <t>FC Koln</t>
+        </is>
+      </c>
+      <c r="D956" t="inlineStr">
+        <is>
+          <t>Schalke 04</t>
+        </is>
+      </c>
+      <c r="E956" t="n">
+        <v>9.880000000000001</v>
+      </c>
+      <c r="F956" t="n">
+        <v>1.15</v>
+      </c>
+    </row>
+    <row r="957">
+      <c r="A957" s="1" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B957" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C957" t="inlineStr">
+        <is>
+          <t>Mainz 05</t>
+        </is>
+      </c>
+      <c r="D957" t="inlineStr">
+        <is>
+          <t>Werder Bremen</t>
+        </is>
+      </c>
+      <c r="E957" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="F957" t="n">
+        <v>2.08</v>
+      </c>
+    </row>
+    <row r="958">
+      <c r="A958" s="1" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B958" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C958" t="inlineStr">
+        <is>
+          <t>Paderborn</t>
+        </is>
+      </c>
+      <c r="D958" t="inlineStr">
+        <is>
+          <t>Hamburger SV</t>
+        </is>
+      </c>
+      <c r="E958" t="n">
+        <v>9.93</v>
+      </c>
+      <c r="F958" t="n">
+        <v>1.11</v>
+      </c>
+    </row>
+    <row r="959">
+      <c r="A959" s="1" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B959" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C959" t="inlineStr">
+        <is>
+          <t>RB Leipzig</t>
+        </is>
+      </c>
+      <c r="D959" t="inlineStr">
+        <is>
+          <t>Elversberg</t>
+        </is>
+      </c>
+      <c r="E959" t="n">
+        <v>10.53</v>
+      </c>
+      <c r="F959" t="n">
+        <v>3.13</v>
+      </c>
+    </row>
+    <row r="960">
+      <c r="A960" s="1" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B960" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C960" t="inlineStr">
+        <is>
+          <t>Arka Gdynia</t>
+        </is>
+      </c>
+      <c r="D960" t="inlineStr">
+        <is>
+          <t>Nieciecza</t>
+        </is>
+      </c>
+      <c r="E960" t="n">
+        <v>10.52</v>
+      </c>
+      <c r="F960" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="961">
+      <c r="A961" s="1" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B961" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C961" t="inlineStr">
+        <is>
+          <t>Puszcza Niepolomice</t>
+        </is>
+      </c>
+      <c r="D961" t="inlineStr">
+        <is>
+          <t>Lechia Gdansk</t>
+        </is>
+      </c>
+      <c r="E961" t="n">
+        <v>10.49</v>
+      </c>
+      <c r="F961" t="n">
+        <v>-0.36</v>
+      </c>
+    </row>
+    <row r="962">
+      <c r="A962" s="1" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B962" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C962" t="inlineStr">
+        <is>
+          <t>Stal Mielec</t>
+        </is>
+      </c>
+      <c r="D962" t="inlineStr">
+        <is>
+          <t>Chrobry Glogow</t>
+        </is>
+      </c>
+      <c r="E962" t="n">
+        <v>10.36</v>
+      </c>
+      <c r="F962" t="n">
+        <v>0.83</v>
+      </c>
+    </row>
+    <row r="963">
+      <c r="A963" s="1" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B963" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C963" t="inlineStr">
+        <is>
+          <t>Unia Skierniewice</t>
+        </is>
+      </c>
+      <c r="D963" t="inlineStr">
+        <is>
+          <t>Polonia Bytom</t>
+        </is>
+      </c>
+      <c r="E963" t="n">
+        <v>10.47</v>
+      </c>
+      <c r="F963" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="964">
+      <c r="A964" s="1" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B964" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C964" t="inlineStr">
+        <is>
+          <t>Korona Kielce</t>
+        </is>
+      </c>
+      <c r="D964" t="inlineStr">
+        <is>
+          <t>GKS Katowice</t>
+        </is>
+      </c>
+      <c r="E964" t="n">
+        <v>10.11</v>
+      </c>
+      <c r="F964" t="n">
+        <v>1.02</v>
+      </c>
+    </row>
+    <row r="965">
+      <c r="A965" s="1" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B965" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C965" t="inlineStr">
+        <is>
+          <t>Piast Gliwice</t>
+        </is>
+      </c>
+      <c r="D965" t="inlineStr">
+        <is>
+          <t>Cracovia Krakow</t>
+        </is>
+      </c>
+      <c r="E965" t="n">
+        <v>10.05</v>
+      </c>
+      <c r="F965" t="n">
+        <v>-0.02</v>
+      </c>
+    </row>
+    <row r="966">
+      <c r="A966" s="1" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B966" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C966" t="inlineStr">
+        <is>
+          <t>Pogon Szczecin</t>
+        </is>
+      </c>
+      <c r="D966" t="inlineStr">
+        <is>
+          <t>Radomiak Radom</t>
+        </is>
+      </c>
+      <c r="E966" t="n">
+        <v>10.28</v>
+      </c>
+      <c r="F966" t="n">
+        <v>1.41</v>
+      </c>
+    </row>
+    <row r="967">
+      <c r="A967" s="1" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B967" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C967" t="inlineStr">
+        <is>
+          <t>Wisla Krakow</t>
+        </is>
+      </c>
+      <c r="D967" t="inlineStr">
+        <is>
+          <t>Rakow Czestochowa</t>
+        </is>
+      </c>
+      <c r="E967" t="n">
+        <v>10.38</v>
+      </c>
+      <c r="F967" t="n">
+        <v>1.48</v>
+      </c>
+    </row>
+    <row r="968">
+      <c r="A968" s="1" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B968" t="inlineStr">
+        <is>
+          <t>Portugal - Primeira Liga</t>
+        </is>
+      </c>
+      <c r="C968" t="inlineStr">
+        <is>
+          <t>Alverca</t>
+        </is>
+      </c>
+      <c r="D968" t="inlineStr">
+        <is>
+          <t>Arouca</t>
+        </is>
+      </c>
+      <c r="E968" t="n">
+        <v>9.359999999999999</v>
+      </c>
+      <c r="F968" t="n">
+        <v>1.45</v>
+      </c>
+    </row>
+    <row r="969">
+      <c r="A969" s="1" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B969" t="inlineStr">
+        <is>
+          <t>Portugal - Primeira Liga</t>
+        </is>
+      </c>
+      <c r="C969" t="inlineStr">
+        <is>
+          <t>Estrela da Amadora</t>
+        </is>
+      </c>
+      <c r="D969" t="inlineStr">
+        <is>
+          <t>Casa Pia</t>
+        </is>
+      </c>
+      <c r="E969" t="n">
+        <v>9.56</v>
+      </c>
+      <c r="F969" t="n">
+        <v>1.21</v>
+      </c>
+    </row>
+    <row r="970">
+      <c r="A970" s="1" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B970" t="inlineStr">
+        <is>
+          <t>Portugal - Primeira Liga</t>
+        </is>
+      </c>
+      <c r="C970" t="inlineStr">
+        <is>
+          <t>Gil Vicente</t>
+        </is>
+      </c>
+      <c r="D970" t="inlineStr">
+        <is>
+          <t>Porto</t>
+        </is>
+      </c>
+      <c r="E970" t="n">
+        <v>9.07</v>
+      </c>
+      <c r="F970" t="n">
+        <v>-1.54</v>
+      </c>
+    </row>
+    <row r="971">
+      <c r="A971" s="1" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B971" t="inlineStr">
+        <is>
+          <t>Turkey - Super Lig</t>
+        </is>
+      </c>
+      <c r="C971" t="inlineStr">
+        <is>
+          <t>Eyupspor</t>
+        </is>
+      </c>
+      <c r="D971" t="inlineStr">
+        <is>
+          <t>Kasimpasa</t>
+        </is>
+      </c>
+      <c r="E971" t="n">
+        <v>9.33</v>
+      </c>
+      <c r="F971" t="n">
+        <v>-0.6</v>
+      </c>
+    </row>
+    <row r="972">
+      <c r="A972" s="1" t="n">
         <v>46320</v>
       </c>
-      <c r="B956" t="inlineStr">
+      <c r="B972" t="inlineStr">
         <is>
           <t>Germany - Bundesliga</t>
         </is>
       </c>
-      <c r="C956" t="inlineStr">
+      <c r="C972" t="inlineStr">
+        <is>
+          <t>Freiburg</t>
+        </is>
+      </c>
+      <c r="D972" t="inlineStr">
+        <is>
+          <t>Bayern Munich</t>
+        </is>
+      </c>
+      <c r="E972" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="F972" t="n">
+        <v>-2.51</v>
+      </c>
+    </row>
+    <row r="973">
+      <c r="A973" s="1" t="n">
+        <v>46320</v>
+      </c>
+      <c r="B973" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C973" t="inlineStr">
         <is>
           <t>Hoffenheim</t>
         </is>
       </c>
-      <c r="D956" t="inlineStr">
+      <c r="D973" t="inlineStr">
         <is>
           <t>Bayer Leverkusen</t>
         </is>
       </c>
-      <c r="E956" t="n">
-        <v>10.75</v>
-      </c>
-      <c r="F956" t="n">
-        <v>0.06</v>
+      <c r="E973" t="n">
+        <v>10.76</v>
+      </c>
+      <c r="F973" t="n">
+        <v>-0.04</v>
+      </c>
+    </row>
+    <row r="974">
+      <c r="A974" s="1" t="n">
+        <v>46320</v>
+      </c>
+      <c r="B974" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C974" t="inlineStr">
+        <is>
+          <t>Odra Opole</t>
+        </is>
+      </c>
+      <c r="D974" t="inlineStr">
+        <is>
+          <t>Pogon Siedlce</t>
+        </is>
+      </c>
+      <c r="E974" t="n">
+        <v>10.27</v>
+      </c>
+      <c r="F974" t="n">
+        <v>1.89</v>
+      </c>
+    </row>
+    <row r="975">
+      <c r="A975" s="1" t="n">
+        <v>46320</v>
+      </c>
+      <c r="B975" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C975" t="inlineStr">
+        <is>
+          <t>Podbeskidzie Bielsko-Biala</t>
+        </is>
+      </c>
+      <c r="D975" t="inlineStr">
+        <is>
+          <t>Stal Rzeszow</t>
+        </is>
+      </c>
+      <c r="E975" t="n">
+        <v>10.66</v>
+      </c>
+      <c r="F975" t="n">
+        <v>1.09</v>
+      </c>
+    </row>
+    <row r="976">
+      <c r="A976" s="1" t="n">
+        <v>46320</v>
+      </c>
+      <c r="B976" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C976" t="inlineStr">
+        <is>
+          <t>Ruch Chorzow</t>
+        </is>
+      </c>
+      <c r="D976" t="inlineStr">
+        <is>
+          <t>Pogon Grodzisk Mazowiecki</t>
+        </is>
+      </c>
+      <c r="E976" t="n">
+        <v>10.82</v>
+      </c>
+      <c r="F976" t="n">
+        <v>2.09</v>
+      </c>
+    </row>
+    <row r="977">
+      <c r="A977" s="1" t="n">
+        <v>46320</v>
+      </c>
+      <c r="B977" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C977" t="inlineStr">
+        <is>
+          <t>Jagiellonia Bialystok</t>
+        </is>
+      </c>
+      <c r="D977" t="inlineStr">
+        <is>
+          <t>Wisla Plock</t>
+        </is>
+      </c>
+      <c r="E977" t="n">
+        <v>10.11</v>
+      </c>
+      <c r="F977" t="n">
+        <v>1.42</v>
+      </c>
+    </row>
+    <row r="978">
+      <c r="A978" s="1" t="n">
+        <v>46320</v>
+      </c>
+      <c r="B978" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C978" t="inlineStr">
+        <is>
+          <t>Legia Warsaw</t>
+        </is>
+      </c>
+      <c r="D978" t="inlineStr">
+        <is>
+          <t>Lech Poznan</t>
+        </is>
+      </c>
+      <c r="E978" t="n">
+        <v>10.16</v>
+      </c>
+      <c r="F978" t="n">
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="979">
+      <c r="A979" s="1" t="n">
+        <v>46320</v>
+      </c>
+      <c r="B979" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C979" t="inlineStr">
+        <is>
+          <t>Slask Wroclaw</t>
+        </is>
+      </c>
+      <c r="D979" t="inlineStr">
+        <is>
+          <t>Wieczysta Krakow</t>
+        </is>
+      </c>
+      <c r="E979" t="n">
+        <v>10.45</v>
+      </c>
+      <c r="F979" t="n">
+        <v>-0.19</v>
+      </c>
+    </row>
+    <row r="980">
+      <c r="A980" s="1" t="n">
+        <v>46320</v>
+      </c>
+      <c r="B980" t="inlineStr">
+        <is>
+          <t>Portugal - Primeira Liga</t>
+        </is>
+      </c>
+      <c r="C980" t="inlineStr">
+        <is>
+          <t>Estoril</t>
+        </is>
+      </c>
+      <c r="D980" t="inlineStr">
+        <is>
+          <t>Moreirense</t>
+        </is>
+      </c>
+      <c r="E980" t="n">
+        <v>9.25</v>
+      </c>
+      <c r="F980" t="n">
+        <v>1.71</v>
+      </c>
+    </row>
+    <row r="981">
+      <c r="A981" s="1" t="n">
+        <v>46320</v>
+      </c>
+      <c r="B981" t="inlineStr">
+        <is>
+          <t>Portugal - Primeira Liga</t>
+        </is>
+      </c>
+      <c r="C981" t="inlineStr">
+        <is>
+          <t>Nacional da Madeira</t>
+        </is>
+      </c>
+      <c r="D981" t="inlineStr">
+        <is>
+          <t>Braga</t>
+        </is>
+      </c>
+      <c r="E981" t="n">
+        <v>9.32</v>
+      </c>
+      <c r="F981" t="n">
+        <v>-1.88</v>
+      </c>
+    </row>
+    <row r="982">
+      <c r="A982" s="1" t="n">
+        <v>46320</v>
+      </c>
+      <c r="B982" t="inlineStr">
+        <is>
+          <t>Portugal - Primeira Liga</t>
+        </is>
+      </c>
+      <c r="C982" t="inlineStr">
+        <is>
+          <t>Rio Ave</t>
+        </is>
+      </c>
+      <c r="D982" t="inlineStr">
+        <is>
+          <t>Famalicao</t>
+        </is>
+      </c>
+      <c r="E982" t="n">
+        <v>9.949999999999999</v>
+      </c>
+      <c r="F982" t="n">
+        <v>-1.21</v>
+      </c>
+    </row>
+    <row r="983">
+      <c r="A983" s="1" t="n">
+        <v>46320</v>
+      </c>
+      <c r="B983" t="inlineStr">
+        <is>
+          <t>Turkey - Super Lig</t>
+        </is>
+      </c>
+      <c r="C983" t="inlineStr">
+        <is>
+          <t>Konyaspor</t>
+        </is>
+      </c>
+      <c r="D983" t="inlineStr">
+        <is>
+          <t>Genclerbirligi</t>
+        </is>
+      </c>
+      <c r="E983" t="n">
+        <v>9.720000000000001</v>
+      </c>
+      <c r="F983" t="n">
+        <v>1.16</v>
+      </c>
+    </row>
+    <row r="984">
+      <c r="A984" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B984" t="inlineStr">
+        <is>
+          <t>Turkey - Super Lig</t>
+        </is>
+      </c>
+      <c r="C984" t="inlineStr">
+        <is>
+          <t>Besiktas</t>
+        </is>
+      </c>
+      <c r="D984" t="inlineStr">
+        <is>
+          <t>Istanbul Basaksehir</t>
+        </is>
+      </c>
+      <c r="E984" t="n">
+        <v>10.22</v>
+      </c>
+      <c r="F984" t="n">
+        <v>2.88</v>
+      </c>
+    </row>
+    <row r="985">
+      <c r="A985" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B985" t="inlineStr">
+        <is>
+          <t>Turkey - Super Lig</t>
+        </is>
+      </c>
+      <c r="C985" t="inlineStr">
+        <is>
+          <t>Caykur Rizespor</t>
+        </is>
+      </c>
+      <c r="D985" t="inlineStr">
+        <is>
+          <t>Trabzonspor</t>
+        </is>
+      </c>
+      <c r="E985" t="n">
+        <v>9.710000000000001</v>
+      </c>
+      <c r="F985" t="n">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="986">
+      <c r="A986" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B986" t="inlineStr">
+        <is>
+          <t>Turkey - Super Lig</t>
+        </is>
+      </c>
+      <c r="C986" t="inlineStr">
+        <is>
+          <t>Galatasaray</t>
+        </is>
+      </c>
+      <c r="D986" t="inlineStr">
+        <is>
+          <t>Fenerbahce</t>
+        </is>
+      </c>
+      <c r="E986" t="n">
+        <v>9.960000000000001</v>
+      </c>
+      <c r="F986" t="n">
+        <v>0.92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-10-24
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F986"/>
+  <dimension ref="A1:F988"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25224,10 +25224,10 @@
         </is>
       </c>
       <c r="E954" t="n">
-        <v>10.55</v>
+        <v>10.57</v>
       </c>
       <c r="F954" t="n">
-        <v>1.02</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="955">
@@ -25250,10 +25250,10 @@
         </is>
       </c>
       <c r="E955" t="n">
-        <v>9.93</v>
+        <v>9.94</v>
       </c>
       <c r="F955" t="n">
-        <v>2.75</v>
+        <v>2.74</v>
       </c>
     </row>
     <row r="956">
@@ -25276,10 +25276,10 @@
         </is>
       </c>
       <c r="E956" t="n">
-        <v>9.880000000000001</v>
+        <v>9.75</v>
       </c>
       <c r="F956" t="n">
-        <v>1.15</v>
+        <v>1.18</v>
       </c>
     </row>
     <row r="957">
@@ -25302,10 +25302,10 @@
         </is>
       </c>
       <c r="E957" t="n">
-        <v>9.800000000000001</v>
+        <v>9.59</v>
       </c>
       <c r="F957" t="n">
-        <v>2.08</v>
+        <v>2.07</v>
       </c>
     </row>
     <row r="958">
@@ -25328,10 +25328,10 @@
         </is>
       </c>
       <c r="E958" t="n">
-        <v>9.93</v>
+        <v>9.9</v>
       </c>
       <c r="F958" t="n">
-        <v>1.11</v>
+        <v>1.14</v>
       </c>
     </row>
     <row r="959">
@@ -25354,10 +25354,10 @@
         </is>
       </c>
       <c r="E959" t="n">
-        <v>10.53</v>
+        <v>10.61</v>
       </c>
       <c r="F959" t="n">
-        <v>3.13</v>
+        <v>3.15</v>
       </c>
     </row>
     <row r="960">
@@ -25380,10 +25380,10 @@
         </is>
       </c>
       <c r="E960" t="n">
-        <v>10.52</v>
+        <v>10.53</v>
       </c>
       <c r="F960" t="n">
-        <v>1</v>
+        <v>0.89</v>
       </c>
     </row>
     <row r="961">
@@ -25406,10 +25406,10 @@
         </is>
       </c>
       <c r="E961" t="n">
-        <v>10.49</v>
+        <v>10.22</v>
       </c>
       <c r="F961" t="n">
-        <v>-0.36</v>
+        <v>-0.34</v>
       </c>
     </row>
     <row r="962">
@@ -25432,10 +25432,10 @@
         </is>
       </c>
       <c r="E962" t="n">
-        <v>10.36</v>
+        <v>10.24</v>
       </c>
       <c r="F962" t="n">
-        <v>0.83</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="963">
@@ -25458,10 +25458,10 @@
         </is>
       </c>
       <c r="E963" t="n">
-        <v>10.47</v>
+        <v>10.3</v>
       </c>
       <c r="F963" t="n">
-        <v>0.4</v>
+        <v>-0.46</v>
       </c>
     </row>
     <row r="964">
@@ -25510,10 +25510,10 @@
         </is>
       </c>
       <c r="E965" t="n">
-        <v>10.05</v>
+        <v>9.85</v>
       </c>
       <c r="F965" t="n">
-        <v>-0.02</v>
+        <v>0</v>
       </c>
     </row>
     <row r="966">
@@ -25536,7 +25536,7 @@
         </is>
       </c>
       <c r="E966" t="n">
-        <v>10.28</v>
+        <v>10.3</v>
       </c>
       <c r="F966" t="n">
         <v>1.41</v>
@@ -25562,7 +25562,7 @@
         </is>
       </c>
       <c r="E967" t="n">
-        <v>10.38</v>
+        <v>10.16</v>
       </c>
       <c r="F967" t="n">
         <v>1.48</v>
@@ -25588,10 +25588,10 @@
         </is>
       </c>
       <c r="E968" t="n">
-        <v>9.359999999999999</v>
+        <v>9.35</v>
       </c>
       <c r="F968" t="n">
-        <v>1.45</v>
+        <v>1.46</v>
       </c>
     </row>
     <row r="969">
@@ -25614,7 +25614,7 @@
         </is>
       </c>
       <c r="E969" t="n">
-        <v>9.56</v>
+        <v>9.6</v>
       </c>
       <c r="F969" t="n">
         <v>1.21</v>
@@ -25640,10 +25640,10 @@
         </is>
       </c>
       <c r="E970" t="n">
-        <v>9.07</v>
+        <v>9.109999999999999</v>
       </c>
       <c r="F970" t="n">
-        <v>-1.54</v>
+        <v>-2.02</v>
       </c>
     </row>
     <row r="971">
@@ -25666,62 +25666,62 @@
         </is>
       </c>
       <c r="E971" t="n">
-        <v>9.33</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="F971" t="n">
-        <v>-0.6</v>
+        <v>-0.89</v>
       </c>
     </row>
     <row r="972">
       <c r="A972" s="1" t="n">
-        <v>46320</v>
+        <v>46319</v>
       </c>
       <c r="B972" t="inlineStr">
         <is>
-          <t>Germany - Bundesliga</t>
+          <t>Turkey - Super Lig</t>
         </is>
       </c>
       <c r="C972" t="inlineStr">
         <is>
-          <t>Freiburg</t>
+          <t>Gaziantep</t>
         </is>
       </c>
       <c r="D972" t="inlineStr">
         <is>
-          <t>Bayern Munich</t>
+          <t>Erzurumspor</t>
         </is>
       </c>
       <c r="E972" t="n">
-        <v>9.800000000000001</v>
+        <v>9.02</v>
       </c>
       <c r="F972" t="n">
-        <v>-2.51</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="973">
       <c r="A973" s="1" t="n">
-        <v>46320</v>
+        <v>46319</v>
       </c>
       <c r="B973" t="inlineStr">
         <is>
-          <t>Germany - Bundesliga</t>
+          <t>Turkey - Super Lig</t>
         </is>
       </c>
       <c r="C973" t="inlineStr">
         <is>
-          <t>Hoffenheim</t>
+          <t>Samsunspor</t>
         </is>
       </c>
       <c r="D973" t="inlineStr">
         <is>
-          <t>Bayer Leverkusen</t>
+          <t>Amedspor</t>
         </is>
       </c>
       <c r="E973" t="n">
-        <v>10.76</v>
+        <v>9.33</v>
       </c>
       <c r="F973" t="n">
-        <v>-0.04</v>
+        <v>-0.13</v>
       </c>
     </row>
     <row r="974">
@@ -25730,24 +25730,24 @@
       </c>
       <c r="B974" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Germany - Bundesliga</t>
         </is>
       </c>
       <c r="C974" t="inlineStr">
         <is>
-          <t>Odra Opole</t>
+          <t>Freiburg</t>
         </is>
       </c>
       <c r="D974" t="inlineStr">
         <is>
-          <t>Pogon Siedlce</t>
+          <t>Bayern Munich</t>
         </is>
       </c>
       <c r="E974" t="n">
-        <v>10.27</v>
+        <v>9.84</v>
       </c>
       <c r="F974" t="n">
-        <v>1.89</v>
+        <v>-2.72</v>
       </c>
     </row>
     <row r="975">
@@ -25756,24 +25756,24 @@
       </c>
       <c r="B975" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Germany - Bundesliga</t>
         </is>
       </c>
       <c r="C975" t="inlineStr">
         <is>
-          <t>Podbeskidzie Bielsko-Biala</t>
+          <t>Hoffenheim</t>
         </is>
       </c>
       <c r="D975" t="inlineStr">
         <is>
-          <t>Stal Rzeszow</t>
+          <t>Bayer Leverkusen</t>
         </is>
       </c>
       <c r="E975" t="n">
-        <v>10.66</v>
+        <v>10.06</v>
       </c>
       <c r="F975" t="n">
-        <v>1.09</v>
+        <v>0</v>
       </c>
     </row>
     <row r="976">
@@ -25787,19 +25787,19 @@
       </c>
       <c r="C976" t="inlineStr">
         <is>
-          <t>Ruch Chorzow</t>
+          <t>Odra Opole</t>
         </is>
       </c>
       <c r="D976" t="inlineStr">
         <is>
-          <t>Pogon Grodzisk Mazowiecki</t>
+          <t>Pogon Siedlce</t>
         </is>
       </c>
       <c r="E976" t="n">
-        <v>10.82</v>
+        <v>10.27</v>
       </c>
       <c r="F976" t="n">
-        <v>2.09</v>
+        <v>1.89</v>
       </c>
     </row>
     <row r="977">
@@ -25808,24 +25808,24 @@
       </c>
       <c r="B977" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C977" t="inlineStr">
         <is>
-          <t>Jagiellonia Bialystok</t>
+          <t>Podbeskidzie Bielsko-Biala</t>
         </is>
       </c>
       <c r="D977" t="inlineStr">
         <is>
-          <t>Wisla Plock</t>
+          <t>Stal Rzeszow</t>
         </is>
       </c>
       <c r="E977" t="n">
-        <v>10.11</v>
+        <v>10.66</v>
       </c>
       <c r="F977" t="n">
-        <v>1.42</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="978">
@@ -25834,24 +25834,24 @@
       </c>
       <c r="B978" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C978" t="inlineStr">
         <is>
-          <t>Legia Warsaw</t>
+          <t>Ruch Chorzow</t>
         </is>
       </c>
       <c r="D978" t="inlineStr">
         <is>
-          <t>Lech Poznan</t>
+          <t>Pogon Grodzisk Mazowiecki</t>
         </is>
       </c>
       <c r="E978" t="n">
-        <v>10.16</v>
+        <v>10.82</v>
       </c>
       <c r="F978" t="n">
-        <v>0.51</v>
+        <v>2.09</v>
       </c>
     </row>
     <row r="979">
@@ -25865,19 +25865,19 @@
       </c>
       <c r="C979" t="inlineStr">
         <is>
-          <t>Slask Wroclaw</t>
+          <t>Jagiellonia Bialystok</t>
         </is>
       </c>
       <c r="D979" t="inlineStr">
         <is>
-          <t>Wieczysta Krakow</t>
+          <t>Wisla Plock</t>
         </is>
       </c>
       <c r="E979" t="n">
-        <v>10.45</v>
+        <v>9.84</v>
       </c>
       <c r="F979" t="n">
-        <v>-0.19</v>
+        <v>1.43</v>
       </c>
     </row>
     <row r="980">
@@ -25886,24 +25886,24 @@
       </c>
       <c r="B980" t="inlineStr">
         <is>
-          <t>Portugal - Primeira Liga</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C980" t="inlineStr">
         <is>
-          <t>Estoril</t>
+          <t>Legia Warsaw</t>
         </is>
       </c>
       <c r="D980" t="inlineStr">
         <is>
-          <t>Moreirense</t>
+          <t>Lech Poznan</t>
         </is>
       </c>
       <c r="E980" t="n">
-        <v>9.25</v>
+        <v>9.869999999999999</v>
       </c>
       <c r="F980" t="n">
-        <v>1.71</v>
+        <v>0.53</v>
       </c>
     </row>
     <row r="981">
@@ -25912,24 +25912,24 @@
       </c>
       <c r="B981" t="inlineStr">
         <is>
-          <t>Portugal - Primeira Liga</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C981" t="inlineStr">
         <is>
-          <t>Nacional da Madeira</t>
+          <t>Slask Wroclaw</t>
         </is>
       </c>
       <c r="D981" t="inlineStr">
         <is>
-          <t>Braga</t>
+          <t>Wieczysta Krakow</t>
         </is>
       </c>
       <c r="E981" t="n">
-        <v>9.32</v>
+        <v>10.45</v>
       </c>
       <c r="F981" t="n">
-        <v>-1.88</v>
+        <v>-0.19</v>
       </c>
     </row>
     <row r="982">
@@ -25943,19 +25943,19 @@
       </c>
       <c r="C982" t="inlineStr">
         <is>
-          <t>Rio Ave</t>
+          <t>Estoril</t>
         </is>
       </c>
       <c r="D982" t="inlineStr">
         <is>
-          <t>Famalicao</t>
+          <t>Moreirense</t>
         </is>
       </c>
       <c r="E982" t="n">
-        <v>9.949999999999999</v>
+        <v>9.25</v>
       </c>
       <c r="F982" t="n">
-        <v>-1.21</v>
+        <v>1.71</v>
       </c>
     </row>
     <row r="983">
@@ -25964,55 +25964,55 @@
       </c>
       <c r="B983" t="inlineStr">
         <is>
-          <t>Turkey - Super Lig</t>
+          <t>Portugal - Primeira Liga</t>
         </is>
       </c>
       <c r="C983" t="inlineStr">
         <is>
-          <t>Konyaspor</t>
+          <t>Nacional da Madeira</t>
         </is>
       </c>
       <c r="D983" t="inlineStr">
         <is>
-          <t>Genclerbirligi</t>
+          <t>Braga</t>
         </is>
       </c>
       <c r="E983" t="n">
-        <v>9.720000000000001</v>
+        <v>9.32</v>
       </c>
       <c r="F983" t="n">
-        <v>1.16</v>
+        <v>-1.88</v>
       </c>
     </row>
     <row r="984">
       <c r="A984" s="1" t="n">
-        <v>46321</v>
+        <v>46320</v>
       </c>
       <c r="B984" t="inlineStr">
         <is>
-          <t>Turkey - Super Lig</t>
+          <t>Portugal - Primeira Liga</t>
         </is>
       </c>
       <c r="C984" t="inlineStr">
         <is>
-          <t>Besiktas</t>
+          <t>Rio Ave</t>
         </is>
       </c>
       <c r="D984" t="inlineStr">
         <is>
-          <t>Istanbul Basaksehir</t>
+          <t>Famalicao</t>
         </is>
       </c>
       <c r="E984" t="n">
-        <v>10.22</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="F984" t="n">
-        <v>2.88</v>
+        <v>-1.21</v>
       </c>
     </row>
     <row r="985">
       <c r="A985" s="1" t="n">
-        <v>46321</v>
+        <v>46320</v>
       </c>
       <c r="B985" t="inlineStr">
         <is>
@@ -26021,19 +26021,19 @@
       </c>
       <c r="C985" t="inlineStr">
         <is>
-          <t>Caykur Rizespor</t>
+          <t>Konyaspor</t>
         </is>
       </c>
       <c r="D985" t="inlineStr">
         <is>
-          <t>Trabzonspor</t>
+          <t>Genclerbirligi</t>
         </is>
       </c>
       <c r="E985" t="n">
-        <v>9.710000000000001</v>
+        <v>9.550000000000001</v>
       </c>
       <c r="F985" t="n">
-        <v>0.32</v>
+        <v>1.17</v>
       </c>
     </row>
     <row r="986">
@@ -26047,18 +26047,70 @@
       </c>
       <c r="C986" t="inlineStr">
         <is>
+          <t>Besiktas</t>
+        </is>
+      </c>
+      <c r="D986" t="inlineStr">
+        <is>
+          <t>Istanbul Basaksehir</t>
+        </is>
+      </c>
+      <c r="E986" t="n">
+        <v>10.22</v>
+      </c>
+      <c r="F986" t="n">
+        <v>2.88</v>
+      </c>
+    </row>
+    <row r="987">
+      <c r="A987" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B987" t="inlineStr">
+        <is>
+          <t>Turkey - Super Lig</t>
+        </is>
+      </c>
+      <c r="C987" t="inlineStr">
+        <is>
+          <t>Caykur Rizespor</t>
+        </is>
+      </c>
+      <c r="D987" t="inlineStr">
+        <is>
+          <t>Trabzonspor</t>
+        </is>
+      </c>
+      <c r="E987" t="n">
+        <v>9.73</v>
+      </c>
+      <c r="F987" t="n">
+        <v>0.19</v>
+      </c>
+    </row>
+    <row r="988">
+      <c r="A988" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B988" t="inlineStr">
+        <is>
+          <t>Turkey - Super Lig</t>
+        </is>
+      </c>
+      <c r="C988" t="inlineStr">
+        <is>
           <t>Galatasaray</t>
         </is>
       </c>
-      <c r="D986" t="inlineStr">
+      <c r="D988" t="inlineStr">
         <is>
           <t>Fenerbahce</t>
         </is>
       </c>
-      <c r="E986" t="n">
+      <c r="E988" t="n">
         <v>9.960000000000001</v>
       </c>
-      <c r="F986" t="n">
+      <c r="F988" t="n">
         <v>0.92</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily scrape output - 2026-10-25
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F988"/>
+  <dimension ref="A1:F990"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25744,10 +25744,10 @@
         </is>
       </c>
       <c r="E974" t="n">
-        <v>9.84</v>
+        <v>9.83</v>
       </c>
       <c r="F974" t="n">
-        <v>-2.72</v>
+        <v>-2.88</v>
       </c>
     </row>
     <row r="975">
@@ -25770,10 +25770,10 @@
         </is>
       </c>
       <c r="E975" t="n">
-        <v>10.06</v>
+        <v>10.07</v>
       </c>
       <c r="F975" t="n">
-        <v>0</v>
+        <v>-0.03</v>
       </c>
     </row>
     <row r="976">
@@ -25796,10 +25796,10 @@
         </is>
       </c>
       <c r="E976" t="n">
-        <v>10.27</v>
+        <v>10.28</v>
       </c>
       <c r="F976" t="n">
-        <v>1.89</v>
+        <v>1.96</v>
       </c>
     </row>
     <row r="977">
@@ -25926,10 +25926,10 @@
         </is>
       </c>
       <c r="E981" t="n">
-        <v>10.45</v>
+        <v>10.31</v>
       </c>
       <c r="F981" t="n">
-        <v>-0.19</v>
+        <v>-0.54</v>
       </c>
     </row>
     <row r="982">
@@ -25952,7 +25952,7 @@
         </is>
       </c>
       <c r="E982" t="n">
-        <v>9.25</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="F982" t="n">
         <v>1.71</v>
@@ -25978,10 +25978,10 @@
         </is>
       </c>
       <c r="E983" t="n">
-        <v>9.32</v>
+        <v>9.359999999999999</v>
       </c>
       <c r="F983" t="n">
-        <v>-1.88</v>
+        <v>-2.26</v>
       </c>
     </row>
     <row r="984">
@@ -26004,7 +26004,7 @@
         </is>
       </c>
       <c r="E984" t="n">
-        <v>9.949999999999999</v>
+        <v>9.99</v>
       </c>
       <c r="F984" t="n">
         <v>-1.21</v>
@@ -26016,29 +26016,29 @@
       </c>
       <c r="B985" t="inlineStr">
         <is>
-          <t>Turkey - Super Lig</t>
+          <t>Portugal - Primeira Liga</t>
         </is>
       </c>
       <c r="C985" t="inlineStr">
         <is>
-          <t>Konyaspor</t>
+          <t>Sporting CP</t>
         </is>
       </c>
       <c r="D985" t="inlineStr">
         <is>
-          <t>Genclerbirligi</t>
+          <t>Academico de Viseu</t>
         </is>
       </c>
       <c r="E985" t="n">
-        <v>9.550000000000001</v>
+        <v>9.640000000000001</v>
       </c>
       <c r="F985" t="n">
-        <v>1.17</v>
+        <v>4.45</v>
       </c>
     </row>
     <row r="986">
       <c r="A986" s="1" t="n">
-        <v>46321</v>
+        <v>46320</v>
       </c>
       <c r="B986" t="inlineStr">
         <is>
@@ -26047,24 +26047,24 @@
       </c>
       <c r="C986" t="inlineStr">
         <is>
-          <t>Besiktas</t>
+          <t>Goztepe</t>
         </is>
       </c>
       <c r="D986" t="inlineStr">
         <is>
-          <t>Istanbul Basaksehir</t>
+          <t>Corum Belediyespor</t>
         </is>
       </c>
       <c r="E986" t="n">
-        <v>10.22</v>
+        <v>9.039999999999999</v>
       </c>
       <c r="F986" t="n">
-        <v>2.88</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="987">
       <c r="A987" s="1" t="n">
-        <v>46321</v>
+        <v>46320</v>
       </c>
       <c r="B987" t="inlineStr">
         <is>
@@ -26073,19 +26073,19 @@
       </c>
       <c r="C987" t="inlineStr">
         <is>
-          <t>Caykur Rizespor</t>
+          <t>Konyaspor</t>
         </is>
       </c>
       <c r="D987" t="inlineStr">
         <is>
-          <t>Trabzonspor</t>
+          <t>Genclerbirligi</t>
         </is>
       </c>
       <c r="E987" t="n">
-        <v>9.73</v>
+        <v>9.539999999999999</v>
       </c>
       <c r="F987" t="n">
-        <v>0.19</v>
+        <v>1.35</v>
       </c>
     </row>
     <row r="988">
@@ -26099,18 +26099,70 @@
       </c>
       <c r="C988" t="inlineStr">
         <is>
+          <t>Besiktas</t>
+        </is>
+      </c>
+      <c r="D988" t="inlineStr">
+        <is>
+          <t>Istanbul Basaksehir</t>
+        </is>
+      </c>
+      <c r="E988" t="n">
+        <v>10.22</v>
+      </c>
+      <c r="F988" t="n">
+        <v>2.88</v>
+      </c>
+    </row>
+    <row r="989">
+      <c r="A989" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B989" t="inlineStr">
+        <is>
+          <t>Turkey - Super Lig</t>
+        </is>
+      </c>
+      <c r="C989" t="inlineStr">
+        <is>
+          <t>Caykur Rizespor</t>
+        </is>
+      </c>
+      <c r="D989" t="inlineStr">
+        <is>
+          <t>Trabzonspor</t>
+        </is>
+      </c>
+      <c r="E989" t="n">
+        <v>9.73</v>
+      </c>
+      <c r="F989" t="n">
+        <v>0.19</v>
+      </c>
+    </row>
+    <row r="990">
+      <c r="A990" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B990" t="inlineStr">
+        <is>
+          <t>Turkey - Super Lig</t>
+        </is>
+      </c>
+      <c r="C990" t="inlineStr">
+        <is>
           <t>Galatasaray</t>
         </is>
       </c>
-      <c r="D988" t="inlineStr">
+      <c r="D990" t="inlineStr">
         <is>
           <t>Fenerbahce</t>
         </is>
       </c>
-      <c r="E988" t="n">
+      <c r="E990" t="n">
         <v>9.960000000000001</v>
       </c>
-      <c r="F988" t="n">
+      <c r="F990" t="n">
         <v>0.92</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily scrape output - 2026-10-26
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F990"/>
+  <dimension ref="A1:F992"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26094,24 +26094,24 @@
       </c>
       <c r="B988" t="inlineStr">
         <is>
-          <t>Turkey - Super Lig</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C988" t="inlineStr">
         <is>
-          <t>Besiktas</t>
+          <t>Warta Poznan</t>
         </is>
       </c>
       <c r="D988" t="inlineStr">
         <is>
-          <t>Istanbul Basaksehir</t>
+          <t>LKS Lodz</t>
         </is>
       </c>
       <c r="E988" t="n">
-        <v>10.22</v>
+        <v>10.71</v>
       </c>
       <c r="F988" t="n">
-        <v>2.88</v>
+        <v>-0.47</v>
       </c>
     </row>
     <row r="989">
@@ -26120,24 +26120,24 @@
       </c>
       <c r="B989" t="inlineStr">
         <is>
-          <t>Turkey - Super Lig</t>
+          <t>Portugal - Primeira Liga</t>
         </is>
       </c>
       <c r="C989" t="inlineStr">
         <is>
-          <t>Caykur Rizespor</t>
+          <t>Santa Clara</t>
         </is>
       </c>
       <c r="D989" t="inlineStr">
         <is>
-          <t>Trabzonspor</t>
+          <t>Benfica</t>
         </is>
       </c>
       <c r="E989" t="n">
-        <v>9.73</v>
+        <v>9.76</v>
       </c>
       <c r="F989" t="n">
-        <v>0.19</v>
+        <v>-2.89</v>
       </c>
     </row>
     <row r="990">
@@ -26151,18 +26151,70 @@
       </c>
       <c r="C990" t="inlineStr">
         <is>
+          <t>Besiktas</t>
+        </is>
+      </c>
+      <c r="D990" t="inlineStr">
+        <is>
+          <t>Istanbul Basaksehir</t>
+        </is>
+      </c>
+      <c r="E990" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="F990" t="n">
+        <v>2.71</v>
+      </c>
+    </row>
+    <row r="991">
+      <c r="A991" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B991" t="inlineStr">
+        <is>
+          <t>Turkey - Super Lig</t>
+        </is>
+      </c>
+      <c r="C991" t="inlineStr">
+        <is>
+          <t>Caykur Rizespor</t>
+        </is>
+      </c>
+      <c r="D991" t="inlineStr">
+        <is>
+          <t>Trabzonspor</t>
+        </is>
+      </c>
+      <c r="E991" t="n">
+        <v>9.76</v>
+      </c>
+      <c r="F991" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="992">
+      <c r="A992" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B992" t="inlineStr">
+        <is>
+          <t>Turkey - Super Lig</t>
+        </is>
+      </c>
+      <c r="C992" t="inlineStr">
+        <is>
           <t>Galatasaray</t>
         </is>
       </c>
-      <c r="D990" t="inlineStr">
+      <c r="D992" t="inlineStr">
         <is>
           <t>Fenerbahce</t>
         </is>
       </c>
-      <c r="E990" t="n">
-        <v>9.960000000000001</v>
-      </c>
-      <c r="F990" t="n">
+      <c r="E992" t="n">
+        <v>10.05</v>
+      </c>
+      <c r="F992" t="n">
         <v>0.92</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily scrape output - 2026-10-27
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F992"/>
+  <dimension ref="A1:F997"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26218,6 +26218,136 @@
         <v>0.92</v>
       </c>
     </row>
+    <row r="993">
+      <c r="A993" s="1" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B993" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C993" t="inlineStr">
+        <is>
+          <t>Augsburg</t>
+        </is>
+      </c>
+      <c r="D993" t="inlineStr">
+        <is>
+          <t>Freiburg</t>
+        </is>
+      </c>
+      <c r="E993" t="n">
+        <v>10.01</v>
+      </c>
+      <c r="F993" t="n">
+        <v>-0.04</v>
+      </c>
+    </row>
+    <row r="994">
+      <c r="A994" s="1" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B994" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C994" t="inlineStr">
+        <is>
+          <t>Bayer Leverkusen</t>
+        </is>
+      </c>
+      <c r="D994" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="E994" t="n">
+        <v>10.53</v>
+      </c>
+      <c r="F994" t="n">
+        <v>1.72</v>
+      </c>
+    </row>
+    <row r="995">
+      <c r="A995" s="1" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B995" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C995" t="inlineStr">
+        <is>
+          <t>Bayern Munich</t>
+        </is>
+      </c>
+      <c r="D995" t="inlineStr">
+        <is>
+          <t>Borussia Dortmund</t>
+        </is>
+      </c>
+      <c r="E995" t="n">
+        <v>10.27</v>
+      </c>
+      <c r="F995" t="n">
+        <v>3.43</v>
+      </c>
+    </row>
+    <row r="996">
+      <c r="A996" s="1" t="n">
+        <v>46327</v>
+      </c>
+      <c r="B996" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C996" t="inlineStr">
+        <is>
+          <t>Eintracht Frankfurt</t>
+        </is>
+      </c>
+      <c r="D996" t="inlineStr">
+        <is>
+          <t>Hamburger SV</t>
+        </is>
+      </c>
+      <c r="E996" t="n">
+        <v>10</v>
+      </c>
+      <c r="F996" t="n">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="997">
+      <c r="A997" s="1" t="n">
+        <v>46327</v>
+      </c>
+      <c r="B997" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C997" t="inlineStr">
+        <is>
+          <t>Union Berlin</t>
+        </is>
+      </c>
+      <c r="D997" t="inlineStr">
+        <is>
+          <t>FC Koln</t>
+        </is>
+      </c>
+      <c r="E997" t="n">
+        <v>10.04</v>
+      </c>
+      <c r="F997" t="n">
+        <v>0.36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily scrape output - 2026-10-28
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F997"/>
+  <dimension ref="A1:F999"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26220,7 +26220,7 @@
     </row>
     <row r="993">
       <c r="A993" s="1" t="n">
-        <v>46326</v>
+        <v>46325</v>
       </c>
       <c r="B993" t="inlineStr">
         <is>
@@ -26229,19 +26229,19 @@
       </c>
       <c r="C993" t="inlineStr">
         <is>
-          <t>Augsburg</t>
+          <t>Elversberg</t>
         </is>
       </c>
       <c r="D993" t="inlineStr">
         <is>
-          <t>Freiburg</t>
+          <t>Mainz 05</t>
         </is>
       </c>
       <c r="E993" t="n">
-        <v>10.01</v>
+        <v>9.98</v>
       </c>
       <c r="F993" t="n">
-        <v>-0.04</v>
+        <v>-0.44</v>
       </c>
     </row>
     <row r="994">
@@ -26255,19 +26255,19 @@
       </c>
       <c r="C994" t="inlineStr">
         <is>
-          <t>Bayer Leverkusen</t>
+          <t>Augsburg</t>
         </is>
       </c>
       <c r="D994" t="inlineStr">
         <is>
-          <t>Stuttgart</t>
+          <t>Freiburg</t>
         </is>
       </c>
       <c r="E994" t="n">
-        <v>10.53</v>
+        <v>10.01</v>
       </c>
       <c r="F994" t="n">
-        <v>1.72</v>
+        <v>-0.04</v>
       </c>
     </row>
     <row r="995">
@@ -26281,24 +26281,24 @@
       </c>
       <c r="C995" t="inlineStr">
         <is>
-          <t>Bayern Munich</t>
+          <t>Bayer Leverkusen</t>
         </is>
       </c>
       <c r="D995" t="inlineStr">
         <is>
-          <t>Borussia Dortmund</t>
+          <t>Stuttgart</t>
         </is>
       </c>
       <c r="E995" t="n">
-        <v>10.27</v>
+        <v>10.53</v>
       </c>
       <c r="F995" t="n">
-        <v>3.43</v>
+        <v>1.72</v>
       </c>
     </row>
     <row r="996">
       <c r="A996" s="1" t="n">
-        <v>46327</v>
+        <v>46326</v>
       </c>
       <c r="B996" t="inlineStr">
         <is>
@@ -26307,44 +26307,96 @@
       </c>
       <c r="C996" t="inlineStr">
         <is>
-          <t>Eintracht Frankfurt</t>
+          <t>Bayern Munich</t>
         </is>
       </c>
       <c r="D996" t="inlineStr">
         <is>
-          <t>Hamburger SV</t>
+          <t>Borussia Dortmund</t>
         </is>
       </c>
       <c r="E996" t="n">
-        <v>10</v>
+        <v>10.29</v>
       </c>
       <c r="F996" t="n">
-        <v>2.7</v>
+        <v>3.65</v>
       </c>
     </row>
     <row r="997">
       <c r="A997" s="1" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B997" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C997" t="inlineStr">
+        <is>
+          <t>Werder Bremen</t>
+        </is>
+      </c>
+      <c r="D997" t="inlineStr">
+        <is>
+          <t>Hoffenheim</t>
+        </is>
+      </c>
+      <c r="E997" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="F997" t="n">
+        <v>-0.49</v>
+      </c>
+    </row>
+    <row r="998">
+      <c r="A998" s="1" t="n">
         <v>46327</v>
       </c>
-      <c r="B997" t="inlineStr">
+      <c r="B998" t="inlineStr">
         <is>
           <t>Germany - Bundesliga</t>
         </is>
       </c>
-      <c r="C997" t="inlineStr">
+      <c r="C998" t="inlineStr">
+        <is>
+          <t>Eintracht Frankfurt</t>
+        </is>
+      </c>
+      <c r="D998" t="inlineStr">
+        <is>
+          <t>Hamburger SV</t>
+        </is>
+      </c>
+      <c r="E998" t="n">
+        <v>10</v>
+      </c>
+      <c r="F998" t="n">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="999">
+      <c r="A999" s="1" t="n">
+        <v>46327</v>
+      </c>
+      <c r="B999" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C999" t="inlineStr">
         <is>
           <t>Union Berlin</t>
         </is>
       </c>
-      <c r="D997" t="inlineStr">
+      <c r="D999" t="inlineStr">
         <is>
           <t>FC Koln</t>
         </is>
       </c>
-      <c r="E997" t="n">
+      <c r="E999" t="n">
         <v>10.04</v>
       </c>
-      <c r="F997" t="n">
+      <c r="F999" t="n">
         <v>0.36</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily scrape output - 2026-10-29
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F999"/>
+  <dimension ref="A1:F1001"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26264,10 +26264,10 @@
         </is>
       </c>
       <c r="E994" t="n">
-        <v>10.01</v>
+        <v>9.98</v>
       </c>
       <c r="F994" t="n">
-        <v>-0.04</v>
+        <v>-0.03</v>
       </c>
     </row>
     <row r="995">
@@ -26316,10 +26316,10 @@
         </is>
       </c>
       <c r="E996" t="n">
-        <v>10.29</v>
+        <v>10.13</v>
       </c>
       <c r="F996" t="n">
-        <v>3.65</v>
+        <v>3.64</v>
       </c>
     </row>
     <row r="997">
@@ -26333,24 +26333,24 @@
       </c>
       <c r="C997" t="inlineStr">
         <is>
-          <t>Werder Bremen</t>
+          <t>Borussia Monchengladbach</t>
         </is>
       </c>
       <c r="D997" t="inlineStr">
         <is>
-          <t>Hoffenheim</t>
+          <t>Paderborn</t>
         </is>
       </c>
       <c r="E997" t="n">
-        <v>10.3</v>
+        <v>9.550000000000001</v>
       </c>
       <c r="F997" t="n">
-        <v>-0.49</v>
+        <v>0.89</v>
       </c>
     </row>
     <row r="998">
       <c r="A998" s="1" t="n">
-        <v>46327</v>
+        <v>46326</v>
       </c>
       <c r="B998" t="inlineStr">
         <is>
@@ -26359,45 +26359,97 @@
       </c>
       <c r="C998" t="inlineStr">
         <is>
-          <t>Eintracht Frankfurt</t>
+          <t>Schalke 04</t>
         </is>
       </c>
       <c r="D998" t="inlineStr">
         <is>
-          <t>Hamburger SV</t>
+          <t>RB Leipzig</t>
         </is>
       </c>
       <c r="E998" t="n">
-        <v>10</v>
+        <v>9.76</v>
       </c>
       <c r="F998" t="n">
-        <v>2.7</v>
+        <v>-0.7</v>
       </c>
     </row>
     <row r="999">
       <c r="A999" s="1" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B999" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C999" t="inlineStr">
+        <is>
+          <t>Werder Bremen</t>
+        </is>
+      </c>
+      <c r="D999" t="inlineStr">
+        <is>
+          <t>Hoffenheim</t>
+        </is>
+      </c>
+      <c r="E999" t="n">
+        <v>10.22</v>
+      </c>
+      <c r="F999" t="n">
+        <v>-0.49</v>
+      </c>
+    </row>
+    <row r="1000">
+      <c r="A1000" s="1" t="n">
         <v>46327</v>
       </c>
-      <c r="B999" t="inlineStr">
+      <c r="B1000" t="inlineStr">
         <is>
           <t>Germany - Bundesliga</t>
         </is>
       </c>
-      <c r="C999" t="inlineStr">
+      <c r="C1000" t="inlineStr">
+        <is>
+          <t>Eintracht Frankfurt</t>
+        </is>
+      </c>
+      <c r="D1000" t="inlineStr">
+        <is>
+          <t>Hamburger SV</t>
+        </is>
+      </c>
+      <c r="E1000" t="n">
+        <v>10</v>
+      </c>
+      <c r="F1000" t="n">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="1001">
+      <c r="A1001" s="1" t="n">
+        <v>46327</v>
+      </c>
+      <c r="B1001" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C1001" t="inlineStr">
         <is>
           <t>Union Berlin</t>
         </is>
       </c>
-      <c r="D999" t="inlineStr">
+      <c r="D1001" t="inlineStr">
         <is>
           <t>FC Koln</t>
         </is>
       </c>
-      <c r="E999" t="n">
-        <v>10.04</v>
-      </c>
-      <c r="F999" t="n">
-        <v>0.36</v>
+      <c r="E1001" t="n">
+        <v>10.03</v>
+      </c>
+      <c r="F1001" t="n">
+        <v>0.51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-10-30
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1001"/>
+  <dimension ref="A1:F1028"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26238,140 +26238,140 @@
         </is>
       </c>
       <c r="E993" t="n">
-        <v>9.98</v>
+        <v>10.14</v>
       </c>
       <c r="F993" t="n">
-        <v>-0.44</v>
+        <v>-0.48</v>
       </c>
     </row>
     <row r="994">
       <c r="A994" s="1" t="n">
-        <v>46326</v>
+        <v>46325</v>
       </c>
       <c r="B994" t="inlineStr">
         <is>
-          <t>Germany - Bundesliga</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C994" t="inlineStr">
         <is>
-          <t>Augsburg</t>
+          <t>Pogon Grodzisk Mazowiecki</t>
         </is>
       </c>
       <c r="D994" t="inlineStr">
         <is>
-          <t>Freiburg</t>
+          <t>Stal Mielec</t>
         </is>
       </c>
       <c r="E994" t="n">
-        <v>9.98</v>
+        <v>10.76</v>
       </c>
       <c r="F994" t="n">
-        <v>-0.03</v>
+        <v>0.48</v>
       </c>
     </row>
     <row r="995">
       <c r="A995" s="1" t="n">
-        <v>46326</v>
+        <v>46325</v>
       </c>
       <c r="B995" t="inlineStr">
         <is>
-          <t>Germany - Bundesliga</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C995" t="inlineStr">
         <is>
-          <t>Bayer Leverkusen</t>
+          <t>Cracovia Krakow</t>
         </is>
       </c>
       <c r="D995" t="inlineStr">
         <is>
-          <t>Stuttgart</t>
+          <t>Motor Lublin</t>
         </is>
       </c>
       <c r="E995" t="n">
-        <v>10.53</v>
+        <v>9.779999999999999</v>
       </c>
       <c r="F995" t="n">
-        <v>1.72</v>
+        <v>0.6899999999999999</v>
       </c>
     </row>
     <row r="996">
       <c r="A996" s="1" t="n">
-        <v>46326</v>
+        <v>46325</v>
       </c>
       <c r="B996" t="inlineStr">
         <is>
-          <t>Germany - Bundesliga</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C996" t="inlineStr">
         <is>
-          <t>Bayern Munich</t>
+          <t>Gornik Zabrze</t>
         </is>
       </c>
       <c r="D996" t="inlineStr">
         <is>
-          <t>Borussia Dortmund</t>
+          <t>Legia Warsaw</t>
         </is>
       </c>
       <c r="E996" t="n">
-        <v>10.13</v>
+        <v>9.470000000000001</v>
       </c>
       <c r="F996" t="n">
-        <v>3.64</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="997">
       <c r="A997" s="1" t="n">
-        <v>46326</v>
+        <v>46325</v>
       </c>
       <c r="B997" t="inlineStr">
         <is>
-          <t>Germany - Bundesliga</t>
+          <t>Portugal - Primeira Liga</t>
         </is>
       </c>
       <c r="C997" t="inlineStr">
         <is>
-          <t>Borussia Monchengladbach</t>
+          <t>Casa Pia</t>
         </is>
       </c>
       <c r="D997" t="inlineStr">
         <is>
-          <t>Paderborn</t>
+          <t>Sporting CP</t>
         </is>
       </c>
       <c r="E997" t="n">
-        <v>9.550000000000001</v>
+        <v>9.65</v>
       </c>
       <c r="F997" t="n">
-        <v>0.89</v>
+        <v>-3.12</v>
       </c>
     </row>
     <row r="998">
       <c r="A998" s="1" t="n">
-        <v>46326</v>
+        <v>46325</v>
       </c>
       <c r="B998" t="inlineStr">
         <is>
-          <t>Germany - Bundesliga</t>
+          <t>Turkey - Super Lig</t>
         </is>
       </c>
       <c r="C998" t="inlineStr">
         <is>
-          <t>Schalke 04</t>
+          <t>Konyaspor</t>
         </is>
       </c>
       <c r="D998" t="inlineStr">
         <is>
-          <t>RB Leipzig</t>
+          <t>Galatasaray</t>
         </is>
       </c>
       <c r="E998" t="n">
-        <v>9.76</v>
+        <v>9.609999999999999</v>
       </c>
       <c r="F998" t="n">
-        <v>-0.7</v>
+        <v>-2.51</v>
       </c>
     </row>
     <row r="999">
@@ -26385,24 +26385,24 @@
       </c>
       <c r="C999" t="inlineStr">
         <is>
-          <t>Werder Bremen</t>
+          <t>Augsburg</t>
         </is>
       </c>
       <c r="D999" t="inlineStr">
         <is>
-          <t>Hoffenheim</t>
+          <t>Freiburg</t>
         </is>
       </c>
       <c r="E999" t="n">
-        <v>10.22</v>
+        <v>9.98</v>
       </c>
       <c r="F999" t="n">
-        <v>-0.49</v>
+        <v>-0.09</v>
       </c>
     </row>
     <row r="1000">
       <c r="A1000" s="1" t="n">
-        <v>46327</v>
+        <v>46326</v>
       </c>
       <c r="B1000" t="inlineStr">
         <is>
@@ -26411,45 +26411,747 @@
       </c>
       <c r="C1000" t="inlineStr">
         <is>
-          <t>Eintracht Frankfurt</t>
+          <t>Bayer Leverkusen</t>
         </is>
       </c>
       <c r="D1000" t="inlineStr">
         <is>
-          <t>Hamburger SV</t>
+          <t>Stuttgart</t>
         </is>
       </c>
       <c r="E1000" t="n">
-        <v>10</v>
+        <v>10.53</v>
       </c>
       <c r="F1000" t="n">
-        <v>2.7</v>
+        <v>1.72</v>
       </c>
     </row>
     <row r="1001">
       <c r="A1001" s="1" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B1001" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C1001" t="inlineStr">
+        <is>
+          <t>Bayern Munich</t>
+        </is>
+      </c>
+      <c r="D1001" t="inlineStr">
+        <is>
+          <t>Borussia Dortmund</t>
+        </is>
+      </c>
+      <c r="E1001" t="n">
+        <v>10.13</v>
+      </c>
+      <c r="F1001" t="n">
+        <v>3.64</v>
+      </c>
+    </row>
+    <row r="1002">
+      <c r="A1002" s="1" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B1002" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C1002" t="inlineStr">
+        <is>
+          <t>Borussia Monchengladbach</t>
+        </is>
+      </c>
+      <c r="D1002" t="inlineStr">
+        <is>
+          <t>Paderborn</t>
+        </is>
+      </c>
+      <c r="E1002" t="n">
+        <v>9.550000000000001</v>
+      </c>
+      <c r="F1002" t="n">
+        <v>0.89</v>
+      </c>
+    </row>
+    <row r="1003">
+      <c r="A1003" s="1" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B1003" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C1003" t="inlineStr">
+        <is>
+          <t>Schalke 04</t>
+        </is>
+      </c>
+      <c r="D1003" t="inlineStr">
+        <is>
+          <t>RB Leipzig</t>
+        </is>
+      </c>
+      <c r="E1003" t="n">
+        <v>9.77</v>
+      </c>
+      <c r="F1003" t="n">
+        <v>-0.87</v>
+      </c>
+    </row>
+    <row r="1004">
+      <c r="A1004" s="1" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B1004" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C1004" t="inlineStr">
+        <is>
+          <t>Werder Bremen</t>
+        </is>
+      </c>
+      <c r="D1004" t="inlineStr">
+        <is>
+          <t>Hoffenheim</t>
+        </is>
+      </c>
+      <c r="E1004" t="n">
+        <v>10.24</v>
+      </c>
+      <c r="F1004" t="n">
+        <v>-0.53</v>
+      </c>
+    </row>
+    <row r="1005">
+      <c r="A1005" s="1" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B1005" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C1005" t="inlineStr">
+        <is>
+          <t>Lechia Gdansk</t>
+        </is>
+      </c>
+      <c r="D1005" t="inlineStr">
+        <is>
+          <t>Unia Skierniewice</t>
+        </is>
+      </c>
+      <c r="E1005" t="n">
+        <v>10.84</v>
+      </c>
+      <c r="F1005" t="n">
+        <v>1.19</v>
+      </c>
+    </row>
+    <row r="1006">
+      <c r="A1006" s="1" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B1006" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C1006" t="inlineStr">
+        <is>
+          <t>Miedz Legnica</t>
+        </is>
+      </c>
+      <c r="D1006" t="inlineStr">
+        <is>
+          <t>Nieciecza</t>
+        </is>
+      </c>
+      <c r="E1006" t="n">
+        <v>11.04</v>
+      </c>
+      <c r="F1006" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="1007">
+      <c r="A1007" s="1" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B1007" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C1007" t="inlineStr">
+        <is>
+          <t>Podbeskidzie Bielsko-Biala</t>
+        </is>
+      </c>
+      <c r="D1007" t="inlineStr">
+        <is>
+          <t>Warta Poznan</t>
+        </is>
+      </c>
+      <c r="E1007" t="n">
+        <v>10.26</v>
+      </c>
+      <c r="F1007" t="n">
+        <v>1.15</v>
+      </c>
+    </row>
+    <row r="1008">
+      <c r="A1008" s="1" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B1008" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C1008" t="inlineStr">
+        <is>
+          <t>GKS Katowice</t>
+        </is>
+      </c>
+      <c r="D1008" t="inlineStr">
+        <is>
+          <t>Widzew Lodz</t>
+        </is>
+      </c>
+      <c r="E1008" t="n">
+        <v>10.38</v>
+      </c>
+      <c r="F1008" t="n">
+        <v>0.31</v>
+      </c>
+    </row>
+    <row r="1009">
+      <c r="A1009" s="1" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B1009" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C1009" t="inlineStr">
+        <is>
+          <t>Lech Poznan</t>
+        </is>
+      </c>
+      <c r="D1009" t="inlineStr">
+        <is>
+          <t>Wisla Krakow</t>
+        </is>
+      </c>
+      <c r="E1009" t="n">
+        <v>10.47</v>
+      </c>
+      <c r="F1009" t="n">
+        <v>1.61</v>
+      </c>
+    </row>
+    <row r="1010">
+      <c r="A1010" s="1" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B1010" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C1010" t="inlineStr">
+        <is>
+          <t>Wieczysta Krakow</t>
+        </is>
+      </c>
+      <c r="D1010" t="inlineStr">
+        <is>
+          <t>Jagiellonia Bialystok</t>
+        </is>
+      </c>
+      <c r="E1010" t="n">
+        <v>10.23</v>
+      </c>
+      <c r="F1010" t="n">
+        <v>0.93</v>
+      </c>
+    </row>
+    <row r="1011">
+      <c r="A1011" s="1" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B1011" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C1011" t="inlineStr">
+        <is>
+          <t>Wisla Plock</t>
+        </is>
+      </c>
+      <c r="D1011" t="inlineStr">
+        <is>
+          <t>Piast Gliwice</t>
+        </is>
+      </c>
+      <c r="E1011" t="n">
+        <v>10.48</v>
+      </c>
+      <c r="F1011" t="n">
+        <v>0.88</v>
+      </c>
+    </row>
+    <row r="1012">
+      <c r="A1012" s="1" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B1012" t="inlineStr">
+        <is>
+          <t>Portugal - Primeira Liga</t>
+        </is>
+      </c>
+      <c r="C1012" t="inlineStr">
+        <is>
+          <t>Moreirense</t>
+        </is>
+      </c>
+      <c r="D1012" t="inlineStr">
+        <is>
+          <t>Estrela da Amadora</t>
+        </is>
+      </c>
+      <c r="E1012" t="n">
+        <v>9.18</v>
+      </c>
+      <c r="F1012" t="n">
+        <v>-0.34</v>
+      </c>
+    </row>
+    <row r="1013">
+      <c r="A1013" s="1" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B1013" t="inlineStr">
+        <is>
+          <t>Turkey - Super Lig</t>
+        </is>
+      </c>
+      <c r="C1013" t="inlineStr">
+        <is>
+          <t>Fenerbahce</t>
+        </is>
+      </c>
+      <c r="D1013" t="inlineStr">
+        <is>
+          <t>Goztepe</t>
+        </is>
+      </c>
+      <c r="E1013" t="n">
+        <v>10.18</v>
+      </c>
+      <c r="F1013" t="n">
+        <v>2.71</v>
+      </c>
+    </row>
+    <row r="1014">
+      <c r="A1014" s="1" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B1014" t="inlineStr">
+        <is>
+          <t>Turkey - Super Lig</t>
+        </is>
+      </c>
+      <c r="C1014" t="inlineStr">
+        <is>
+          <t>Kocaelispor</t>
+        </is>
+      </c>
+      <c r="D1014" t="inlineStr">
+        <is>
+          <t>Caykur Rizespor</t>
+        </is>
+      </c>
+      <c r="E1014" t="n">
+        <v>9.220000000000001</v>
+      </c>
+      <c r="F1014" t="n">
+        <v>0.67</v>
+      </c>
+    </row>
+    <row r="1015">
+      <c r="A1015" s="1" t="n">
         <v>46327</v>
       </c>
-      <c r="B1001" t="inlineStr">
+      <c r="B1015" t="inlineStr">
         <is>
           <t>Germany - Bundesliga</t>
         </is>
       </c>
-      <c r="C1001" t="inlineStr">
+      <c r="C1015" t="inlineStr">
+        <is>
+          <t>Eintracht Frankfurt</t>
+        </is>
+      </c>
+      <c r="D1015" t="inlineStr">
+        <is>
+          <t>Hamburger SV</t>
+        </is>
+      </c>
+      <c r="E1015" t="n">
+        <v>10</v>
+      </c>
+      <c r="F1015" t="n">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="1016">
+      <c r="A1016" s="1" t="n">
+        <v>46327</v>
+      </c>
+      <c r="B1016" t="inlineStr">
+        <is>
+          <t>Germany - Bundesliga</t>
+        </is>
+      </c>
+      <c r="C1016" t="inlineStr">
         <is>
           <t>Union Berlin</t>
         </is>
       </c>
-      <c r="D1001" t="inlineStr">
+      <c r="D1016" t="inlineStr">
         <is>
           <t>FC Koln</t>
         </is>
       </c>
-      <c r="E1001" t="n">
-        <v>10.03</v>
-      </c>
-      <c r="F1001" t="n">
-        <v>0.51</v>
+      <c r="E1016" t="n">
+        <v>9.789999999999999</v>
+      </c>
+      <c r="F1016" t="n">
+        <v>0.53</v>
+      </c>
+    </row>
+    <row r="1017">
+      <c r="A1017" s="1" t="n">
+        <v>46327</v>
+      </c>
+      <c r="B1017" t="inlineStr">
+        <is>
+          <t>Portugal - Primeira Liga</t>
+        </is>
+      </c>
+      <c r="C1017" t="inlineStr">
+        <is>
+          <t>Arouca</t>
+        </is>
+      </c>
+      <c r="D1017" t="inlineStr">
+        <is>
+          <t>Nacional da Madeira</t>
+        </is>
+      </c>
+      <c r="E1017" t="n">
+        <v>9.640000000000001</v>
+      </c>
+      <c r="F1017" t="n">
+        <v>1.53</v>
+      </c>
+    </row>
+    <row r="1018">
+      <c r="A1018" s="1" t="n">
+        <v>46327</v>
+      </c>
+      <c r="B1018" t="inlineStr">
+        <is>
+          <t>Portugal - Primeira Liga</t>
+        </is>
+      </c>
+      <c r="C1018" t="inlineStr">
+        <is>
+          <t>Braga</t>
+        </is>
+      </c>
+      <c r="D1018" t="inlineStr">
+        <is>
+          <t>Famalicao</t>
+        </is>
+      </c>
+      <c r="E1018" t="n">
+        <v>9.359999999999999</v>
+      </c>
+      <c r="F1018" t="n">
+        <v>2.44</v>
+      </c>
+    </row>
+    <row r="1019">
+      <c r="A1019" s="1" t="n">
+        <v>46327</v>
+      </c>
+      <c r="B1019" t="inlineStr">
+        <is>
+          <t>Turkey - Super Lig</t>
+        </is>
+      </c>
+      <c r="C1019" t="inlineStr">
+        <is>
+          <t>Istanbul Basaksehir</t>
+        </is>
+      </c>
+      <c r="D1019" t="inlineStr">
+        <is>
+          <t>Samsunspor</t>
+        </is>
+      </c>
+      <c r="E1019" t="n">
+        <v>9.710000000000001</v>
+      </c>
+      <c r="F1019" t="n">
+        <v>1.42</v>
+      </c>
+    </row>
+    <row r="1020">
+      <c r="A1020" s="1" t="n">
+        <v>46327</v>
+      </c>
+      <c r="B1020" t="inlineStr">
+        <is>
+          <t>Turkey - Super Lig</t>
+        </is>
+      </c>
+      <c r="C1020" t="inlineStr">
+        <is>
+          <t>Kasimpasa</t>
+        </is>
+      </c>
+      <c r="D1020" t="inlineStr">
+        <is>
+          <t>Besiktas</t>
+        </is>
+      </c>
+      <c r="E1020" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="F1020" t="n">
+        <v>-1.96</v>
+      </c>
+    </row>
+    <row r="1021">
+      <c r="A1021" s="1" t="n">
+        <v>46327</v>
+      </c>
+      <c r="B1021" t="inlineStr">
+        <is>
+          <t>Turkey - Super Lig</t>
+        </is>
+      </c>
+      <c r="C1021" t="inlineStr">
+        <is>
+          <t>Trabzonspor</t>
+        </is>
+      </c>
+      <c r="D1021" t="inlineStr">
+        <is>
+          <t>Gaziantep</t>
+        </is>
+      </c>
+      <c r="E1021" t="n">
+        <v>9.710000000000001</v>
+      </c>
+      <c r="F1021" t="n">
+        <v>2.24</v>
+      </c>
+    </row>
+    <row r="1022">
+      <c r="A1022" s="1" t="n">
+        <v>46328</v>
+      </c>
+      <c r="B1022" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C1022" t="inlineStr">
+        <is>
+          <t>LKS Lodz</t>
+        </is>
+      </c>
+      <c r="D1022" t="inlineStr">
+        <is>
+          <t>Polonia Warsaw</t>
+        </is>
+      </c>
+      <c r="E1022" t="n">
+        <v>10.78</v>
+      </c>
+      <c r="F1022" t="n">
+        <v>0.84</v>
+      </c>
+    </row>
+    <row r="1023">
+      <c r="A1023" s="1" t="n">
+        <v>46328</v>
+      </c>
+      <c r="B1023" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C1023" t="inlineStr">
+        <is>
+          <t>Polonia Bytom</t>
+        </is>
+      </c>
+      <c r="D1023" t="inlineStr">
+        <is>
+          <t>Odra Opole</t>
+        </is>
+      </c>
+      <c r="E1023" t="n">
+        <v>10.38</v>
+      </c>
+      <c r="F1023" t="n">
+        <v>1.09</v>
+      </c>
+    </row>
+    <row r="1024">
+      <c r="A1024" s="1" t="n">
+        <v>46328</v>
+      </c>
+      <c r="B1024" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C1024" t="inlineStr">
+        <is>
+          <t>Stal Rzeszow</t>
+        </is>
+      </c>
+      <c r="D1024" t="inlineStr">
+        <is>
+          <t>Puszcza Niepolomice</t>
+        </is>
+      </c>
+      <c r="E1024" t="n">
+        <v>10.63</v>
+      </c>
+      <c r="F1024" t="n">
+        <v>0.67</v>
+      </c>
+    </row>
+    <row r="1025">
+      <c r="A1025" s="1" t="n">
+        <v>46328</v>
+      </c>
+      <c r="B1025" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C1025" t="inlineStr">
+        <is>
+          <t>Radomiak Radom</t>
+        </is>
+      </c>
+      <c r="D1025" t="inlineStr">
+        <is>
+          <t>Slask Wroclaw</t>
+        </is>
+      </c>
+      <c r="E1025" t="n">
+        <v>10.52</v>
+      </c>
+      <c r="F1025" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="1026">
+      <c r="A1026" s="1" t="n">
+        <v>46328</v>
+      </c>
+      <c r="B1026" t="inlineStr">
+        <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C1026" t="inlineStr">
+        <is>
+          <t>Zaglebie Lubin</t>
+        </is>
+      </c>
+      <c r="D1026" t="inlineStr">
+        <is>
+          <t>Korona Kielce</t>
+        </is>
+      </c>
+      <c r="E1026" t="n">
+        <v>10.28</v>
+      </c>
+      <c r="F1026" t="n">
+        <v>-0.68</v>
+      </c>
+    </row>
+    <row r="1027">
+      <c r="A1027" s="1" t="n">
+        <v>46328</v>
+      </c>
+      <c r="B1027" t="inlineStr">
+        <is>
+          <t>Portugal - Primeira Liga</t>
+        </is>
+      </c>
+      <c r="C1027" t="inlineStr">
+        <is>
+          <t>Gil Vicente</t>
+        </is>
+      </c>
+      <c r="D1027" t="inlineStr">
+        <is>
+          <t>Vitoria Guimaraes</t>
+        </is>
+      </c>
+      <c r="E1027" t="n">
+        <v>9.220000000000001</v>
+      </c>
+      <c r="F1027" t="n">
+        <v>-0.1</v>
+      </c>
+    </row>
+    <row r="1028">
+      <c r="A1028" s="1" t="n">
+        <v>46328</v>
+      </c>
+      <c r="B1028" t="inlineStr">
+        <is>
+          <t>Turkey - Super Lig</t>
+        </is>
+      </c>
+      <c r="C1028" t="inlineStr">
+        <is>
+          <t>Genclerbirligi</t>
+        </is>
+      </c>
+      <c r="D1028" t="inlineStr">
+        <is>
+          <t>Alanyaspor</t>
+        </is>
+      </c>
+      <c r="E1028" t="n">
+        <v>9.550000000000001</v>
+      </c>
+      <c r="F1028" t="n">
+        <v>-0.02</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily scrape output - 2026-10-31
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_historical.xlsx
+++ b/outputs/pinnacle_corners_historical.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1028"/>
+  <dimension ref="A1:F1032"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26420,7 +26420,7 @@
         </is>
       </c>
       <c r="E1000" t="n">
-        <v>10.53</v>
+        <v>10.63</v>
       </c>
       <c r="F1000" t="n">
         <v>1.72</v>
@@ -26446,10 +26446,10 @@
         </is>
       </c>
       <c r="E1001" t="n">
-        <v>10.13</v>
+        <v>10.02</v>
       </c>
       <c r="F1001" t="n">
-        <v>3.64</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="1002">
@@ -26472,10 +26472,10 @@
         </is>
       </c>
       <c r="E1002" t="n">
-        <v>9.550000000000001</v>
+        <v>9.44</v>
       </c>
       <c r="F1002" t="n">
-        <v>0.89</v>
+        <v>0.86</v>
       </c>
     </row>
     <row r="1003">
@@ -26498,10 +26498,10 @@
         </is>
       </c>
       <c r="E1003" t="n">
-        <v>9.77</v>
+        <v>9.82</v>
       </c>
       <c r="F1003" t="n">
-        <v>-0.87</v>
+        <v>-0.88</v>
       </c>
     </row>
     <row r="1004">
@@ -26524,7 +26524,7 @@
         </is>
       </c>
       <c r="E1004" t="n">
-        <v>10.24</v>
+        <v>10.19</v>
       </c>
       <c r="F1004" t="n">
         <v>-0.53</v>
@@ -26553,7 +26553,7 @@
         <v>10.84</v>
       </c>
       <c r="F1005" t="n">
-        <v>1.19</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="1006">
@@ -26576,10 +26576,10 @@
         </is>
       </c>
       <c r="E1006" t="n">
-        <v>11.04</v>
+        <v>11.1</v>
       </c>
       <c r="F1006" t="n">
-        <v>0.7</v>
+        <v>0.57</v>
       </c>
     </row>
     <row r="1007">
@@ -26602,10 +26602,10 @@
         </is>
       </c>
       <c r="E1007" t="n">
-        <v>10.26</v>
+        <v>10.28</v>
       </c>
       <c r="F1007" t="n">
-        <v>1.15</v>
+        <v>0.9399999999999999</v>
       </c>
     </row>
     <row r="1008">
@@ -26680,10 +26680,10 @@
         </is>
       </c>
       <c r="E1010" t="n">
-        <v>10.23</v>
+        <v>10.26</v>
       </c>
       <c r="F1010" t="n">
-        <v>0.93</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="1011">
@@ -26732,10 +26732,10 @@
         </is>
       </c>
       <c r="E1012" t="n">
-        <v>9.18</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="F1012" t="n">
-        <v>-0.34</v>
+        <v>-0.33</v>
       </c>
     </row>
     <row r="1013">
@@ -26744,24 +26744,24 @@
       </c>
       <c r="B1013" t="inlineStr">
         <is>
-          <t>Turkey - Super Lig</t>
+          <t>Portugal - Primeira Liga</t>
         </is>
       </c>
       <c r="C1013" t="inlineStr">
         <is>
-          <t>Fenerbahce</t>
+          <t>Porto</t>
         </is>
       </c>
       <c r="D1013" t="inlineStr">
         <is>
-          <t>Goztepe</t>
+          <t>Estoril</t>
         </is>
       </c>
       <c r="E1013" t="n">
-        <v>10.18</v>
+        <v>9.82</v>
       </c>
       <c r="F1013" t="n">
-        <v>2.71</v>
+        <v>4.22</v>
       </c>
     </row>
     <row r="1014">
@@ -26775,45 +26775,45 @@
       </c>
       <c r="C1014" t="inlineStr">
         <is>
-          <t>Kocaelispor</t>
+          <t>Fenerbahce</t>
         </is>
       </c>
       <c r="D1014" t="inlineStr">
         <is>
-          <t>Caykur Rizespor</t>
+          <t>Goztepe</t>
         </is>
       </c>
       <c r="E1014" t="n">
-        <v>9.220000000000001</v>
+        <v>10.2</v>
       </c>
       <c r="F1014" t="n">
-        <v>0.67</v>
+        <v>3.08</v>
       </c>
     </row>
     <row r="1015">
       <c r="A1015" s="1" t="n">
-        <v>46327</v>
+        <v>46326</v>
       </c>
       <c r="B1015" t="inlineStr">
         <is>
-          <t>Germany - Bundesliga</t>
+          <t>Turkey - Super Lig</t>
         </is>
       </c>
       <c r="C1015" t="inlineStr">
         <is>
-          <t>Eintracht Frankfurt</t>
+          <t>Kocaelispor</t>
         </is>
       </c>
       <c r="D1015" t="inlineStr">
         <is>
-          <t>Hamburger SV</t>
+          <t>Caykur Rizespor</t>
         </is>
       </c>
       <c r="E1015" t="n">
-        <v>10</v>
+        <v>9.23</v>
       </c>
       <c r="F1015" t="n">
-        <v>2.7</v>
+        <v>0.57</v>
       </c>
     </row>
     <row r="1016">
@@ -26827,19 +26827,19 @@
       </c>
       <c r="C1016" t="inlineStr">
         <is>
-          <t>Union Berlin</t>
+          <t>Eintracht Frankfurt</t>
         </is>
       </c>
       <c r="D1016" t="inlineStr">
         <is>
-          <t>FC Koln</t>
+          <t>Hamburger SV</t>
         </is>
       </c>
       <c r="E1016" t="n">
-        <v>9.789999999999999</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="F1016" t="n">
-        <v>0.53</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="1017">
@@ -26848,24 +26848,24 @@
       </c>
       <c r="B1017" t="inlineStr">
         <is>
-          <t>Portugal - Primeira Liga</t>
+          <t>Germany - Bundesliga</t>
         </is>
       </c>
       <c r="C1017" t="inlineStr">
         <is>
-          <t>Arouca</t>
+          <t>Union Berlin</t>
         </is>
       </c>
       <c r="D1017" t="inlineStr">
         <is>
-          <t>Nacional da Madeira</t>
+          <t>FC Koln</t>
         </is>
       </c>
       <c r="E1017" t="n">
-        <v>9.640000000000001</v>
+        <v>9.789999999999999</v>
       </c>
       <c r="F1017" t="n">
-        <v>1.53</v>
+        <v>0.53</v>
       </c>
     </row>
     <row r="1018">
@@ -26879,19 +26879,19 @@
       </c>
       <c r="C1018" t="inlineStr">
         <is>
-          <t>Braga</t>
+          <t>Arouca</t>
         </is>
       </c>
       <c r="D1018" t="inlineStr">
         <is>
-          <t>Famalicao</t>
+          <t>Nacional da Madeira</t>
         </is>
       </c>
       <c r="E1018" t="n">
-        <v>9.359999999999999</v>
+        <v>9.640000000000001</v>
       </c>
       <c r="F1018" t="n">
-        <v>2.44</v>
+        <v>1.53</v>
       </c>
     </row>
     <row r="1019">
@@ -26900,24 +26900,24 @@
       </c>
       <c r="B1019" t="inlineStr">
         <is>
-          <t>Turkey - Super Lig</t>
+          <t>Portugal - Primeira Liga</t>
         </is>
       </c>
       <c r="C1019" t="inlineStr">
         <is>
-          <t>Istanbul Basaksehir</t>
+          <t>Braga</t>
         </is>
       </c>
       <c r="D1019" t="inlineStr">
         <is>
-          <t>Samsunspor</t>
+          <t>Famalicao</t>
         </is>
       </c>
       <c r="E1019" t="n">
-        <v>9.710000000000001</v>
+        <v>9.27</v>
       </c>
       <c r="F1019" t="n">
-        <v>1.42</v>
+        <v>2.44</v>
       </c>
     </row>
     <row r="1020">
@@ -26931,19 +26931,19 @@
       </c>
       <c r="C1020" t="inlineStr">
         <is>
-          <t>Kasimpasa</t>
+          <t>Istanbul Basaksehir</t>
         </is>
       </c>
       <c r="D1020" t="inlineStr">
         <is>
-          <t>Besiktas</t>
+          <t>Samsunspor</t>
         </is>
       </c>
       <c r="E1020" t="n">
-        <v>10.1</v>
+        <v>9.710000000000001</v>
       </c>
       <c r="F1020" t="n">
-        <v>-1.96</v>
+        <v>1.42</v>
       </c>
     </row>
     <row r="1021">
@@ -26957,45 +26957,45 @@
       </c>
       <c r="C1021" t="inlineStr">
         <is>
-          <t>Trabzonspor</t>
+          <t>Kasimpasa</t>
         </is>
       </c>
       <c r="D1021" t="inlineStr">
         <is>
-          <t>Gaziantep</t>
+          <t>Besiktas</t>
         </is>
       </c>
       <c r="E1021" t="n">
-        <v>9.710000000000001</v>
+        <v>10.01</v>
       </c>
       <c r="F1021" t="n">
-        <v>2.24</v>
+        <v>-1.94</v>
       </c>
     </row>
     <row r="1022">
       <c r="A1022" s="1" t="n">
-        <v>46328</v>
+        <v>46327</v>
       </c>
       <c r="B1022" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Turkey - Super Lig</t>
         </is>
       </c>
       <c r="C1022" t="inlineStr">
         <is>
-          <t>LKS Lodz</t>
+          <t>Trabzonspor</t>
         </is>
       </c>
       <c r="D1022" t="inlineStr">
         <is>
-          <t>Polonia Warsaw</t>
+          <t>Gaziantep</t>
         </is>
       </c>
       <c r="E1022" t="n">
-        <v>10.78</v>
+        <v>9.73</v>
       </c>
       <c r="F1022" t="n">
-        <v>0.84</v>
+        <v>2.22</v>
       </c>
     </row>
     <row r="1023">
@@ -27009,19 +27009,19 @@
       </c>
       <c r="C1023" t="inlineStr">
         <is>
-          <t>Polonia Bytom</t>
+          <t>LKS Lodz</t>
         </is>
       </c>
       <c r="D1023" t="inlineStr">
         <is>
-          <t>Odra Opole</t>
+          <t>Polonia Warsaw</t>
         </is>
       </c>
       <c r="E1023" t="n">
-        <v>10.38</v>
+        <v>10.78</v>
       </c>
       <c r="F1023" t="n">
-        <v>1.09</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="1024">
@@ -27035,19 +27035,19 @@
       </c>
       <c r="C1024" t="inlineStr">
         <is>
-          <t>Stal Rzeszow</t>
+          <t>Polonia Bytom</t>
         </is>
       </c>
       <c r="D1024" t="inlineStr">
         <is>
-          <t>Puszcza Niepolomice</t>
+          <t>Odra Opole</t>
         </is>
       </c>
       <c r="E1024" t="n">
-        <v>10.63</v>
+        <v>10.38</v>
       </c>
       <c r="F1024" t="n">
-        <v>0.67</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="1025">
@@ -27056,24 +27056,24 @@
       </c>
       <c r="B1025" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="C1025" t="inlineStr">
         <is>
-          <t>Radomiak Radom</t>
+          <t>Stal Rzeszow</t>
         </is>
       </c>
       <c r="D1025" t="inlineStr">
         <is>
-          <t>Slask Wroclaw</t>
+          <t>Puszcza Niepolomice</t>
         </is>
       </c>
       <c r="E1025" t="n">
-        <v>10.52</v>
+        <v>10.63</v>
       </c>
       <c r="F1025" t="n">
-        <v>1.4</v>
+        <v>0.67</v>
       </c>
     </row>
     <row r="1026">
@@ -27087,19 +27087,19 @@
       </c>
       <c r="C1026" t="inlineStr">
         <is>
-          <t>Zaglebie Lubin</t>
+          <t>Radomiak Radom</t>
         </is>
       </c>
       <c r="D1026" t="inlineStr">
         <is>
-          <t>Korona Kielce</t>
+          <t>Slask Wroclaw</t>
         </is>
       </c>
       <c r="E1026" t="n">
-        <v>10.28</v>
+        <v>10.52</v>
       </c>
       <c r="F1026" t="n">
-        <v>-0.68</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="1027">
@@ -27108,24 +27108,24 @@
       </c>
       <c r="B1027" t="inlineStr">
         <is>
-          <t>Portugal - Primeira Liga</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="C1027" t="inlineStr">
         <is>
-          <t>Gil Vicente</t>
+          <t>Rakow Czestochowa</t>
         </is>
       </c>
       <c r="D1027" t="inlineStr">
         <is>
-          <t>Vitoria Guimaraes</t>
+          <t>Pogon Szczecin</t>
         </is>
       </c>
       <c r="E1027" t="n">
-        <v>9.220000000000001</v>
+        <v>9.73</v>
       </c>
       <c r="F1027" t="n">
-        <v>-0.1</v>
+        <v>1.21</v>
       </c>
     </row>
     <row r="1028">
@@ -27134,24 +27134,128 @@
       </c>
       <c r="B1028" t="inlineStr">
         <is>
+          <t>Poland - Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="C1028" t="inlineStr">
+        <is>
+          <t>Zaglebie Lubin</t>
+        </is>
+      </c>
+      <c r="D1028" t="inlineStr">
+        <is>
+          <t>Korona Kielce</t>
+        </is>
+      </c>
+      <c r="E1028" t="n">
+        <v>10.28</v>
+      </c>
+      <c r="F1028" t="n">
+        <v>-0.68</v>
+      </c>
+    </row>
+    <row r="1029">
+      <c r="A1029" s="1" t="n">
+        <v>46328</v>
+      </c>
+      <c r="B1029" t="inlineStr">
+        <is>
+          <t>Portugal - Primeira Liga</t>
+        </is>
+      </c>
+      <c r="C1029" t="inlineStr">
+        <is>
+          <t>Gil Vicente</t>
+        </is>
+      </c>
+      <c r="D1029" t="inlineStr">
+        <is>
+          <t>Vitoria Guimaraes</t>
+        </is>
+      </c>
+      <c r="E1029" t="n">
+        <v>9.220000000000001</v>
+      </c>
+      <c r="F1029" t="n">
+        <v>-0.1</v>
+      </c>
+    </row>
+    <row r="1030">
+      <c r="A1030" s="1" t="n">
+        <v>46328</v>
+      </c>
+      <c r="B1030" t="inlineStr">
+        <is>
           <t>Turkey - Super Lig</t>
         </is>
       </c>
-      <c r="C1028" t="inlineStr">
+      <c r="C1030" t="inlineStr">
         <is>
           <t>Genclerbirligi</t>
         </is>
       </c>
-      <c r="D1028" t="inlineStr">
+      <c r="D1030" t="inlineStr">
         <is>
           <t>Alanyaspor</t>
         </is>
       </c>
-      <c r="E1028" t="n">
-        <v>9.550000000000001</v>
-      </c>
-      <c r="F1028" t="n">
-        <v>-0.02</v>
+      <c r="E1030" t="n">
+        <v>9.609999999999999</v>
+      </c>
+      <c r="F1030" t="n">
+        <v>-0.03</v>
+      </c>
+    </row>
+    <row r="1031">
+      <c r="A1031" s="1" t="n">
+        <v>46329</v>
+      </c>
+      <c r="B1031" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C1031" t="inlineStr">
+        <is>
+          <t>Chrobry Glogow</t>
+        </is>
+      </c>
+      <c r="D1031" t="inlineStr">
+        <is>
+          <t>Arka Gdynia</t>
+        </is>
+      </c>
+      <c r="E1031" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="F1031" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+    </row>
+    <row r="1032">
+      <c r="A1032" s="1" t="n">
+        <v>46329</v>
+      </c>
+      <c r="B1032" t="inlineStr">
+        <is>
+          <t>Poland - 1st Liga</t>
+        </is>
+      </c>
+      <c r="C1032" t="inlineStr">
+        <is>
+          <t>Pogon Siedlce</t>
+        </is>
+      </c>
+      <c r="D1032" t="inlineStr">
+        <is>
+          <t>Ruch Chorzow</t>
+        </is>
+      </c>
+      <c r="E1032" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="F1032" t="n">
+        <v>-1.68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>